<commit_message>
v1.0.26 - Use two-decimal PS and WS values
</commit_message>
<xml_diff>
--- a/templates/ECR official Template.xlsx
+++ b/templates/ECR official Template.xlsx
@@ -741,7 +741,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="88">
+  <cellXfs count="99">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1040,6 +1040,39 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="15" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="15" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="15" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="15" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="15" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="15" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="15" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="15" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="15" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="15" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="15" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1961,22 +1994,22 @@
       <c r="I18" s="48"/>
       <c r="J18" s="49"/>
       <c r="K18" s="50"/>
-      <c r="L18" s="51"/>
-      <c r="M18" s="52"/>
+      <c r="L18" s="89"/>
+      <c r="M18" s="90"/>
       <c r="N18" s="53"/>
       <c r="O18" s="48"/>
       <c r="P18" s="49"/>
       <c r="Q18" s="50"/>
-      <c r="R18" s="51"/>
-      <c r="S18" s="52"/>
+      <c r="R18" s="89"/>
+      <c r="S18" s="90"/>
       <c r="T18" s="53"/>
       <c r="U18" s="48"/>
       <c r="V18" s="49"/>
-      <c r="W18" s="54"/>
-      <c r="X18" s="55"/>
-      <c r="Y18" s="56"/>
-      <c r="Z18" s="50"/>
-      <c r="AA18" s="52"/>
+      <c r="W18" s="91"/>
+      <c r="X18" s="92"/>
+      <c r="Y18" s="93"/>
+      <c r="Z18" s="88"/>
+      <c r="AA18" s="90"/>
       <c r="AB18" s="57"/>
       <c r="AC18" s="58"/>
       <c r="AD18" s="59"/>
@@ -1997,22 +2030,22 @@
       <c r="I19" s="61"/>
       <c r="J19" s="62"/>
       <c r="K19" s="54"/>
-      <c r="L19" s="55"/>
-      <c r="M19" s="63"/>
+      <c r="L19" s="92"/>
+      <c r="M19" s="94"/>
       <c r="N19" s="64"/>
       <c r="O19" s="61"/>
       <c r="P19" s="62"/>
       <c r="Q19" s="54"/>
-      <c r="R19" s="55"/>
-      <c r="S19" s="63"/>
+      <c r="R19" s="92"/>
+      <c r="S19" s="94"/>
       <c r="T19" s="64"/>
       <c r="U19" s="61"/>
       <c r="V19" s="62"/>
-      <c r="W19" s="54"/>
-      <c r="X19" s="55"/>
-      <c r="Y19" s="56"/>
-      <c r="Z19" s="54"/>
-      <c r="AA19" s="63"/>
+      <c r="W19" s="91"/>
+      <c r="X19" s="92"/>
+      <c r="Y19" s="93"/>
+      <c r="Z19" s="91"/>
+      <c r="AA19" s="94"/>
       <c r="AB19" s="57"/>
       <c r="AC19" s="58"/>
       <c r="AD19" s="59"/>
@@ -2033,22 +2066,22 @@
       <c r="I20" s="61"/>
       <c r="J20" s="62"/>
       <c r="K20" s="54"/>
-      <c r="L20" s="55"/>
-      <c r="M20" s="63"/>
+      <c r="L20" s="92"/>
+      <c r="M20" s="94"/>
       <c r="N20" s="64"/>
       <c r="O20" s="61"/>
       <c r="P20" s="62"/>
       <c r="Q20" s="54"/>
-      <c r="R20" s="55"/>
-      <c r="S20" s="63"/>
+      <c r="R20" s="92"/>
+      <c r="S20" s="94"/>
       <c r="T20" s="64"/>
       <c r="U20" s="61"/>
       <c r="V20" s="62"/>
-      <c r="W20" s="54"/>
-      <c r="X20" s="55"/>
-      <c r="Y20" s="56"/>
-      <c r="Z20" s="54"/>
-      <c r="AA20" s="63"/>
+      <c r="W20" s="91"/>
+      <c r="X20" s="92"/>
+      <c r="Y20" s="93"/>
+      <c r="Z20" s="91"/>
+      <c r="AA20" s="94"/>
       <c r="AB20" s="57"/>
       <c r="AC20" s="58"/>
       <c r="AD20" s="59"/>
@@ -2069,22 +2102,22 @@
       <c r="I21" s="61"/>
       <c r="J21" s="62"/>
       <c r="K21" s="54"/>
-      <c r="L21" s="55"/>
-      <c r="M21" s="63"/>
+      <c r="L21" s="92"/>
+      <c r="M21" s="94"/>
       <c r="N21" s="64"/>
       <c r="O21" s="61"/>
       <c r="P21" s="62"/>
       <c r="Q21" s="54"/>
-      <c r="R21" s="55"/>
-      <c r="S21" s="63"/>
+      <c r="R21" s="92"/>
+      <c r="S21" s="94"/>
       <c r="T21" s="64"/>
       <c r="U21" s="61"/>
       <c r="V21" s="62"/>
-      <c r="W21" s="54"/>
-      <c r="X21" s="55"/>
-      <c r="Y21" s="56"/>
-      <c r="Z21" s="54"/>
-      <c r="AA21" s="63"/>
+      <c r="W21" s="91"/>
+      <c r="X21" s="92"/>
+      <c r="Y21" s="93"/>
+      <c r="Z21" s="91"/>
+      <c r="AA21" s="94"/>
       <c r="AB21" s="57"/>
       <c r="AC21" s="58"/>
       <c r="AD21" s="59"/>
@@ -2105,22 +2138,22 @@
       <c r="I22" s="61"/>
       <c r="J22" s="62"/>
       <c r="K22" s="54"/>
-      <c r="L22" s="55"/>
-      <c r="M22" s="63"/>
+      <c r="L22" s="92"/>
+      <c r="M22" s="94"/>
       <c r="N22" s="64"/>
       <c r="O22" s="61"/>
       <c r="P22" s="62"/>
       <c r="Q22" s="54"/>
-      <c r="R22" s="55"/>
-      <c r="S22" s="63"/>
+      <c r="R22" s="92"/>
+      <c r="S22" s="94"/>
       <c r="T22" s="64"/>
       <c r="U22" s="61"/>
       <c r="V22" s="62"/>
-      <c r="W22" s="54"/>
-      <c r="X22" s="55"/>
-      <c r="Y22" s="56"/>
-      <c r="Z22" s="54"/>
-      <c r="AA22" s="63"/>
+      <c r="W22" s="91"/>
+      <c r="X22" s="92"/>
+      <c r="Y22" s="93"/>
+      <c r="Z22" s="91"/>
+      <c r="AA22" s="94"/>
       <c r="AB22" s="57"/>
       <c r="AC22" s="58"/>
       <c r="AD22" s="59"/>
@@ -2141,22 +2174,22 @@
       <c r="I23" s="61"/>
       <c r="J23" s="62"/>
       <c r="K23" s="54"/>
-      <c r="L23" s="55"/>
-      <c r="M23" s="63"/>
+      <c r="L23" s="92"/>
+      <c r="M23" s="94"/>
       <c r="N23" s="64"/>
       <c r="O23" s="61"/>
       <c r="P23" s="62"/>
       <c r="Q23" s="54"/>
-      <c r="R23" s="55"/>
-      <c r="S23" s="63"/>
+      <c r="R23" s="92"/>
+      <c r="S23" s="94"/>
       <c r="T23" s="64"/>
       <c r="U23" s="61"/>
       <c r="V23" s="62"/>
-      <c r="W23" s="54"/>
-      <c r="X23" s="55"/>
-      <c r="Y23" s="56"/>
-      <c r="Z23" s="54"/>
-      <c r="AA23" s="63"/>
+      <c r="W23" s="91"/>
+      <c r="X23" s="92"/>
+      <c r="Y23" s="93"/>
+      <c r="Z23" s="91"/>
+      <c r="AA23" s="94"/>
       <c r="AB23" s="57"/>
       <c r="AC23" s="58"/>
       <c r="AD23" s="59"/>
@@ -2177,22 +2210,22 @@
       <c r="I24" s="61"/>
       <c r="J24" s="62"/>
       <c r="K24" s="54"/>
-      <c r="L24" s="55"/>
-      <c r="M24" s="63"/>
+      <c r="L24" s="92"/>
+      <c r="M24" s="94"/>
       <c r="N24" s="64"/>
       <c r="O24" s="61"/>
       <c r="P24" s="62"/>
       <c r="Q24" s="54"/>
-      <c r="R24" s="55"/>
-      <c r="S24" s="63"/>
+      <c r="R24" s="92"/>
+      <c r="S24" s="94"/>
       <c r="T24" s="64"/>
       <c r="U24" s="61"/>
       <c r="V24" s="62"/>
-      <c r="W24" s="54"/>
-      <c r="X24" s="55"/>
-      <c r="Y24" s="56"/>
-      <c r="Z24" s="54"/>
-      <c r="AA24" s="63"/>
+      <c r="W24" s="91"/>
+      <c r="X24" s="92"/>
+      <c r="Y24" s="93"/>
+      <c r="Z24" s="91"/>
+      <c r="AA24" s="94"/>
       <c r="AB24" s="57"/>
       <c r="AC24" s="58"/>
       <c r="AD24" s="59"/>
@@ -2213,22 +2246,22 @@
       <c r="I25" s="61"/>
       <c r="J25" s="62"/>
       <c r="K25" s="54"/>
-      <c r="L25" s="55"/>
-      <c r="M25" s="63"/>
+      <c r="L25" s="92"/>
+      <c r="M25" s="94"/>
       <c r="N25" s="64"/>
       <c r="O25" s="61"/>
       <c r="P25" s="62"/>
       <c r="Q25" s="54"/>
-      <c r="R25" s="55"/>
-      <c r="S25" s="63"/>
+      <c r="R25" s="92"/>
+      <c r="S25" s="94"/>
       <c r="T25" s="64"/>
       <c r="U25" s="61"/>
       <c r="V25" s="62"/>
-      <c r="W25" s="54"/>
-      <c r="X25" s="55"/>
-      <c r="Y25" s="56"/>
-      <c r="Z25" s="54"/>
-      <c r="AA25" s="63"/>
+      <c r="W25" s="91"/>
+      <c r="X25" s="92"/>
+      <c r="Y25" s="93"/>
+      <c r="Z25" s="91"/>
+      <c r="AA25" s="94"/>
       <c r="AB25" s="57"/>
       <c r="AC25" s="58"/>
       <c r="AD25" s="59"/>
@@ -2249,22 +2282,22 @@
       <c r="I26" s="61"/>
       <c r="J26" s="62"/>
       <c r="K26" s="54"/>
-      <c r="L26" s="55"/>
-      <c r="M26" s="63"/>
+      <c r="L26" s="92"/>
+      <c r="M26" s="94"/>
       <c r="N26" s="64"/>
       <c r="O26" s="61"/>
       <c r="P26" s="62"/>
       <c r="Q26" s="54"/>
-      <c r="R26" s="55"/>
-      <c r="S26" s="63"/>
+      <c r="R26" s="92"/>
+      <c r="S26" s="94"/>
       <c r="T26" s="64"/>
       <c r="U26" s="61"/>
       <c r="V26" s="62"/>
-      <c r="W26" s="54"/>
-      <c r="X26" s="55"/>
-      <c r="Y26" s="56"/>
-      <c r="Z26" s="54"/>
-      <c r="AA26" s="63"/>
+      <c r="W26" s="91"/>
+      <c r="X26" s="92"/>
+      <c r="Y26" s="93"/>
+      <c r="Z26" s="91"/>
+      <c r="AA26" s="94"/>
       <c r="AB26" s="57"/>
       <c r="AC26" s="58"/>
       <c r="AD26" s="59"/>
@@ -2285,22 +2318,22 @@
       <c r="I27" s="61"/>
       <c r="J27" s="62"/>
       <c r="K27" s="54"/>
-      <c r="L27" s="55"/>
-      <c r="M27" s="63"/>
+      <c r="L27" s="92"/>
+      <c r="M27" s="94"/>
       <c r="N27" s="64"/>
       <c r="O27" s="61"/>
       <c r="P27" s="62"/>
       <c r="Q27" s="54"/>
-      <c r="R27" s="55"/>
-      <c r="S27" s="63"/>
+      <c r="R27" s="92"/>
+      <c r="S27" s="94"/>
       <c r="T27" s="64"/>
       <c r="U27" s="61"/>
       <c r="V27" s="62"/>
-      <c r="W27" s="54"/>
-      <c r="X27" s="55"/>
-      <c r="Y27" s="56"/>
-      <c r="Z27" s="54"/>
-      <c r="AA27" s="63"/>
+      <c r="W27" s="91"/>
+      <c r="X27" s="92"/>
+      <c r="Y27" s="93"/>
+      <c r="Z27" s="91"/>
+      <c r="AA27" s="94"/>
       <c r="AB27" s="57"/>
       <c r="AC27" s="58"/>
       <c r="AD27" s="59"/>
@@ -2321,22 +2354,22 @@
       <c r="I28" s="61"/>
       <c r="J28" s="62"/>
       <c r="K28" s="54"/>
-      <c r="L28" s="55"/>
-      <c r="M28" s="63"/>
+      <c r="L28" s="92"/>
+      <c r="M28" s="94"/>
       <c r="N28" s="64"/>
       <c r="O28" s="61"/>
       <c r="P28" s="62"/>
       <c r="Q28" s="54"/>
-      <c r="R28" s="55"/>
-      <c r="S28" s="63"/>
+      <c r="R28" s="92"/>
+      <c r="S28" s="94"/>
       <c r="T28" s="64"/>
       <c r="U28" s="61"/>
       <c r="V28" s="62"/>
-      <c r="W28" s="54"/>
-      <c r="X28" s="55"/>
-      <c r="Y28" s="56"/>
-      <c r="Z28" s="54"/>
-      <c r="AA28" s="63"/>
+      <c r="W28" s="91"/>
+      <c r="X28" s="92"/>
+      <c r="Y28" s="93"/>
+      <c r="Z28" s="91"/>
+      <c r="AA28" s="94"/>
       <c r="AB28" s="57"/>
       <c r="AC28" s="58"/>
       <c r="AD28" s="59"/>
@@ -2357,22 +2390,22 @@
       <c r="I29" s="61"/>
       <c r="J29" s="62"/>
       <c r="K29" s="54"/>
-      <c r="L29" s="55"/>
-      <c r="M29" s="63"/>
+      <c r="L29" s="92"/>
+      <c r="M29" s="94"/>
       <c r="N29" s="64"/>
       <c r="O29" s="61"/>
       <c r="P29" s="62"/>
       <c r="Q29" s="54"/>
-      <c r="R29" s="55"/>
-      <c r="S29" s="63"/>
+      <c r="R29" s="92"/>
+      <c r="S29" s="94"/>
       <c r="T29" s="64"/>
       <c r="U29" s="61"/>
       <c r="V29" s="62"/>
-      <c r="W29" s="54"/>
-      <c r="X29" s="55"/>
-      <c r="Y29" s="56"/>
-      <c r="Z29" s="54"/>
-      <c r="AA29" s="63"/>
+      <c r="W29" s="91"/>
+      <c r="X29" s="92"/>
+      <c r="Y29" s="93"/>
+      <c r="Z29" s="91"/>
+      <c r="AA29" s="94"/>
       <c r="AB29" s="57"/>
       <c r="AC29" s="58"/>
       <c r="AD29" s="59"/>
@@ -2393,22 +2426,22 @@
       <c r="I30" s="61"/>
       <c r="J30" s="62"/>
       <c r="K30" s="54"/>
-      <c r="L30" s="55"/>
-      <c r="M30" s="63"/>
+      <c r="L30" s="92"/>
+      <c r="M30" s="94"/>
       <c r="N30" s="64"/>
       <c r="O30" s="61"/>
       <c r="P30" s="62"/>
       <c r="Q30" s="54"/>
-      <c r="R30" s="55"/>
-      <c r="S30" s="63"/>
+      <c r="R30" s="92"/>
+      <c r="S30" s="94"/>
       <c r="T30" s="64"/>
       <c r="U30" s="61"/>
       <c r="V30" s="62"/>
-      <c r="W30" s="54"/>
-      <c r="X30" s="55"/>
-      <c r="Y30" s="56"/>
-      <c r="Z30" s="54"/>
-      <c r="AA30" s="63"/>
+      <c r="W30" s="91"/>
+      <c r="X30" s="92"/>
+      <c r="Y30" s="93"/>
+      <c r="Z30" s="91"/>
+      <c r="AA30" s="94"/>
       <c r="AB30" s="57"/>
       <c r="AC30" s="58"/>
       <c r="AD30" s="59"/>
@@ -2429,22 +2462,22 @@
       <c r="I31" s="61"/>
       <c r="J31" s="62"/>
       <c r="K31" s="54"/>
-      <c r="L31" s="55"/>
-      <c r="M31" s="63"/>
+      <c r="L31" s="92"/>
+      <c r="M31" s="94"/>
       <c r="N31" s="64"/>
       <c r="O31" s="61"/>
       <c r="P31" s="62"/>
       <c r="Q31" s="54"/>
-      <c r="R31" s="55"/>
-      <c r="S31" s="63"/>
+      <c r="R31" s="92"/>
+      <c r="S31" s="94"/>
       <c r="T31" s="64"/>
       <c r="U31" s="61"/>
       <c r="V31" s="62"/>
-      <c r="W31" s="54"/>
-      <c r="X31" s="55"/>
-      <c r="Y31" s="56"/>
-      <c r="Z31" s="54"/>
-      <c r="AA31" s="63"/>
+      <c r="W31" s="91"/>
+      <c r="X31" s="92"/>
+      <c r="Y31" s="93"/>
+      <c r="Z31" s="91"/>
+      <c r="AA31" s="94"/>
       <c r="AB31" s="57"/>
       <c r="AC31" s="58"/>
       <c r="AD31" s="59"/>
@@ -2465,22 +2498,22 @@
       <c r="I32" s="61"/>
       <c r="J32" s="62"/>
       <c r="K32" s="54"/>
-      <c r="L32" s="55"/>
-      <c r="M32" s="63"/>
+      <c r="L32" s="92"/>
+      <c r="M32" s="94"/>
       <c r="N32" s="64"/>
       <c r="O32" s="61"/>
       <c r="P32" s="62"/>
       <c r="Q32" s="54"/>
-      <c r="R32" s="55"/>
-      <c r="S32" s="63"/>
+      <c r="R32" s="92"/>
+      <c r="S32" s="94"/>
       <c r="T32" s="64"/>
       <c r="U32" s="61"/>
       <c r="V32" s="62"/>
-      <c r="W32" s="54"/>
-      <c r="X32" s="55"/>
-      <c r="Y32" s="56"/>
-      <c r="Z32" s="54"/>
-      <c r="AA32" s="63"/>
+      <c r="W32" s="91"/>
+      <c r="X32" s="92"/>
+      <c r="Y32" s="93"/>
+      <c r="Z32" s="91"/>
+      <c r="AA32" s="94"/>
       <c r="AB32" s="57"/>
       <c r="AC32" s="58"/>
       <c r="AD32" s="59"/>
@@ -2501,22 +2534,22 @@
       <c r="I33" s="61"/>
       <c r="J33" s="62"/>
       <c r="K33" s="54"/>
-      <c r="L33" s="55"/>
-      <c r="M33" s="63"/>
+      <c r="L33" s="92"/>
+      <c r="M33" s="94"/>
       <c r="N33" s="64"/>
       <c r="O33" s="61"/>
       <c r="P33" s="62"/>
       <c r="Q33" s="54"/>
-      <c r="R33" s="55"/>
-      <c r="S33" s="63"/>
+      <c r="R33" s="92"/>
+      <c r="S33" s="94"/>
       <c r="T33" s="64"/>
       <c r="U33" s="61"/>
       <c r="V33" s="62"/>
-      <c r="W33" s="54"/>
-      <c r="X33" s="55"/>
-      <c r="Y33" s="56"/>
-      <c r="Z33" s="54"/>
-      <c r="AA33" s="63"/>
+      <c r="W33" s="91"/>
+      <c r="X33" s="92"/>
+      <c r="Y33" s="93"/>
+      <c r="Z33" s="91"/>
+      <c r="AA33" s="94"/>
       <c r="AB33" s="57"/>
       <c r="AC33" s="58"/>
       <c r="AD33" s="59"/>
@@ -2537,22 +2570,22 @@
       <c r="I34" s="61"/>
       <c r="J34" s="62"/>
       <c r="K34" s="54"/>
-      <c r="L34" s="55"/>
-      <c r="M34" s="63"/>
+      <c r="L34" s="92"/>
+      <c r="M34" s="94"/>
       <c r="N34" s="64"/>
       <c r="O34" s="61"/>
       <c r="P34" s="62"/>
       <c r="Q34" s="54"/>
-      <c r="R34" s="55"/>
-      <c r="S34" s="63"/>
+      <c r="R34" s="92"/>
+      <c r="S34" s="94"/>
       <c r="T34" s="64"/>
       <c r="U34" s="61"/>
       <c r="V34" s="62"/>
-      <c r="W34" s="54"/>
-      <c r="X34" s="55"/>
-      <c r="Y34" s="56"/>
-      <c r="Z34" s="54"/>
-      <c r="AA34" s="63"/>
+      <c r="W34" s="91"/>
+      <c r="X34" s="92"/>
+      <c r="Y34" s="93"/>
+      <c r="Z34" s="91"/>
+      <c r="AA34" s="94"/>
       <c r="AB34" s="57"/>
       <c r="AC34" s="58"/>
       <c r="AD34" s="59"/>
@@ -2573,22 +2606,22 @@
       <c r="I35" s="61"/>
       <c r="J35" s="62"/>
       <c r="K35" s="54"/>
-      <c r="L35" s="55"/>
-      <c r="M35" s="63"/>
+      <c r="L35" s="92"/>
+      <c r="M35" s="94"/>
       <c r="N35" s="64"/>
       <c r="O35" s="61"/>
       <c r="P35" s="62"/>
       <c r="Q35" s="54"/>
-      <c r="R35" s="55"/>
-      <c r="S35" s="63"/>
+      <c r="R35" s="92"/>
+      <c r="S35" s="94"/>
       <c r="T35" s="64"/>
       <c r="U35" s="61"/>
       <c r="V35" s="62"/>
-      <c r="W35" s="54"/>
-      <c r="X35" s="55"/>
-      <c r="Y35" s="56"/>
-      <c r="Z35" s="54"/>
-      <c r="AA35" s="63"/>
+      <c r="W35" s="91"/>
+      <c r="X35" s="92"/>
+      <c r="Y35" s="93"/>
+      <c r="Z35" s="91"/>
+      <c r="AA35" s="94"/>
       <c r="AB35" s="57"/>
       <c r="AC35" s="58"/>
       <c r="AD35" s="59"/>
@@ -2609,22 +2642,22 @@
       <c r="I36" s="61"/>
       <c r="J36" s="62"/>
       <c r="K36" s="54"/>
-      <c r="L36" s="55"/>
-      <c r="M36" s="63"/>
+      <c r="L36" s="92"/>
+      <c r="M36" s="94"/>
       <c r="N36" s="64"/>
       <c r="O36" s="61"/>
       <c r="P36" s="62"/>
       <c r="Q36" s="54"/>
-      <c r="R36" s="55"/>
-      <c r="S36" s="63"/>
+      <c r="R36" s="92"/>
+      <c r="S36" s="94"/>
       <c r="T36" s="64"/>
       <c r="U36" s="61"/>
       <c r="V36" s="62"/>
-      <c r="W36" s="54"/>
-      <c r="X36" s="55"/>
-      <c r="Y36" s="56"/>
-      <c r="Z36" s="54"/>
-      <c r="AA36" s="63"/>
+      <c r="W36" s="91"/>
+      <c r="X36" s="92"/>
+      <c r="Y36" s="93"/>
+      <c r="Z36" s="91"/>
+      <c r="AA36" s="94"/>
       <c r="AB36" s="57"/>
       <c r="AC36" s="58"/>
       <c r="AD36" s="59"/>
@@ -2645,22 +2678,22 @@
       <c r="I37" s="61"/>
       <c r="J37" s="62"/>
       <c r="K37" s="54"/>
-      <c r="L37" s="55"/>
-      <c r="M37" s="63"/>
+      <c r="L37" s="92"/>
+      <c r="M37" s="94"/>
       <c r="N37" s="64"/>
       <c r="O37" s="61"/>
       <c r="P37" s="62"/>
       <c r="Q37" s="54"/>
-      <c r="R37" s="55"/>
-      <c r="S37" s="63"/>
+      <c r="R37" s="92"/>
+      <c r="S37" s="94"/>
       <c r="T37" s="64"/>
       <c r="U37" s="61"/>
       <c r="V37" s="62"/>
-      <c r="W37" s="54"/>
-      <c r="X37" s="55"/>
-      <c r="Y37" s="56"/>
-      <c r="Z37" s="54"/>
-      <c r="AA37" s="63"/>
+      <c r="W37" s="91"/>
+      <c r="X37" s="92"/>
+      <c r="Y37" s="93"/>
+      <c r="Z37" s="91"/>
+      <c r="AA37" s="94"/>
       <c r="AB37" s="57"/>
       <c r="AC37" s="58"/>
       <c r="AD37" s="59"/>
@@ -2681,22 +2714,22 @@
       <c r="I38" s="61"/>
       <c r="J38" s="62"/>
       <c r="K38" s="54"/>
-      <c r="L38" s="55"/>
-      <c r="M38" s="63"/>
+      <c r="L38" s="92"/>
+      <c r="M38" s="94"/>
       <c r="N38" s="64"/>
       <c r="O38" s="61"/>
       <c r="P38" s="62"/>
       <c r="Q38" s="54"/>
-      <c r="R38" s="55"/>
-      <c r="S38" s="63"/>
+      <c r="R38" s="92"/>
+      <c r="S38" s="94"/>
       <c r="T38" s="64"/>
       <c r="U38" s="61"/>
       <c r="V38" s="62"/>
-      <c r="W38" s="54"/>
-      <c r="X38" s="55"/>
-      <c r="Y38" s="56"/>
-      <c r="Z38" s="54"/>
-      <c r="AA38" s="63"/>
+      <c r="W38" s="91"/>
+      <c r="X38" s="92"/>
+      <c r="Y38" s="93"/>
+      <c r="Z38" s="91"/>
+      <c r="AA38" s="94"/>
       <c r="AB38" s="57"/>
       <c r="AC38" s="58"/>
       <c r="AD38" s="59"/>
@@ -2717,22 +2750,22 @@
       <c r="I39" s="61"/>
       <c r="J39" s="62"/>
       <c r="K39" s="54"/>
-      <c r="L39" s="55"/>
-      <c r="M39" s="63"/>
+      <c r="L39" s="92"/>
+      <c r="M39" s="94"/>
       <c r="N39" s="64"/>
       <c r="O39" s="61"/>
       <c r="P39" s="62"/>
       <c r="Q39" s="54"/>
-      <c r="R39" s="55"/>
-      <c r="S39" s="63"/>
+      <c r="R39" s="92"/>
+      <c r="S39" s="94"/>
       <c r="T39" s="64"/>
       <c r="U39" s="61"/>
       <c r="V39" s="62"/>
-      <c r="W39" s="54"/>
-      <c r="X39" s="55"/>
-      <c r="Y39" s="56"/>
-      <c r="Z39" s="54"/>
-      <c r="AA39" s="63"/>
+      <c r="W39" s="91"/>
+      <c r="X39" s="92"/>
+      <c r="Y39" s="93"/>
+      <c r="Z39" s="91"/>
+      <c r="AA39" s="94"/>
       <c r="AB39" s="57"/>
       <c r="AC39" s="58"/>
       <c r="AD39" s="59"/>
@@ -2753,22 +2786,22 @@
       <c r="I40" s="61"/>
       <c r="J40" s="62"/>
       <c r="K40" s="54"/>
-      <c r="L40" s="55"/>
-      <c r="M40" s="63"/>
+      <c r="L40" s="92"/>
+      <c r="M40" s="94"/>
       <c r="N40" s="64"/>
       <c r="O40" s="61"/>
       <c r="P40" s="62"/>
       <c r="Q40" s="54"/>
-      <c r="R40" s="55"/>
-      <c r="S40" s="63"/>
+      <c r="R40" s="92"/>
+      <c r="S40" s="94"/>
       <c r="T40" s="64"/>
       <c r="U40" s="61"/>
       <c r="V40" s="62"/>
-      <c r="W40" s="54"/>
-      <c r="X40" s="55"/>
-      <c r="Y40" s="56"/>
-      <c r="Z40" s="54"/>
-      <c r="AA40" s="63"/>
+      <c r="W40" s="91"/>
+      <c r="X40" s="92"/>
+      <c r="Y40" s="93"/>
+      <c r="Z40" s="91"/>
+      <c r="AA40" s="94"/>
       <c r="AB40" s="57"/>
       <c r="AC40" s="58"/>
       <c r="AD40" s="59"/>
@@ -2789,22 +2822,22 @@
       <c r="I41" s="61"/>
       <c r="J41" s="62"/>
       <c r="K41" s="54"/>
-      <c r="L41" s="55"/>
-      <c r="M41" s="63"/>
+      <c r="L41" s="92"/>
+      <c r="M41" s="94"/>
       <c r="N41" s="64"/>
       <c r="O41" s="61"/>
       <c r="P41" s="62"/>
       <c r="Q41" s="54"/>
-      <c r="R41" s="55"/>
-      <c r="S41" s="63"/>
+      <c r="R41" s="92"/>
+      <c r="S41" s="94"/>
       <c r="T41" s="64"/>
       <c r="U41" s="61"/>
       <c r="V41" s="62"/>
-      <c r="W41" s="54"/>
-      <c r="X41" s="55"/>
-      <c r="Y41" s="56"/>
-      <c r="Z41" s="54"/>
-      <c r="AA41" s="63"/>
+      <c r="W41" s="91"/>
+      <c r="X41" s="92"/>
+      <c r="Y41" s="93"/>
+      <c r="Z41" s="91"/>
+      <c r="AA41" s="94"/>
       <c r="AB41" s="57"/>
       <c r="AC41" s="58"/>
       <c r="AD41" s="59"/>
@@ -2825,22 +2858,22 @@
       <c r="I42" s="61"/>
       <c r="J42" s="62"/>
       <c r="K42" s="54"/>
-      <c r="L42" s="55"/>
-      <c r="M42" s="63"/>
+      <c r="L42" s="92"/>
+      <c r="M42" s="94"/>
       <c r="N42" s="64"/>
       <c r="O42" s="61"/>
       <c r="P42" s="62"/>
       <c r="Q42" s="54"/>
-      <c r="R42" s="55"/>
-      <c r="S42" s="63"/>
+      <c r="R42" s="92"/>
+      <c r="S42" s="94"/>
       <c r="T42" s="64"/>
       <c r="U42" s="61"/>
       <c r="V42" s="62"/>
-      <c r="W42" s="54"/>
-      <c r="X42" s="55"/>
-      <c r="Y42" s="56"/>
-      <c r="Z42" s="54"/>
-      <c r="AA42" s="63"/>
+      <c r="W42" s="91"/>
+      <c r="X42" s="92"/>
+      <c r="Y42" s="93"/>
+      <c r="Z42" s="91"/>
+      <c r="AA42" s="94"/>
       <c r="AB42" s="57"/>
       <c r="AC42" s="58"/>
       <c r="AD42" s="59"/>
@@ -2861,22 +2894,22 @@
       <c r="I43" s="61"/>
       <c r="J43" s="62"/>
       <c r="K43" s="54"/>
-      <c r="L43" s="55"/>
-      <c r="M43" s="63"/>
+      <c r="L43" s="92"/>
+      <c r="M43" s="94"/>
       <c r="N43" s="64"/>
       <c r="O43" s="61"/>
       <c r="P43" s="62"/>
       <c r="Q43" s="54"/>
-      <c r="R43" s="55"/>
-      <c r="S43" s="63"/>
+      <c r="R43" s="92"/>
+      <c r="S43" s="94"/>
       <c r="T43" s="64"/>
       <c r="U43" s="61"/>
       <c r="V43" s="62"/>
-      <c r="W43" s="54"/>
-      <c r="X43" s="55"/>
-      <c r="Y43" s="56"/>
-      <c r="Z43" s="54"/>
-      <c r="AA43" s="63"/>
+      <c r="W43" s="91"/>
+      <c r="X43" s="92"/>
+      <c r="Y43" s="93"/>
+      <c r="Z43" s="91"/>
+      <c r="AA43" s="94"/>
       <c r="AB43" s="57"/>
       <c r="AC43" s="58"/>
       <c r="AD43" s="59"/>
@@ -2897,22 +2930,22 @@
       <c r="I44" s="61"/>
       <c r="J44" s="62"/>
       <c r="K44" s="54"/>
-      <c r="L44" s="55"/>
-      <c r="M44" s="63"/>
+      <c r="L44" s="92"/>
+      <c r="M44" s="94"/>
       <c r="N44" s="64"/>
       <c r="O44" s="61"/>
       <c r="P44" s="62"/>
       <c r="Q44" s="54"/>
-      <c r="R44" s="55"/>
-      <c r="S44" s="63"/>
+      <c r="R44" s="92"/>
+      <c r="S44" s="94"/>
       <c r="T44" s="64"/>
       <c r="U44" s="61"/>
       <c r="V44" s="62"/>
-      <c r="W44" s="54"/>
-      <c r="X44" s="55"/>
-      <c r="Y44" s="56"/>
-      <c r="Z44" s="54"/>
-      <c r="AA44" s="63"/>
+      <c r="W44" s="91"/>
+      <c r="X44" s="92"/>
+      <c r="Y44" s="93"/>
+      <c r="Z44" s="91"/>
+      <c r="AA44" s="94"/>
       <c r="AB44" s="57"/>
       <c r="AC44" s="58"/>
       <c r="AD44" s="59"/>
@@ -2933,22 +2966,22 @@
       <c r="I45" s="61"/>
       <c r="J45" s="62"/>
       <c r="K45" s="54"/>
-      <c r="L45" s="55"/>
-      <c r="M45" s="63"/>
+      <c r="L45" s="92"/>
+      <c r="M45" s="94"/>
       <c r="N45" s="64"/>
       <c r="O45" s="61"/>
       <c r="P45" s="62"/>
       <c r="Q45" s="54"/>
-      <c r="R45" s="55"/>
-      <c r="S45" s="63"/>
+      <c r="R45" s="92"/>
+      <c r="S45" s="94"/>
       <c r="T45" s="64"/>
       <c r="U45" s="61"/>
       <c r="V45" s="62"/>
-      <c r="W45" s="54"/>
-      <c r="X45" s="55"/>
-      <c r="Y45" s="56"/>
-      <c r="Z45" s="54"/>
-      <c r="AA45" s="63"/>
+      <c r="W45" s="91"/>
+      <c r="X45" s="92"/>
+      <c r="Y45" s="93"/>
+      <c r="Z45" s="91"/>
+      <c r="AA45" s="94"/>
       <c r="AB45" s="57"/>
       <c r="AC45" s="58"/>
       <c r="AD45" s="59"/>
@@ -2969,22 +3002,22 @@
       <c r="I46" s="61"/>
       <c r="J46" s="62"/>
       <c r="K46" s="54"/>
-      <c r="L46" s="55"/>
-      <c r="M46" s="63"/>
+      <c r="L46" s="92"/>
+      <c r="M46" s="94"/>
       <c r="N46" s="64"/>
       <c r="O46" s="61"/>
       <c r="P46" s="62"/>
       <c r="Q46" s="54"/>
-      <c r="R46" s="55"/>
-      <c r="S46" s="63"/>
+      <c r="R46" s="92"/>
+      <c r="S46" s="94"/>
       <c r="T46" s="64"/>
       <c r="U46" s="61"/>
       <c r="V46" s="62"/>
-      <c r="W46" s="54"/>
-      <c r="X46" s="55"/>
-      <c r="Y46" s="56"/>
-      <c r="Z46" s="54"/>
-      <c r="AA46" s="63"/>
+      <c r="W46" s="91"/>
+      <c r="X46" s="92"/>
+      <c r="Y46" s="93"/>
+      <c r="Z46" s="91"/>
+      <c r="AA46" s="94"/>
       <c r="AB46" s="57"/>
       <c r="AC46" s="58"/>
       <c r="AD46" s="59"/>
@@ -3005,22 +3038,22 @@
       <c r="I47" s="61"/>
       <c r="J47" s="62"/>
       <c r="K47" s="54"/>
-      <c r="L47" s="55"/>
-      <c r="M47" s="63"/>
+      <c r="L47" s="92"/>
+      <c r="M47" s="94"/>
       <c r="N47" s="64"/>
       <c r="O47" s="61"/>
       <c r="P47" s="62"/>
       <c r="Q47" s="54"/>
-      <c r="R47" s="55"/>
-      <c r="S47" s="63"/>
+      <c r="R47" s="92"/>
+      <c r="S47" s="94"/>
       <c r="T47" s="64"/>
       <c r="U47" s="61"/>
       <c r="V47" s="62"/>
-      <c r="W47" s="54"/>
-      <c r="X47" s="55"/>
-      <c r="Y47" s="56"/>
-      <c r="Z47" s="54"/>
-      <c r="AA47" s="63"/>
+      <c r="W47" s="91"/>
+      <c r="X47" s="92"/>
+      <c r="Y47" s="93"/>
+      <c r="Z47" s="91"/>
+      <c r="AA47" s="94"/>
       <c r="AB47" s="57"/>
       <c r="AC47" s="58"/>
       <c r="AD47" s="59"/>
@@ -3041,22 +3074,22 @@
       <c r="I48" s="61"/>
       <c r="J48" s="62"/>
       <c r="K48" s="54"/>
-      <c r="L48" s="55"/>
-      <c r="M48" s="63"/>
+      <c r="L48" s="92"/>
+      <c r="M48" s="94"/>
       <c r="N48" s="64"/>
       <c r="O48" s="61"/>
       <c r="P48" s="62"/>
       <c r="Q48" s="54"/>
-      <c r="R48" s="55"/>
-      <c r="S48" s="63"/>
+      <c r="R48" s="92"/>
+      <c r="S48" s="94"/>
       <c r="T48" s="64"/>
       <c r="U48" s="61"/>
       <c r="V48" s="62"/>
-      <c r="W48" s="54"/>
-      <c r="X48" s="55"/>
-      <c r="Y48" s="56"/>
-      <c r="Z48" s="54"/>
-      <c r="AA48" s="63"/>
+      <c r="W48" s="91"/>
+      <c r="X48" s="92"/>
+      <c r="Y48" s="93"/>
+      <c r="Z48" s="91"/>
+      <c r="AA48" s="94"/>
       <c r="AB48" s="57"/>
       <c r="AC48" s="58"/>
       <c r="AD48" s="59"/>
@@ -3077,22 +3110,22 @@
       <c r="I49" s="61"/>
       <c r="J49" s="62"/>
       <c r="K49" s="54"/>
-      <c r="L49" s="55"/>
-      <c r="M49" s="63"/>
+      <c r="L49" s="92"/>
+      <c r="M49" s="94"/>
       <c r="N49" s="64"/>
       <c r="O49" s="61"/>
       <c r="P49" s="62"/>
       <c r="Q49" s="54"/>
-      <c r="R49" s="55"/>
-      <c r="S49" s="63"/>
+      <c r="R49" s="92"/>
+      <c r="S49" s="94"/>
       <c r="T49" s="64"/>
       <c r="U49" s="61"/>
       <c r="V49" s="62"/>
-      <c r="W49" s="54"/>
-      <c r="X49" s="55"/>
-      <c r="Y49" s="56"/>
-      <c r="Z49" s="54"/>
-      <c r="AA49" s="63"/>
+      <c r="W49" s="91"/>
+      <c r="X49" s="92"/>
+      <c r="Y49" s="93"/>
+      <c r="Z49" s="91"/>
+      <c r="AA49" s="94"/>
       <c r="AB49" s="57"/>
       <c r="AC49" s="58"/>
       <c r="AD49" s="59"/>
@@ -3113,22 +3146,22 @@
       <c r="I50" s="61"/>
       <c r="J50" s="62"/>
       <c r="K50" s="54"/>
-      <c r="L50" s="55"/>
-      <c r="M50" s="63"/>
+      <c r="L50" s="92"/>
+      <c r="M50" s="94"/>
       <c r="N50" s="64"/>
       <c r="O50" s="61"/>
       <c r="P50" s="62"/>
       <c r="Q50" s="54"/>
-      <c r="R50" s="55"/>
-      <c r="S50" s="63"/>
+      <c r="R50" s="92"/>
+      <c r="S50" s="94"/>
       <c r="T50" s="64"/>
       <c r="U50" s="61"/>
       <c r="V50" s="62"/>
-      <c r="W50" s="54"/>
-      <c r="X50" s="55"/>
-      <c r="Y50" s="56"/>
-      <c r="Z50" s="54"/>
-      <c r="AA50" s="63"/>
+      <c r="W50" s="91"/>
+      <c r="X50" s="92"/>
+      <c r="Y50" s="93"/>
+      <c r="Z50" s="91"/>
+      <c r="AA50" s="94"/>
       <c r="AB50" s="57"/>
       <c r="AC50" s="58"/>
       <c r="AD50" s="59"/>
@@ -3149,22 +3182,22 @@
       <c r="I51" s="61"/>
       <c r="J51" s="62"/>
       <c r="K51" s="54"/>
-      <c r="L51" s="55"/>
-      <c r="M51" s="63"/>
+      <c r="L51" s="92"/>
+      <c r="M51" s="94"/>
       <c r="N51" s="64"/>
       <c r="O51" s="61"/>
       <c r="P51" s="62"/>
       <c r="Q51" s="54"/>
-      <c r="R51" s="55"/>
-      <c r="S51" s="63"/>
+      <c r="R51" s="92"/>
+      <c r="S51" s="94"/>
       <c r="T51" s="64"/>
       <c r="U51" s="61"/>
       <c r="V51" s="62"/>
-      <c r="W51" s="54"/>
-      <c r="X51" s="55"/>
-      <c r="Y51" s="56"/>
-      <c r="Z51" s="54"/>
-      <c r="AA51" s="63"/>
+      <c r="W51" s="91"/>
+      <c r="X51" s="92"/>
+      <c r="Y51" s="93"/>
+      <c r="Z51" s="91"/>
+      <c r="AA51" s="94"/>
       <c r="AB51" s="57"/>
       <c r="AC51" s="58"/>
       <c r="AD51" s="59"/>
@@ -3185,22 +3218,22 @@
       <c r="I52" s="61"/>
       <c r="J52" s="62"/>
       <c r="K52" s="54"/>
-      <c r="L52" s="55"/>
-      <c r="M52" s="63"/>
+      <c r="L52" s="92"/>
+      <c r="M52" s="94"/>
       <c r="N52" s="64"/>
       <c r="O52" s="61"/>
       <c r="P52" s="62"/>
       <c r="Q52" s="54"/>
-      <c r="R52" s="55"/>
-      <c r="S52" s="63"/>
+      <c r="R52" s="92"/>
+      <c r="S52" s="94"/>
       <c r="T52" s="64"/>
       <c r="U52" s="61"/>
       <c r="V52" s="62"/>
-      <c r="W52" s="54"/>
-      <c r="X52" s="55"/>
-      <c r="Y52" s="56"/>
-      <c r="Z52" s="54"/>
-      <c r="AA52" s="63"/>
+      <c r="W52" s="91"/>
+      <c r="X52" s="92"/>
+      <c r="Y52" s="93"/>
+      <c r="Z52" s="91"/>
+      <c r="AA52" s="94"/>
       <c r="AB52" s="57"/>
       <c r="AC52" s="58"/>
       <c r="AD52" s="59"/>
@@ -3221,22 +3254,22 @@
       <c r="I53" s="61"/>
       <c r="J53" s="62"/>
       <c r="K53" s="54"/>
-      <c r="L53" s="55"/>
-      <c r="M53" s="63"/>
+      <c r="L53" s="92"/>
+      <c r="M53" s="94"/>
       <c r="N53" s="64"/>
       <c r="O53" s="61"/>
       <c r="P53" s="62"/>
       <c r="Q53" s="54"/>
-      <c r="R53" s="55"/>
-      <c r="S53" s="63"/>
+      <c r="R53" s="92"/>
+      <c r="S53" s="94"/>
       <c r="T53" s="64"/>
       <c r="U53" s="61"/>
       <c r="V53" s="62"/>
-      <c r="W53" s="54"/>
-      <c r="X53" s="55"/>
-      <c r="Y53" s="56"/>
-      <c r="Z53" s="54"/>
-      <c r="AA53" s="63"/>
+      <c r="W53" s="91"/>
+      <c r="X53" s="92"/>
+      <c r="Y53" s="93"/>
+      <c r="Z53" s="91"/>
+      <c r="AA53" s="94"/>
       <c r="AB53" s="57"/>
       <c r="AC53" s="58"/>
       <c r="AD53" s="59"/>
@@ -3257,22 +3290,22 @@
       <c r="I54" s="61"/>
       <c r="J54" s="62"/>
       <c r="K54" s="54"/>
-      <c r="L54" s="55"/>
-      <c r="M54" s="63"/>
+      <c r="L54" s="92"/>
+      <c r="M54" s="94"/>
       <c r="N54" s="64"/>
       <c r="O54" s="61"/>
       <c r="P54" s="62"/>
       <c r="Q54" s="54"/>
-      <c r="R54" s="55"/>
-      <c r="S54" s="63"/>
+      <c r="R54" s="92"/>
+      <c r="S54" s="94"/>
       <c r="T54" s="64"/>
       <c r="U54" s="61"/>
       <c r="V54" s="62"/>
-      <c r="W54" s="54"/>
-      <c r="X54" s="55"/>
-      <c r="Y54" s="56"/>
-      <c r="Z54" s="54"/>
-      <c r="AA54" s="63"/>
+      <c r="W54" s="91"/>
+      <c r="X54" s="92"/>
+      <c r="Y54" s="93"/>
+      <c r="Z54" s="91"/>
+      <c r="AA54" s="94"/>
       <c r="AB54" s="57"/>
       <c r="AC54" s="58"/>
       <c r="AD54" s="59"/>
@@ -3293,22 +3326,22 @@
       <c r="I55" s="61"/>
       <c r="J55" s="62"/>
       <c r="K55" s="54"/>
-      <c r="L55" s="55"/>
-      <c r="M55" s="63"/>
+      <c r="L55" s="92"/>
+      <c r="M55" s="94"/>
       <c r="N55" s="64"/>
       <c r="O55" s="61"/>
       <c r="P55" s="62"/>
       <c r="Q55" s="54"/>
-      <c r="R55" s="55"/>
-      <c r="S55" s="63"/>
+      <c r="R55" s="92"/>
+      <c r="S55" s="94"/>
       <c r="T55" s="64"/>
       <c r="U55" s="61"/>
       <c r="V55" s="62"/>
-      <c r="W55" s="54"/>
-      <c r="X55" s="55"/>
-      <c r="Y55" s="56"/>
-      <c r="Z55" s="54"/>
-      <c r="AA55" s="63"/>
+      <c r="W55" s="91"/>
+      <c r="X55" s="92"/>
+      <c r="Y55" s="93"/>
+      <c r="Z55" s="91"/>
+      <c r="AA55" s="94"/>
       <c r="AB55" s="57"/>
       <c r="AC55" s="58"/>
       <c r="AD55" s="59"/>
@@ -3329,22 +3362,22 @@
       <c r="I56" s="61"/>
       <c r="J56" s="62"/>
       <c r="K56" s="54"/>
-      <c r="L56" s="55"/>
-      <c r="M56" s="63"/>
+      <c r="L56" s="92"/>
+      <c r="M56" s="94"/>
       <c r="N56" s="64"/>
       <c r="O56" s="61"/>
       <c r="P56" s="62"/>
       <c r="Q56" s="54"/>
-      <c r="R56" s="55"/>
-      <c r="S56" s="63"/>
+      <c r="R56" s="92"/>
+      <c r="S56" s="94"/>
       <c r="T56" s="64"/>
       <c r="U56" s="61"/>
       <c r="V56" s="62"/>
-      <c r="W56" s="54"/>
-      <c r="X56" s="55"/>
-      <c r="Y56" s="56"/>
-      <c r="Z56" s="54"/>
-      <c r="AA56" s="63"/>
+      <c r="W56" s="91"/>
+      <c r="X56" s="92"/>
+      <c r="Y56" s="93"/>
+      <c r="Z56" s="91"/>
+      <c r="AA56" s="94"/>
       <c r="AB56" s="57"/>
       <c r="AC56" s="58"/>
       <c r="AD56" s="59"/>
@@ -3365,22 +3398,22 @@
       <c r="I57" s="61"/>
       <c r="J57" s="62"/>
       <c r="K57" s="54"/>
-      <c r="L57" s="55"/>
-      <c r="M57" s="63"/>
+      <c r="L57" s="92"/>
+      <c r="M57" s="94"/>
       <c r="N57" s="64"/>
       <c r="O57" s="61"/>
       <c r="P57" s="62"/>
       <c r="Q57" s="54"/>
-      <c r="R57" s="55"/>
-      <c r="S57" s="63"/>
+      <c r="R57" s="92"/>
+      <c r="S57" s="94"/>
       <c r="T57" s="64"/>
       <c r="U57" s="61"/>
       <c r="V57" s="62"/>
-      <c r="W57" s="54"/>
-      <c r="X57" s="55"/>
-      <c r="Y57" s="56"/>
-      <c r="Z57" s="54"/>
-      <c r="AA57" s="63"/>
+      <c r="W57" s="91"/>
+      <c r="X57" s="92"/>
+      <c r="Y57" s="93"/>
+      <c r="Z57" s="91"/>
+      <c r="AA57" s="94"/>
       <c r="AB57" s="57"/>
       <c r="AC57" s="58"/>
       <c r="AD57" s="59"/>
@@ -3401,22 +3434,22 @@
       <c r="I58" s="61"/>
       <c r="J58" s="62"/>
       <c r="K58" s="54"/>
-      <c r="L58" s="55"/>
-      <c r="M58" s="63"/>
+      <c r="L58" s="92"/>
+      <c r="M58" s="94"/>
       <c r="N58" s="64"/>
       <c r="O58" s="61"/>
       <c r="P58" s="62"/>
       <c r="Q58" s="54"/>
-      <c r="R58" s="55"/>
-      <c r="S58" s="63"/>
+      <c r="R58" s="92"/>
+      <c r="S58" s="94"/>
       <c r="T58" s="64"/>
       <c r="U58" s="61"/>
       <c r="V58" s="62"/>
-      <c r="W58" s="54"/>
-      <c r="X58" s="55"/>
-      <c r="Y58" s="56"/>
-      <c r="Z58" s="54"/>
-      <c r="AA58" s="63"/>
+      <c r="W58" s="91"/>
+      <c r="X58" s="92"/>
+      <c r="Y58" s="93"/>
+      <c r="Z58" s="91"/>
+      <c r="AA58" s="94"/>
       <c r="AB58" s="57"/>
       <c r="AC58" s="58"/>
       <c r="AD58" s="59"/>
@@ -3437,22 +3470,22 @@
       <c r="I59" s="61"/>
       <c r="J59" s="62"/>
       <c r="K59" s="54"/>
-      <c r="L59" s="55"/>
-      <c r="M59" s="63"/>
+      <c r="L59" s="92"/>
+      <c r="M59" s="94"/>
       <c r="N59" s="64"/>
       <c r="O59" s="61"/>
       <c r="P59" s="62"/>
       <c r="Q59" s="54"/>
-      <c r="R59" s="55"/>
-      <c r="S59" s="63"/>
+      <c r="R59" s="92"/>
+      <c r="S59" s="94"/>
       <c r="T59" s="64"/>
       <c r="U59" s="61"/>
       <c r="V59" s="62"/>
-      <c r="W59" s="54"/>
-      <c r="X59" s="55"/>
-      <c r="Y59" s="56"/>
-      <c r="Z59" s="54"/>
-      <c r="AA59" s="63"/>
+      <c r="W59" s="91"/>
+      <c r="X59" s="92"/>
+      <c r="Y59" s="93"/>
+      <c r="Z59" s="91"/>
+      <c r="AA59" s="94"/>
       <c r="AB59" s="57"/>
       <c r="AC59" s="58"/>
       <c r="AD59" s="59"/>
@@ -3473,22 +3506,22 @@
       <c r="I60" s="61"/>
       <c r="J60" s="62"/>
       <c r="K60" s="54"/>
-      <c r="L60" s="55"/>
-      <c r="M60" s="63"/>
+      <c r="L60" s="92"/>
+      <c r="M60" s="94"/>
       <c r="N60" s="64"/>
       <c r="O60" s="61"/>
       <c r="P60" s="62"/>
       <c r="Q60" s="54"/>
-      <c r="R60" s="55"/>
-      <c r="S60" s="63"/>
+      <c r="R60" s="92"/>
+      <c r="S60" s="94"/>
       <c r="T60" s="64"/>
       <c r="U60" s="61"/>
       <c r="V60" s="62"/>
-      <c r="W60" s="54"/>
-      <c r="X60" s="55"/>
-      <c r="Y60" s="56"/>
-      <c r="Z60" s="54"/>
-      <c r="AA60" s="63"/>
+      <c r="W60" s="91"/>
+      <c r="X60" s="92"/>
+      <c r="Y60" s="93"/>
+      <c r="Z60" s="91"/>
+      <c r="AA60" s="94"/>
       <c r="AB60" s="57"/>
       <c r="AC60" s="58"/>
       <c r="AD60" s="59"/>
@@ -3509,22 +3542,22 @@
       <c r="I61" s="61"/>
       <c r="J61" s="62"/>
       <c r="K61" s="54"/>
-      <c r="L61" s="55"/>
-      <c r="M61" s="63"/>
+      <c r="L61" s="92"/>
+      <c r="M61" s="94"/>
       <c r="N61" s="64"/>
       <c r="O61" s="61"/>
       <c r="P61" s="62"/>
       <c r="Q61" s="54"/>
-      <c r="R61" s="55"/>
-      <c r="S61" s="63"/>
+      <c r="R61" s="92"/>
+      <c r="S61" s="94"/>
       <c r="T61" s="64"/>
       <c r="U61" s="61"/>
       <c r="V61" s="62"/>
-      <c r="W61" s="54"/>
-      <c r="X61" s="55"/>
-      <c r="Y61" s="56"/>
-      <c r="Z61" s="54"/>
-      <c r="AA61" s="63"/>
+      <c r="W61" s="91"/>
+      <c r="X61" s="92"/>
+      <c r="Y61" s="93"/>
+      <c r="Z61" s="91"/>
+      <c r="AA61" s="94"/>
       <c r="AB61" s="57"/>
       <c r="AC61" s="58"/>
       <c r="AD61" s="59"/>
@@ -3545,22 +3578,22 @@
       <c r="I62" s="61"/>
       <c r="J62" s="62"/>
       <c r="K62" s="54"/>
-      <c r="L62" s="55"/>
-      <c r="M62" s="63"/>
+      <c r="L62" s="92"/>
+      <c r="M62" s="94"/>
       <c r="N62" s="64"/>
       <c r="O62" s="61"/>
       <c r="P62" s="62"/>
       <c r="Q62" s="54"/>
-      <c r="R62" s="55"/>
-      <c r="S62" s="63"/>
+      <c r="R62" s="92"/>
+      <c r="S62" s="94"/>
       <c r="T62" s="64"/>
       <c r="U62" s="61"/>
       <c r="V62" s="62"/>
-      <c r="W62" s="54"/>
-      <c r="X62" s="55"/>
-      <c r="Y62" s="56"/>
-      <c r="Z62" s="54"/>
-      <c r="AA62" s="63"/>
+      <c r="W62" s="91"/>
+      <c r="X62" s="92"/>
+      <c r="Y62" s="93"/>
+      <c r="Z62" s="91"/>
+      <c r="AA62" s="94"/>
       <c r="AB62" s="57"/>
       <c r="AC62" s="58"/>
       <c r="AD62" s="59"/>
@@ -3581,22 +3614,22 @@
       <c r="I63" s="61"/>
       <c r="J63" s="62"/>
       <c r="K63" s="54"/>
-      <c r="L63" s="55"/>
-      <c r="M63" s="63"/>
+      <c r="L63" s="92"/>
+      <c r="M63" s="94"/>
       <c r="N63" s="64"/>
       <c r="O63" s="61"/>
       <c r="P63" s="62"/>
       <c r="Q63" s="54"/>
-      <c r="R63" s="55"/>
-      <c r="S63" s="63"/>
+      <c r="R63" s="92"/>
+      <c r="S63" s="94"/>
       <c r="T63" s="64"/>
       <c r="U63" s="61"/>
       <c r="V63" s="62"/>
-      <c r="W63" s="54"/>
-      <c r="X63" s="55"/>
-      <c r="Y63" s="56"/>
-      <c r="Z63" s="54"/>
-      <c r="AA63" s="63"/>
+      <c r="W63" s="91"/>
+      <c r="X63" s="92"/>
+      <c r="Y63" s="93"/>
+      <c r="Z63" s="91"/>
+      <c r="AA63" s="94"/>
       <c r="AB63" s="57"/>
       <c r="AC63" s="58"/>
       <c r="AD63" s="59"/>
@@ -3617,22 +3650,22 @@
       <c r="I64" s="61"/>
       <c r="J64" s="62"/>
       <c r="K64" s="54"/>
-      <c r="L64" s="55"/>
-      <c r="M64" s="63"/>
+      <c r="L64" s="92"/>
+      <c r="M64" s="94"/>
       <c r="N64" s="64"/>
       <c r="O64" s="61"/>
       <c r="P64" s="62"/>
       <c r="Q64" s="54"/>
-      <c r="R64" s="55"/>
-      <c r="S64" s="63"/>
+      <c r="R64" s="92"/>
+      <c r="S64" s="94"/>
       <c r="T64" s="64"/>
       <c r="U64" s="61"/>
       <c r="V64" s="62"/>
-      <c r="W64" s="54"/>
-      <c r="X64" s="55"/>
-      <c r="Y64" s="56"/>
-      <c r="Z64" s="54"/>
-      <c r="AA64" s="63"/>
+      <c r="W64" s="91"/>
+      <c r="X64" s="92"/>
+      <c r="Y64" s="93"/>
+      <c r="Z64" s="91"/>
+      <c r="AA64" s="94"/>
       <c r="AB64" s="57"/>
       <c r="AC64" s="58"/>
       <c r="AD64" s="59"/>
@@ -3653,22 +3686,22 @@
       <c r="I65" s="61"/>
       <c r="J65" s="62"/>
       <c r="K65" s="54"/>
-      <c r="L65" s="55"/>
-      <c r="M65" s="63"/>
+      <c r="L65" s="92"/>
+      <c r="M65" s="94"/>
       <c r="N65" s="64"/>
       <c r="O65" s="61"/>
       <c r="P65" s="62"/>
       <c r="Q65" s="54"/>
-      <c r="R65" s="55"/>
-      <c r="S65" s="63"/>
+      <c r="R65" s="92"/>
+      <c r="S65" s="94"/>
       <c r="T65" s="64"/>
       <c r="U65" s="61"/>
       <c r="V65" s="62"/>
-      <c r="W65" s="54"/>
-      <c r="X65" s="55"/>
-      <c r="Y65" s="56"/>
-      <c r="Z65" s="54"/>
-      <c r="AA65" s="63"/>
+      <c r="W65" s="91"/>
+      <c r="X65" s="92"/>
+      <c r="Y65" s="93"/>
+      <c r="Z65" s="91"/>
+      <c r="AA65" s="94"/>
       <c r="AB65" s="57"/>
       <c r="AC65" s="58"/>
       <c r="AD65" s="59"/>
@@ -3689,22 +3722,22 @@
       <c r="I66" s="61"/>
       <c r="J66" s="62"/>
       <c r="K66" s="54"/>
-      <c r="L66" s="55"/>
-      <c r="M66" s="63"/>
+      <c r="L66" s="92"/>
+      <c r="M66" s="94"/>
       <c r="N66" s="64"/>
       <c r="O66" s="61"/>
       <c r="P66" s="62"/>
       <c r="Q66" s="54"/>
-      <c r="R66" s="55"/>
-      <c r="S66" s="63"/>
+      <c r="R66" s="92"/>
+      <c r="S66" s="94"/>
       <c r="T66" s="64"/>
       <c r="U66" s="61"/>
       <c r="V66" s="62"/>
-      <c r="W66" s="54"/>
-      <c r="X66" s="55"/>
-      <c r="Y66" s="56"/>
-      <c r="Z66" s="54"/>
-      <c r="AA66" s="63"/>
+      <c r="W66" s="91"/>
+      <c r="X66" s="92"/>
+      <c r="Y66" s="93"/>
+      <c r="Z66" s="91"/>
+      <c r="AA66" s="94"/>
       <c r="AB66" s="57"/>
       <c r="AC66" s="58"/>
       <c r="AD66" s="59"/>
@@ -3725,22 +3758,22 @@
       <c r="I67" s="61"/>
       <c r="J67" s="62"/>
       <c r="K67" s="54"/>
-      <c r="L67" s="55"/>
-      <c r="M67" s="63"/>
+      <c r="L67" s="92"/>
+      <c r="M67" s="94"/>
       <c r="N67" s="64"/>
       <c r="O67" s="61"/>
       <c r="P67" s="62"/>
       <c r="Q67" s="54"/>
-      <c r="R67" s="55"/>
-      <c r="S67" s="63"/>
+      <c r="R67" s="92"/>
+      <c r="S67" s="94"/>
       <c r="T67" s="64"/>
       <c r="U67" s="61"/>
       <c r="V67" s="62"/>
-      <c r="W67" s="54"/>
-      <c r="X67" s="55"/>
-      <c r="Y67" s="56"/>
-      <c r="Z67" s="54"/>
-      <c r="AA67" s="63"/>
+      <c r="W67" s="91"/>
+      <c r="X67" s="92"/>
+      <c r="Y67" s="93"/>
+      <c r="Z67" s="91"/>
+      <c r="AA67" s="94"/>
       <c r="AB67" s="57"/>
       <c r="AC67" s="58"/>
       <c r="AD67" s="59"/>
@@ -3797,22 +3830,22 @@
       <c r="I69" s="48"/>
       <c r="J69" s="49"/>
       <c r="K69" s="50"/>
-      <c r="L69" s="51"/>
-      <c r="M69" s="52"/>
+      <c r="L69" s="89"/>
+      <c r="M69" s="90"/>
       <c r="N69" s="53"/>
       <c r="O69" s="48"/>
       <c r="P69" s="49"/>
       <c r="Q69" s="50"/>
-      <c r="R69" s="51"/>
-      <c r="S69" s="52"/>
+      <c r="R69" s="89"/>
+      <c r="S69" s="90"/>
       <c r="T69" s="53"/>
       <c r="U69" s="48"/>
       <c r="V69" s="49"/>
-      <c r="W69" s="54"/>
-      <c r="X69" s="55"/>
-      <c r="Y69" s="56"/>
-      <c r="Z69" s="50"/>
-      <c r="AA69" s="52"/>
+      <c r="W69" s="91"/>
+      <c r="X69" s="92"/>
+      <c r="Y69" s="93"/>
+      <c r="Z69" s="88"/>
+      <c r="AA69" s="90"/>
       <c r="AB69" s="57"/>
       <c r="AC69" s="58"/>
       <c r="AD69" s="69"/>
@@ -3833,22 +3866,22 @@
       <c r="I70" s="61"/>
       <c r="J70" s="62"/>
       <c r="K70" s="54"/>
-      <c r="L70" s="55"/>
-      <c r="M70" s="63"/>
+      <c r="L70" s="92"/>
+      <c r="M70" s="94"/>
       <c r="N70" s="64"/>
       <c r="O70" s="61"/>
       <c r="P70" s="62"/>
       <c r="Q70" s="54"/>
-      <c r="R70" s="55"/>
-      <c r="S70" s="63"/>
+      <c r="R70" s="92"/>
+      <c r="S70" s="94"/>
       <c r="T70" s="64"/>
       <c r="U70" s="61"/>
       <c r="V70" s="62"/>
-      <c r="W70" s="54"/>
-      <c r="X70" s="55"/>
-      <c r="Y70" s="56"/>
-      <c r="Z70" s="54"/>
-      <c r="AA70" s="63"/>
+      <c r="W70" s="91"/>
+      <c r="X70" s="92"/>
+      <c r="Y70" s="93"/>
+      <c r="Z70" s="91"/>
+      <c r="AA70" s="94"/>
       <c r="AB70" s="57"/>
       <c r="AC70" s="58"/>
       <c r="AD70" s="59"/>
@@ -3869,22 +3902,22 @@
       <c r="I71" s="61"/>
       <c r="J71" s="62"/>
       <c r="K71" s="54"/>
-      <c r="L71" s="55"/>
-      <c r="M71" s="63"/>
+      <c r="L71" s="92"/>
+      <c r="M71" s="94"/>
       <c r="N71" s="64"/>
       <c r="O71" s="61"/>
       <c r="P71" s="62"/>
       <c r="Q71" s="54"/>
-      <c r="R71" s="55"/>
-      <c r="S71" s="63"/>
+      <c r="R71" s="92"/>
+      <c r="S71" s="94"/>
       <c r="T71" s="64"/>
       <c r="U71" s="61"/>
       <c r="V71" s="62"/>
-      <c r="W71" s="54"/>
-      <c r="X71" s="55"/>
-      <c r="Y71" s="56"/>
-      <c r="Z71" s="54"/>
-      <c r="AA71" s="63"/>
+      <c r="W71" s="91"/>
+      <c r="X71" s="92"/>
+      <c r="Y71" s="93"/>
+      <c r="Z71" s="91"/>
+      <c r="AA71" s="94"/>
       <c r="AB71" s="57"/>
       <c r="AC71" s="58"/>
       <c r="AD71" s="59"/>
@@ -3905,22 +3938,22 @@
       <c r="I72" s="61"/>
       <c r="J72" s="62"/>
       <c r="K72" s="54"/>
-      <c r="L72" s="55"/>
-      <c r="M72" s="63"/>
+      <c r="L72" s="92"/>
+      <c r="M72" s="94"/>
       <c r="N72" s="64"/>
       <c r="O72" s="61"/>
       <c r="P72" s="62"/>
       <c r="Q72" s="54"/>
-      <c r="R72" s="55"/>
-      <c r="S72" s="63"/>
+      <c r="R72" s="92"/>
+      <c r="S72" s="94"/>
       <c r="T72" s="64"/>
       <c r="U72" s="61"/>
       <c r="V72" s="62"/>
-      <c r="W72" s="54"/>
-      <c r="X72" s="55"/>
-      <c r="Y72" s="56"/>
-      <c r="Z72" s="54"/>
-      <c r="AA72" s="63"/>
+      <c r="W72" s="91"/>
+      <c r="X72" s="92"/>
+      <c r="Y72" s="93"/>
+      <c r="Z72" s="91"/>
+      <c r="AA72" s="94"/>
       <c r="AB72" s="57"/>
       <c r="AC72" s="58"/>
       <c r="AD72" s="59"/>
@@ -3941,22 +3974,22 @@
       <c r="I73" s="61"/>
       <c r="J73" s="62"/>
       <c r="K73" s="54"/>
-      <c r="L73" s="55"/>
-      <c r="M73" s="63"/>
+      <c r="L73" s="92"/>
+      <c r="M73" s="94"/>
       <c r="N73" s="64"/>
       <c r="O73" s="61"/>
       <c r="P73" s="62"/>
       <c r="Q73" s="54"/>
-      <c r="R73" s="55"/>
-      <c r="S73" s="63"/>
+      <c r="R73" s="92"/>
+      <c r="S73" s="94"/>
       <c r="T73" s="64"/>
       <c r="U73" s="61"/>
       <c r="V73" s="62"/>
-      <c r="W73" s="54"/>
-      <c r="X73" s="55"/>
-      <c r="Y73" s="56"/>
-      <c r="Z73" s="54"/>
-      <c r="AA73" s="63"/>
+      <c r="W73" s="91"/>
+      <c r="X73" s="92"/>
+      <c r="Y73" s="93"/>
+      <c r="Z73" s="91"/>
+      <c r="AA73" s="94"/>
       <c r="AB73" s="57"/>
       <c r="AC73" s="58"/>
       <c r="AD73" s="72"/>
@@ -3977,22 +4010,22 @@
       <c r="I74" s="61"/>
       <c r="J74" s="62"/>
       <c r="K74" s="54"/>
-      <c r="L74" s="55"/>
-      <c r="M74" s="63"/>
+      <c r="L74" s="92"/>
+      <c r="M74" s="94"/>
       <c r="N74" s="64"/>
       <c r="O74" s="61"/>
       <c r="P74" s="62"/>
       <c r="Q74" s="54"/>
-      <c r="R74" s="55"/>
-      <c r="S74" s="63"/>
+      <c r="R74" s="92"/>
+      <c r="S74" s="94"/>
       <c r="T74" s="64"/>
       <c r="U74" s="61"/>
       <c r="V74" s="62"/>
-      <c r="W74" s="54"/>
-      <c r="X74" s="55"/>
-      <c r="Y74" s="56"/>
-      <c r="Z74" s="54"/>
-      <c r="AA74" s="63"/>
+      <c r="W74" s="91"/>
+      <c r="X74" s="92"/>
+      <c r="Y74" s="93"/>
+      <c r="Z74" s="91"/>
+      <c r="AA74" s="94"/>
       <c r="AB74" s="57"/>
       <c r="AC74" s="58"/>
       <c r="AD74" s="72"/>
@@ -4013,22 +4046,22 @@
       <c r="I75" s="61"/>
       <c r="J75" s="62"/>
       <c r="K75" s="54"/>
-      <c r="L75" s="55"/>
-      <c r="M75" s="63"/>
+      <c r="L75" s="92"/>
+      <c r="M75" s="94"/>
       <c r="N75" s="64"/>
       <c r="O75" s="61"/>
       <c r="P75" s="62"/>
       <c r="Q75" s="54"/>
-      <c r="R75" s="55"/>
-      <c r="S75" s="63"/>
+      <c r="R75" s="92"/>
+      <c r="S75" s="94"/>
       <c r="T75" s="64"/>
       <c r="U75" s="61"/>
       <c r="V75" s="62"/>
-      <c r="W75" s="54"/>
-      <c r="X75" s="55"/>
-      <c r="Y75" s="56"/>
-      <c r="Z75" s="54"/>
-      <c r="AA75" s="63"/>
+      <c r="W75" s="91"/>
+      <c r="X75" s="92"/>
+      <c r="Y75" s="93"/>
+      <c r="Z75" s="91"/>
+      <c r="AA75" s="94"/>
       <c r="AB75" s="57"/>
       <c r="AC75" s="58"/>
       <c r="AD75" s="72"/>
@@ -4049,22 +4082,22 @@
       <c r="I76" s="61"/>
       <c r="J76" s="62"/>
       <c r="K76" s="54"/>
-      <c r="L76" s="55"/>
-      <c r="M76" s="63"/>
+      <c r="L76" s="92"/>
+      <c r="M76" s="94"/>
       <c r="N76" s="64"/>
       <c r="O76" s="61"/>
       <c r="P76" s="62"/>
       <c r="Q76" s="54"/>
-      <c r="R76" s="55"/>
-      <c r="S76" s="63"/>
+      <c r="R76" s="92"/>
+      <c r="S76" s="94"/>
       <c r="T76" s="64"/>
       <c r="U76" s="61"/>
       <c r="V76" s="62"/>
-      <c r="W76" s="54"/>
-      <c r="X76" s="55"/>
-      <c r="Y76" s="56"/>
-      <c r="Z76" s="54"/>
-      <c r="AA76" s="63"/>
+      <c r="W76" s="91"/>
+      <c r="X76" s="92"/>
+      <c r="Y76" s="93"/>
+      <c r="Z76" s="91"/>
+      <c r="AA76" s="94"/>
       <c r="AB76" s="57"/>
       <c r="AC76" s="58"/>
       <c r="AD76" s="72"/>
@@ -4085,22 +4118,22 @@
       <c r="I77" s="61"/>
       <c r="J77" s="62"/>
       <c r="K77" s="54"/>
-      <c r="L77" s="55"/>
-      <c r="M77" s="63"/>
+      <c r="L77" s="92"/>
+      <c r="M77" s="94"/>
       <c r="N77" s="64"/>
       <c r="O77" s="61"/>
       <c r="P77" s="62"/>
       <c r="Q77" s="54"/>
-      <c r="R77" s="55"/>
-      <c r="S77" s="63"/>
+      <c r="R77" s="92"/>
+      <c r="S77" s="94"/>
       <c r="T77" s="64"/>
       <c r="U77" s="61"/>
       <c r="V77" s="62"/>
-      <c r="W77" s="54"/>
-      <c r="X77" s="55"/>
-      <c r="Y77" s="56"/>
-      <c r="Z77" s="54"/>
-      <c r="AA77" s="63"/>
+      <c r="W77" s="91"/>
+      <c r="X77" s="92"/>
+      <c r="Y77" s="93"/>
+      <c r="Z77" s="91"/>
+      <c r="AA77" s="94"/>
       <c r="AB77" s="57"/>
       <c r="AC77" s="58"/>
       <c r="AD77" s="72"/>
@@ -4121,22 +4154,22 @@
       <c r="I78" s="61"/>
       <c r="J78" s="62"/>
       <c r="K78" s="54"/>
-      <c r="L78" s="55"/>
-      <c r="M78" s="63"/>
+      <c r="L78" s="92"/>
+      <c r="M78" s="94"/>
       <c r="N78" s="64"/>
       <c r="O78" s="61"/>
       <c r="P78" s="62"/>
       <c r="Q78" s="54"/>
-      <c r="R78" s="55"/>
-      <c r="S78" s="63"/>
+      <c r="R78" s="92"/>
+      <c r="S78" s="94"/>
       <c r="T78" s="64"/>
       <c r="U78" s="61"/>
       <c r="V78" s="62"/>
-      <c r="W78" s="54"/>
-      <c r="X78" s="55"/>
-      <c r="Y78" s="56"/>
-      <c r="Z78" s="54"/>
-      <c r="AA78" s="63"/>
+      <c r="W78" s="91"/>
+      <c r="X78" s="92"/>
+      <c r="Y78" s="93"/>
+      <c r="Z78" s="91"/>
+      <c r="AA78" s="94"/>
       <c r="AB78" s="57"/>
       <c r="AC78" s="58"/>
       <c r="AD78" s="72"/>
@@ -4157,22 +4190,22 @@
       <c r="I79" s="61"/>
       <c r="J79" s="62"/>
       <c r="K79" s="54"/>
-      <c r="L79" s="55"/>
-      <c r="M79" s="63"/>
+      <c r="L79" s="92"/>
+      <c r="M79" s="94"/>
       <c r="N79" s="64"/>
       <c r="O79" s="61"/>
       <c r="P79" s="62"/>
       <c r="Q79" s="54"/>
-      <c r="R79" s="55"/>
-      <c r="S79" s="63"/>
+      <c r="R79" s="92"/>
+      <c r="S79" s="94"/>
       <c r="T79" s="64"/>
       <c r="U79" s="61"/>
       <c r="V79" s="62"/>
-      <c r="W79" s="54"/>
-      <c r="X79" s="55"/>
-      <c r="Y79" s="56"/>
-      <c r="Z79" s="54"/>
-      <c r="AA79" s="63"/>
+      <c r="W79" s="91"/>
+      <c r="X79" s="92"/>
+      <c r="Y79" s="93"/>
+      <c r="Z79" s="91"/>
+      <c r="AA79" s="94"/>
       <c r="AB79" s="57"/>
       <c r="AC79" s="58"/>
       <c r="AD79" s="72"/>
@@ -4193,22 +4226,22 @@
       <c r="I80" s="61"/>
       <c r="J80" s="62"/>
       <c r="K80" s="54"/>
-      <c r="L80" s="55"/>
-      <c r="M80" s="63"/>
+      <c r="L80" s="92"/>
+      <c r="M80" s="94"/>
       <c r="N80" s="64"/>
       <c r="O80" s="61"/>
       <c r="P80" s="62"/>
       <c r="Q80" s="54"/>
-      <c r="R80" s="55"/>
-      <c r="S80" s="63"/>
+      <c r="R80" s="92"/>
+      <c r="S80" s="94"/>
       <c r="T80" s="64"/>
       <c r="U80" s="61"/>
       <c r="V80" s="62"/>
-      <c r="W80" s="54"/>
-      <c r="X80" s="55"/>
-      <c r="Y80" s="56"/>
-      <c r="Z80" s="54"/>
-      <c r="AA80" s="63"/>
+      <c r="W80" s="91"/>
+      <c r="X80" s="92"/>
+      <c r="Y80" s="93"/>
+      <c r="Z80" s="91"/>
+      <c r="AA80" s="94"/>
       <c r="AB80" s="57"/>
       <c r="AC80" s="58"/>
       <c r="AD80" s="72"/>
@@ -4229,22 +4262,22 @@
       <c r="I81" s="61"/>
       <c r="J81" s="62"/>
       <c r="K81" s="54"/>
-      <c r="L81" s="55"/>
-      <c r="M81" s="63"/>
+      <c r="L81" s="92"/>
+      <c r="M81" s="94"/>
       <c r="N81" s="64"/>
       <c r="O81" s="61"/>
       <c r="P81" s="62"/>
       <c r="Q81" s="54"/>
-      <c r="R81" s="55"/>
-      <c r="S81" s="63"/>
+      <c r="R81" s="92"/>
+      <c r="S81" s="94"/>
       <c r="T81" s="64"/>
       <c r="U81" s="61"/>
       <c r="V81" s="62"/>
-      <c r="W81" s="54"/>
-      <c r="X81" s="55"/>
-      <c r="Y81" s="56"/>
-      <c r="Z81" s="54"/>
-      <c r="AA81" s="63"/>
+      <c r="W81" s="91"/>
+      <c r="X81" s="92"/>
+      <c r="Y81" s="93"/>
+      <c r="Z81" s="91"/>
+      <c r="AA81" s="94"/>
       <c r="AB81" s="57"/>
       <c r="AC81" s="58"/>
       <c r="AD81" s="72"/>
@@ -4265,22 +4298,22 @@
       <c r="I82" s="61"/>
       <c r="J82" s="62"/>
       <c r="K82" s="54"/>
-      <c r="L82" s="55"/>
-      <c r="M82" s="63"/>
+      <c r="L82" s="92"/>
+      <c r="M82" s="94"/>
       <c r="N82" s="64"/>
       <c r="O82" s="61"/>
       <c r="P82" s="62"/>
       <c r="Q82" s="54"/>
-      <c r="R82" s="55"/>
-      <c r="S82" s="63"/>
+      <c r="R82" s="92"/>
+      <c r="S82" s="94"/>
       <c r="T82" s="64"/>
       <c r="U82" s="61"/>
       <c r="V82" s="62"/>
-      <c r="W82" s="54"/>
-      <c r="X82" s="55"/>
-      <c r="Y82" s="56"/>
-      <c r="Z82" s="54"/>
-      <c r="AA82" s="63"/>
+      <c r="W82" s="91"/>
+      <c r="X82" s="92"/>
+      <c r="Y82" s="93"/>
+      <c r="Z82" s="91"/>
+      <c r="AA82" s="94"/>
       <c r="AB82" s="57"/>
       <c r="AC82" s="58"/>
       <c r="AD82" s="72"/>
@@ -4301,22 +4334,22 @@
       <c r="I83" s="61"/>
       <c r="J83" s="62"/>
       <c r="K83" s="54"/>
-      <c r="L83" s="55"/>
-      <c r="M83" s="63"/>
+      <c r="L83" s="92"/>
+      <c r="M83" s="94"/>
       <c r="N83" s="64"/>
       <c r="O83" s="61"/>
       <c r="P83" s="62"/>
       <c r="Q83" s="54"/>
-      <c r="R83" s="55"/>
-      <c r="S83" s="63"/>
+      <c r="R83" s="92"/>
+      <c r="S83" s="94"/>
       <c r="T83" s="64"/>
       <c r="U83" s="61"/>
       <c r="V83" s="62"/>
-      <c r="W83" s="54"/>
-      <c r="X83" s="55"/>
-      <c r="Y83" s="56"/>
-      <c r="Z83" s="54"/>
-      <c r="AA83" s="63"/>
+      <c r="W83" s="91"/>
+      <c r="X83" s="92"/>
+      <c r="Y83" s="93"/>
+      <c r="Z83" s="91"/>
+      <c r="AA83" s="94"/>
       <c r="AB83" s="57"/>
       <c r="AC83" s="58"/>
       <c r="AD83" s="72"/>
@@ -4337,22 +4370,22 @@
       <c r="I84" s="61"/>
       <c r="J84" s="62"/>
       <c r="K84" s="54"/>
-      <c r="L84" s="55"/>
-      <c r="M84" s="63"/>
+      <c r="L84" s="92"/>
+      <c r="M84" s="94"/>
       <c r="N84" s="64"/>
       <c r="O84" s="61"/>
       <c r="P84" s="62"/>
       <c r="Q84" s="54"/>
-      <c r="R84" s="55"/>
-      <c r="S84" s="63"/>
+      <c r="R84" s="92"/>
+      <c r="S84" s="94"/>
       <c r="T84" s="64"/>
       <c r="U84" s="61"/>
       <c r="V84" s="62"/>
-      <c r="W84" s="54"/>
-      <c r="X84" s="55"/>
-      <c r="Y84" s="56"/>
-      <c r="Z84" s="54"/>
-      <c r="AA84" s="63"/>
+      <c r="W84" s="91"/>
+      <c r="X84" s="92"/>
+      <c r="Y84" s="93"/>
+      <c r="Z84" s="91"/>
+      <c r="AA84" s="94"/>
       <c r="AB84" s="57"/>
       <c r="AC84" s="58"/>
       <c r="AD84" s="72"/>
@@ -4373,22 +4406,22 @@
       <c r="I85" s="61"/>
       <c r="J85" s="62"/>
       <c r="K85" s="54"/>
-      <c r="L85" s="55"/>
-      <c r="M85" s="63"/>
+      <c r="L85" s="92"/>
+      <c r="M85" s="94"/>
       <c r="N85" s="64"/>
       <c r="O85" s="61"/>
       <c r="P85" s="62"/>
       <c r="Q85" s="54"/>
-      <c r="R85" s="55"/>
-      <c r="S85" s="63"/>
+      <c r="R85" s="92"/>
+      <c r="S85" s="94"/>
       <c r="T85" s="64"/>
       <c r="U85" s="61"/>
       <c r="V85" s="62"/>
-      <c r="W85" s="54"/>
-      <c r="X85" s="55"/>
-      <c r="Y85" s="56"/>
-      <c r="Z85" s="54"/>
-      <c r="AA85" s="63"/>
+      <c r="W85" s="91"/>
+      <c r="X85" s="92"/>
+      <c r="Y85" s="93"/>
+      <c r="Z85" s="91"/>
+      <c r="AA85" s="94"/>
       <c r="AB85" s="57"/>
       <c r="AC85" s="58"/>
       <c r="AD85" s="72"/>
@@ -4409,22 +4442,22 @@
       <c r="I86" s="61"/>
       <c r="J86" s="62"/>
       <c r="K86" s="54"/>
-      <c r="L86" s="55"/>
-      <c r="M86" s="63"/>
+      <c r="L86" s="92"/>
+      <c r="M86" s="94"/>
       <c r="N86" s="64"/>
       <c r="O86" s="61"/>
       <c r="P86" s="62"/>
       <c r="Q86" s="54"/>
-      <c r="R86" s="55"/>
-      <c r="S86" s="63"/>
+      <c r="R86" s="92"/>
+      <c r="S86" s="94"/>
       <c r="T86" s="64"/>
       <c r="U86" s="61"/>
       <c r="V86" s="62"/>
-      <c r="W86" s="54"/>
-      <c r="X86" s="55"/>
-      <c r="Y86" s="56"/>
-      <c r="Z86" s="54"/>
-      <c r="AA86" s="63"/>
+      <c r="W86" s="91"/>
+      <c r="X86" s="92"/>
+      <c r="Y86" s="93"/>
+      <c r="Z86" s="91"/>
+      <c r="AA86" s="94"/>
       <c r="AB86" s="57"/>
       <c r="AC86" s="58"/>
       <c r="AD86" s="72"/>
@@ -4445,22 +4478,22 @@
       <c r="I87" s="61"/>
       <c r="J87" s="62"/>
       <c r="K87" s="54"/>
-      <c r="L87" s="55"/>
-      <c r="M87" s="63"/>
+      <c r="L87" s="92"/>
+      <c r="M87" s="94"/>
       <c r="N87" s="64"/>
       <c r="O87" s="61"/>
       <c r="P87" s="62"/>
       <c r="Q87" s="54"/>
-      <c r="R87" s="55"/>
-      <c r="S87" s="63"/>
+      <c r="R87" s="92"/>
+      <c r="S87" s="94"/>
       <c r="T87" s="64"/>
       <c r="U87" s="61"/>
       <c r="V87" s="62"/>
-      <c r="W87" s="54"/>
-      <c r="X87" s="55"/>
-      <c r="Y87" s="56"/>
-      <c r="Z87" s="54"/>
-      <c r="AA87" s="63"/>
+      <c r="W87" s="91"/>
+      <c r="X87" s="92"/>
+      <c r="Y87" s="93"/>
+      <c r="Z87" s="91"/>
+      <c r="AA87" s="94"/>
       <c r="AB87" s="57"/>
       <c r="AC87" s="58"/>
       <c r="AD87" s="72"/>
@@ -4481,22 +4514,22 @@
       <c r="I88" s="61"/>
       <c r="J88" s="62"/>
       <c r="K88" s="54"/>
-      <c r="L88" s="55"/>
-      <c r="M88" s="63"/>
+      <c r="L88" s="92"/>
+      <c r="M88" s="94"/>
       <c r="N88" s="64"/>
       <c r="O88" s="61"/>
       <c r="P88" s="62"/>
       <c r="Q88" s="54"/>
-      <c r="R88" s="55"/>
-      <c r="S88" s="63"/>
+      <c r="R88" s="92"/>
+      <c r="S88" s="94"/>
       <c r="T88" s="64"/>
       <c r="U88" s="61"/>
       <c r="V88" s="62"/>
-      <c r="W88" s="54"/>
-      <c r="X88" s="55"/>
-      <c r="Y88" s="56"/>
-      <c r="Z88" s="54"/>
-      <c r="AA88" s="63"/>
+      <c r="W88" s="91"/>
+      <c r="X88" s="92"/>
+      <c r="Y88" s="93"/>
+      <c r="Z88" s="91"/>
+      <c r="AA88" s="94"/>
       <c r="AB88" s="57"/>
       <c r="AC88" s="58"/>
       <c r="AD88" s="72"/>
@@ -4517,22 +4550,22 @@
       <c r="I89" s="61"/>
       <c r="J89" s="62"/>
       <c r="K89" s="54"/>
-      <c r="L89" s="55"/>
-      <c r="M89" s="63"/>
+      <c r="L89" s="92"/>
+      <c r="M89" s="94"/>
       <c r="N89" s="64"/>
       <c r="O89" s="61"/>
       <c r="P89" s="62"/>
       <c r="Q89" s="54"/>
-      <c r="R89" s="55"/>
-      <c r="S89" s="63"/>
+      <c r="R89" s="92"/>
+      <c r="S89" s="94"/>
       <c r="T89" s="64"/>
       <c r="U89" s="61"/>
       <c r="V89" s="62"/>
-      <c r="W89" s="54"/>
-      <c r="X89" s="55"/>
-      <c r="Y89" s="56"/>
-      <c r="Z89" s="54"/>
-      <c r="AA89" s="63"/>
+      <c r="W89" s="91"/>
+      <c r="X89" s="92"/>
+      <c r="Y89" s="93"/>
+      <c r="Z89" s="91"/>
+      <c r="AA89" s="94"/>
       <c r="AB89" s="57"/>
       <c r="AC89" s="58"/>
       <c r="AD89" s="72"/>
@@ -4553,22 +4586,22 @@
       <c r="I90" s="61"/>
       <c r="J90" s="62"/>
       <c r="K90" s="54"/>
-      <c r="L90" s="55"/>
-      <c r="M90" s="63"/>
+      <c r="L90" s="92"/>
+      <c r="M90" s="94"/>
       <c r="N90" s="64"/>
       <c r="O90" s="61"/>
       <c r="P90" s="62"/>
       <c r="Q90" s="54"/>
-      <c r="R90" s="55"/>
-      <c r="S90" s="63"/>
+      <c r="R90" s="92"/>
+      <c r="S90" s="94"/>
       <c r="T90" s="64"/>
       <c r="U90" s="61"/>
       <c r="V90" s="62"/>
-      <c r="W90" s="54"/>
-      <c r="X90" s="55"/>
-      <c r="Y90" s="56"/>
-      <c r="Z90" s="54"/>
-      <c r="AA90" s="63"/>
+      <c r="W90" s="91"/>
+      <c r="X90" s="92"/>
+      <c r="Y90" s="93"/>
+      <c r="Z90" s="91"/>
+      <c r="AA90" s="94"/>
       <c r="AB90" s="57"/>
       <c r="AC90" s="58"/>
       <c r="AD90" s="72"/>
@@ -4589,22 +4622,22 @@
       <c r="I91" s="61"/>
       <c r="J91" s="62"/>
       <c r="K91" s="54"/>
-      <c r="L91" s="55"/>
-      <c r="M91" s="63"/>
+      <c r="L91" s="92"/>
+      <c r="M91" s="94"/>
       <c r="N91" s="64"/>
       <c r="O91" s="61"/>
       <c r="P91" s="62"/>
       <c r="Q91" s="54"/>
-      <c r="R91" s="55"/>
-      <c r="S91" s="63"/>
+      <c r="R91" s="92"/>
+      <c r="S91" s="94"/>
       <c r="T91" s="64"/>
       <c r="U91" s="61"/>
       <c r="V91" s="62"/>
-      <c r="W91" s="54"/>
-      <c r="X91" s="55"/>
-      <c r="Y91" s="56"/>
-      <c r="Z91" s="54"/>
-      <c r="AA91" s="63"/>
+      <c r="W91" s="91"/>
+      <c r="X91" s="92"/>
+      <c r="Y91" s="93"/>
+      <c r="Z91" s="91"/>
+      <c r="AA91" s="94"/>
       <c r="AB91" s="57"/>
       <c r="AC91" s="58"/>
       <c r="AD91" s="72"/>
@@ -4625,22 +4658,22 @@
       <c r="I92" s="61"/>
       <c r="J92" s="62"/>
       <c r="K92" s="54"/>
-      <c r="L92" s="55"/>
-      <c r="M92" s="63"/>
+      <c r="L92" s="92"/>
+      <c r="M92" s="94"/>
       <c r="N92" s="64"/>
       <c r="O92" s="61"/>
       <c r="P92" s="62"/>
       <c r="Q92" s="54"/>
-      <c r="R92" s="55"/>
-      <c r="S92" s="63"/>
+      <c r="R92" s="92"/>
+      <c r="S92" s="94"/>
       <c r="T92" s="64"/>
       <c r="U92" s="61"/>
       <c r="V92" s="62"/>
-      <c r="W92" s="54"/>
-      <c r="X92" s="55"/>
-      <c r="Y92" s="56"/>
-      <c r="Z92" s="54"/>
-      <c r="AA92" s="63"/>
+      <c r="W92" s="91"/>
+      <c r="X92" s="92"/>
+      <c r="Y92" s="93"/>
+      <c r="Z92" s="91"/>
+      <c r="AA92" s="94"/>
       <c r="AB92" s="57"/>
       <c r="AC92" s="58"/>
       <c r="AD92" s="72"/>
@@ -4661,22 +4694,22 @@
       <c r="I93" s="61"/>
       <c r="J93" s="62"/>
       <c r="K93" s="54"/>
-      <c r="L93" s="55"/>
-      <c r="M93" s="63"/>
+      <c r="L93" s="92"/>
+      <c r="M93" s="94"/>
       <c r="N93" s="64"/>
       <c r="O93" s="61"/>
       <c r="P93" s="62"/>
       <c r="Q93" s="54"/>
-      <c r="R93" s="55"/>
-      <c r="S93" s="63"/>
+      <c r="R93" s="92"/>
+      <c r="S93" s="94"/>
       <c r="T93" s="64"/>
       <c r="U93" s="61"/>
       <c r="V93" s="62"/>
-      <c r="W93" s="54"/>
-      <c r="X93" s="55"/>
-      <c r="Y93" s="56"/>
-      <c r="Z93" s="54"/>
-      <c r="AA93" s="63"/>
+      <c r="W93" s="91"/>
+      <c r="X93" s="92"/>
+      <c r="Y93" s="93"/>
+      <c r="Z93" s="91"/>
+      <c r="AA93" s="94"/>
       <c r="AB93" s="57"/>
       <c r="AC93" s="58"/>
       <c r="AD93" s="72"/>
@@ -4697,22 +4730,22 @@
       <c r="I94" s="61"/>
       <c r="J94" s="62"/>
       <c r="K94" s="54"/>
-      <c r="L94" s="55"/>
-      <c r="M94" s="63"/>
+      <c r="L94" s="92"/>
+      <c r="M94" s="94"/>
       <c r="N94" s="64"/>
       <c r="O94" s="61"/>
       <c r="P94" s="62"/>
       <c r="Q94" s="54"/>
-      <c r="R94" s="55"/>
-      <c r="S94" s="63"/>
+      <c r="R94" s="92"/>
+      <c r="S94" s="94"/>
       <c r="T94" s="64"/>
       <c r="U94" s="61"/>
       <c r="V94" s="62"/>
-      <c r="W94" s="54"/>
-      <c r="X94" s="55"/>
-      <c r="Y94" s="56"/>
-      <c r="Z94" s="54"/>
-      <c r="AA94" s="63"/>
+      <c r="W94" s="91"/>
+      <c r="X94" s="92"/>
+      <c r="Y94" s="93"/>
+      <c r="Z94" s="91"/>
+      <c r="AA94" s="94"/>
       <c r="AB94" s="57"/>
       <c r="AC94" s="58"/>
       <c r="AD94" s="72"/>
@@ -4733,22 +4766,22 @@
       <c r="I95" s="61"/>
       <c r="J95" s="62"/>
       <c r="K95" s="54"/>
-      <c r="L95" s="55"/>
-      <c r="M95" s="63"/>
+      <c r="L95" s="92"/>
+      <c r="M95" s="94"/>
       <c r="N95" s="64"/>
       <c r="O95" s="61"/>
       <c r="P95" s="62"/>
       <c r="Q95" s="54"/>
-      <c r="R95" s="55"/>
-      <c r="S95" s="63"/>
+      <c r="R95" s="92"/>
+      <c r="S95" s="94"/>
       <c r="T95" s="64"/>
       <c r="U95" s="61"/>
       <c r="V95" s="62"/>
-      <c r="W95" s="54"/>
-      <c r="X95" s="55"/>
-      <c r="Y95" s="56"/>
-      <c r="Z95" s="54"/>
-      <c r="AA95" s="63"/>
+      <c r="W95" s="91"/>
+      <c r="X95" s="92"/>
+      <c r="Y95" s="93"/>
+      <c r="Z95" s="91"/>
+      <c r="AA95" s="94"/>
       <c r="AB95" s="57"/>
       <c r="AC95" s="58"/>
       <c r="AD95" s="72"/>
@@ -4769,22 +4802,22 @@
       <c r="I96" s="61"/>
       <c r="J96" s="62"/>
       <c r="K96" s="54"/>
-      <c r="L96" s="55"/>
-      <c r="M96" s="63"/>
+      <c r="L96" s="92"/>
+      <c r="M96" s="94"/>
       <c r="N96" s="64"/>
       <c r="O96" s="61"/>
       <c r="P96" s="62"/>
       <c r="Q96" s="54"/>
-      <c r="R96" s="55"/>
-      <c r="S96" s="63"/>
+      <c r="R96" s="92"/>
+      <c r="S96" s="94"/>
       <c r="T96" s="64"/>
       <c r="U96" s="61"/>
       <c r="V96" s="62"/>
-      <c r="W96" s="54"/>
-      <c r="X96" s="55"/>
-      <c r="Y96" s="56"/>
-      <c r="Z96" s="54"/>
-      <c r="AA96" s="63"/>
+      <c r="W96" s="91"/>
+      <c r="X96" s="92"/>
+      <c r="Y96" s="93"/>
+      <c r="Z96" s="91"/>
+      <c r="AA96" s="94"/>
       <c r="AB96" s="57"/>
       <c r="AC96" s="58"/>
       <c r="AD96" s="72"/>
@@ -4805,22 +4838,22 @@
       <c r="I97" s="61"/>
       <c r="J97" s="62"/>
       <c r="K97" s="54"/>
-      <c r="L97" s="55"/>
-      <c r="M97" s="63"/>
+      <c r="L97" s="92"/>
+      <c r="M97" s="94"/>
       <c r="N97" s="64"/>
       <c r="O97" s="61"/>
       <c r="P97" s="62"/>
       <c r="Q97" s="54"/>
-      <c r="R97" s="55"/>
-      <c r="S97" s="63"/>
+      <c r="R97" s="92"/>
+      <c r="S97" s="94"/>
       <c r="T97" s="64"/>
       <c r="U97" s="61"/>
       <c r="V97" s="62"/>
-      <c r="W97" s="54"/>
-      <c r="X97" s="55"/>
-      <c r="Y97" s="56"/>
-      <c r="Z97" s="54"/>
-      <c r="AA97" s="63"/>
+      <c r="W97" s="91"/>
+      <c r="X97" s="92"/>
+      <c r="Y97" s="93"/>
+      <c r="Z97" s="91"/>
+      <c r="AA97" s="94"/>
       <c r="AB97" s="57"/>
       <c r="AC97" s="58"/>
       <c r="AD97" s="72"/>
@@ -4841,22 +4874,22 @@
       <c r="I98" s="61"/>
       <c r="J98" s="62"/>
       <c r="K98" s="54"/>
-      <c r="L98" s="55"/>
-      <c r="M98" s="63"/>
+      <c r="L98" s="92"/>
+      <c r="M98" s="94"/>
       <c r="N98" s="64"/>
       <c r="O98" s="61"/>
       <c r="P98" s="62"/>
       <c r="Q98" s="54"/>
-      <c r="R98" s="55"/>
-      <c r="S98" s="63"/>
+      <c r="R98" s="92"/>
+      <c r="S98" s="94"/>
       <c r="T98" s="64"/>
       <c r="U98" s="61"/>
       <c r="V98" s="62"/>
-      <c r="W98" s="54"/>
-      <c r="X98" s="55"/>
-      <c r="Y98" s="56"/>
-      <c r="Z98" s="54"/>
-      <c r="AA98" s="63"/>
+      <c r="W98" s="91"/>
+      <c r="X98" s="92"/>
+      <c r="Y98" s="93"/>
+      <c r="Z98" s="91"/>
+      <c r="AA98" s="94"/>
       <c r="AB98" s="57"/>
       <c r="AC98" s="58"/>
       <c r="AD98" s="72"/>
@@ -4877,22 +4910,22 @@
       <c r="I99" s="61"/>
       <c r="J99" s="62"/>
       <c r="K99" s="54"/>
-      <c r="L99" s="55"/>
-      <c r="M99" s="63"/>
+      <c r="L99" s="92"/>
+      <c r="M99" s="94"/>
       <c r="N99" s="64"/>
       <c r="O99" s="61"/>
       <c r="P99" s="62"/>
       <c r="Q99" s="54"/>
-      <c r="R99" s="55"/>
-      <c r="S99" s="63"/>
+      <c r="R99" s="92"/>
+      <c r="S99" s="94"/>
       <c r="T99" s="64"/>
       <c r="U99" s="61"/>
       <c r="V99" s="62"/>
-      <c r="W99" s="54"/>
-      <c r="X99" s="55"/>
-      <c r="Y99" s="56"/>
-      <c r="Z99" s="54"/>
-      <c r="AA99" s="63"/>
+      <c r="W99" s="91"/>
+      <c r="X99" s="92"/>
+      <c r="Y99" s="93"/>
+      <c r="Z99" s="91"/>
+      <c r="AA99" s="94"/>
       <c r="AB99" s="57"/>
       <c r="AC99" s="58"/>
       <c r="AD99" s="72"/>
@@ -4913,22 +4946,22 @@
       <c r="I100" s="61"/>
       <c r="J100" s="62"/>
       <c r="K100" s="54"/>
-      <c r="L100" s="55"/>
-      <c r="M100" s="63"/>
+      <c r="L100" s="92"/>
+      <c r="M100" s="94"/>
       <c r="N100" s="64"/>
       <c r="O100" s="61"/>
       <c r="P100" s="62"/>
       <c r="Q100" s="54"/>
-      <c r="R100" s="55"/>
-      <c r="S100" s="63"/>
+      <c r="R100" s="92"/>
+      <c r="S100" s="94"/>
       <c r="T100" s="64"/>
       <c r="U100" s="61"/>
       <c r="V100" s="62"/>
-      <c r="W100" s="54"/>
-      <c r="X100" s="55"/>
-      <c r="Y100" s="56"/>
-      <c r="Z100" s="54"/>
-      <c r="AA100" s="63"/>
+      <c r="W100" s="91"/>
+      <c r="X100" s="92"/>
+      <c r="Y100" s="93"/>
+      <c r="Z100" s="91"/>
+      <c r="AA100" s="94"/>
       <c r="AB100" s="57"/>
       <c r="AC100" s="58"/>
       <c r="AD100" s="72"/>
@@ -4949,22 +4982,22 @@
       <c r="I101" s="61"/>
       <c r="J101" s="62"/>
       <c r="K101" s="54"/>
-      <c r="L101" s="55"/>
-      <c r="M101" s="63"/>
+      <c r="L101" s="92"/>
+      <c r="M101" s="94"/>
       <c r="N101" s="64"/>
       <c r="O101" s="61"/>
       <c r="P101" s="62"/>
       <c r="Q101" s="54"/>
-      <c r="R101" s="55"/>
-      <c r="S101" s="63"/>
+      <c r="R101" s="92"/>
+      <c r="S101" s="94"/>
       <c r="T101" s="64"/>
       <c r="U101" s="61"/>
       <c r="V101" s="62"/>
-      <c r="W101" s="54"/>
-      <c r="X101" s="55"/>
-      <c r="Y101" s="56"/>
-      <c r="Z101" s="54"/>
-      <c r="AA101" s="63"/>
+      <c r="W101" s="91"/>
+      <c r="X101" s="92"/>
+      <c r="Y101" s="93"/>
+      <c r="Z101" s="91"/>
+      <c r="AA101" s="94"/>
       <c r="AB101" s="57"/>
       <c r="AC101" s="58"/>
       <c r="AD101" s="72"/>
@@ -4985,22 +5018,22 @@
       <c r="I102" s="61"/>
       <c r="J102" s="62"/>
       <c r="K102" s="54"/>
-      <c r="L102" s="55"/>
-      <c r="M102" s="63"/>
+      <c r="L102" s="92"/>
+      <c r="M102" s="94"/>
       <c r="N102" s="64"/>
       <c r="O102" s="61"/>
       <c r="P102" s="62"/>
       <c r="Q102" s="54"/>
-      <c r="R102" s="55"/>
-      <c r="S102" s="63"/>
+      <c r="R102" s="92"/>
+      <c r="S102" s="94"/>
       <c r="T102" s="64"/>
       <c r="U102" s="61"/>
       <c r="V102" s="62"/>
-      <c r="W102" s="54"/>
-      <c r="X102" s="55"/>
-      <c r="Y102" s="56"/>
-      <c r="Z102" s="54"/>
-      <c r="AA102" s="63"/>
+      <c r="W102" s="91"/>
+      <c r="X102" s="92"/>
+      <c r="Y102" s="93"/>
+      <c r="Z102" s="91"/>
+      <c r="AA102" s="94"/>
       <c r="AB102" s="57"/>
       <c r="AC102" s="58"/>
       <c r="AD102" s="72"/>
@@ -5021,22 +5054,22 @@
       <c r="I103" s="61"/>
       <c r="J103" s="62"/>
       <c r="K103" s="54"/>
-      <c r="L103" s="55"/>
-      <c r="M103" s="63"/>
+      <c r="L103" s="92"/>
+      <c r="M103" s="94"/>
       <c r="N103" s="64"/>
       <c r="O103" s="61"/>
       <c r="P103" s="62"/>
       <c r="Q103" s="54"/>
-      <c r="R103" s="55"/>
-      <c r="S103" s="63"/>
+      <c r="R103" s="92"/>
+      <c r="S103" s="94"/>
       <c r="T103" s="64"/>
       <c r="U103" s="61"/>
       <c r="V103" s="62"/>
-      <c r="W103" s="54"/>
-      <c r="X103" s="55"/>
-      <c r="Y103" s="56"/>
-      <c r="Z103" s="54"/>
-      <c r="AA103" s="63"/>
+      <c r="W103" s="91"/>
+      <c r="X103" s="92"/>
+      <c r="Y103" s="93"/>
+      <c r="Z103" s="91"/>
+      <c r="AA103" s="94"/>
       <c r="AB103" s="57"/>
       <c r="AC103" s="58"/>
       <c r="AD103" s="72"/>
@@ -5057,22 +5090,22 @@
       <c r="I104" s="61"/>
       <c r="J104" s="62"/>
       <c r="K104" s="54"/>
-      <c r="L104" s="55"/>
-      <c r="M104" s="63"/>
+      <c r="L104" s="92"/>
+      <c r="M104" s="94"/>
       <c r="N104" s="64"/>
       <c r="O104" s="61"/>
       <c r="P104" s="62"/>
       <c r="Q104" s="54"/>
-      <c r="R104" s="55"/>
-      <c r="S104" s="63"/>
+      <c r="R104" s="92"/>
+      <c r="S104" s="94"/>
       <c r="T104" s="64"/>
       <c r="U104" s="61"/>
       <c r="V104" s="62"/>
-      <c r="W104" s="54"/>
-      <c r="X104" s="55"/>
-      <c r="Y104" s="56"/>
-      <c r="Z104" s="54"/>
-      <c r="AA104" s="63"/>
+      <c r="W104" s="91"/>
+      <c r="X104" s="92"/>
+      <c r="Y104" s="93"/>
+      <c r="Z104" s="91"/>
+      <c r="AA104" s="94"/>
       <c r="AB104" s="57"/>
       <c r="AC104" s="58"/>
       <c r="AD104" s="72"/>
@@ -5093,22 +5126,22 @@
       <c r="I105" s="61"/>
       <c r="J105" s="62"/>
       <c r="K105" s="54"/>
-      <c r="L105" s="55"/>
-      <c r="M105" s="63"/>
+      <c r="L105" s="92"/>
+      <c r="M105" s="94"/>
       <c r="N105" s="64"/>
       <c r="O105" s="61"/>
       <c r="P105" s="62"/>
       <c r="Q105" s="54"/>
-      <c r="R105" s="55"/>
-      <c r="S105" s="63"/>
+      <c r="R105" s="92"/>
+      <c r="S105" s="94"/>
       <c r="T105" s="64"/>
       <c r="U105" s="61"/>
       <c r="V105" s="62"/>
-      <c r="W105" s="54"/>
-      <c r="X105" s="55"/>
-      <c r="Y105" s="56"/>
-      <c r="Z105" s="54"/>
-      <c r="AA105" s="63"/>
+      <c r="W105" s="91"/>
+      <c r="X105" s="92"/>
+      <c r="Y105" s="93"/>
+      <c r="Z105" s="91"/>
+      <c r="AA105" s="94"/>
       <c r="AB105" s="57"/>
       <c r="AC105" s="58"/>
       <c r="AD105" s="72"/>
@@ -5129,22 +5162,22 @@
       <c r="I106" s="61"/>
       <c r="J106" s="62"/>
       <c r="K106" s="54"/>
-      <c r="L106" s="55"/>
-      <c r="M106" s="63"/>
+      <c r="L106" s="92"/>
+      <c r="M106" s="94"/>
       <c r="N106" s="64"/>
       <c r="O106" s="61"/>
       <c r="P106" s="62"/>
       <c r="Q106" s="54"/>
-      <c r="R106" s="55"/>
-      <c r="S106" s="63"/>
+      <c r="R106" s="92"/>
+      <c r="S106" s="94"/>
       <c r="T106" s="64"/>
       <c r="U106" s="61"/>
       <c r="V106" s="62"/>
-      <c r="W106" s="54"/>
-      <c r="X106" s="55"/>
-      <c r="Y106" s="56"/>
-      <c r="Z106" s="54"/>
-      <c r="AA106" s="63"/>
+      <c r="W106" s="91"/>
+      <c r="X106" s="92"/>
+      <c r="Y106" s="93"/>
+      <c r="Z106" s="91"/>
+      <c r="AA106" s="94"/>
       <c r="AB106" s="57"/>
       <c r="AC106" s="58"/>
       <c r="AD106" s="72"/>
@@ -5165,22 +5198,22 @@
       <c r="I107" s="61"/>
       <c r="J107" s="62"/>
       <c r="K107" s="54"/>
-      <c r="L107" s="55"/>
-      <c r="M107" s="63"/>
+      <c r="L107" s="92"/>
+      <c r="M107" s="94"/>
       <c r="N107" s="64"/>
       <c r="O107" s="61"/>
       <c r="P107" s="62"/>
       <c r="Q107" s="54"/>
-      <c r="R107" s="55"/>
-      <c r="S107" s="63"/>
+      <c r="R107" s="92"/>
+      <c r="S107" s="94"/>
       <c r="T107" s="64"/>
       <c r="U107" s="61"/>
       <c r="V107" s="62"/>
-      <c r="W107" s="54"/>
-      <c r="X107" s="55"/>
-      <c r="Y107" s="56"/>
-      <c r="Z107" s="54"/>
-      <c r="AA107" s="63"/>
+      <c r="W107" s="91"/>
+      <c r="X107" s="92"/>
+      <c r="Y107" s="93"/>
+      <c r="Z107" s="91"/>
+      <c r="AA107" s="94"/>
       <c r="AB107" s="57"/>
       <c r="AC107" s="58"/>
       <c r="AD107" s="72"/>
@@ -5201,22 +5234,22 @@
       <c r="I108" s="61"/>
       <c r="J108" s="62"/>
       <c r="K108" s="54"/>
-      <c r="L108" s="55"/>
-      <c r="M108" s="63"/>
+      <c r="L108" s="92"/>
+      <c r="M108" s="94"/>
       <c r="N108" s="64"/>
       <c r="O108" s="61"/>
       <c r="P108" s="62"/>
       <c r="Q108" s="54"/>
-      <c r="R108" s="55"/>
-      <c r="S108" s="63"/>
+      <c r="R108" s="92"/>
+      <c r="S108" s="94"/>
       <c r="T108" s="64"/>
       <c r="U108" s="61"/>
       <c r="V108" s="62"/>
-      <c r="W108" s="54"/>
-      <c r="X108" s="55"/>
-      <c r="Y108" s="56"/>
-      <c r="Z108" s="54"/>
-      <c r="AA108" s="63"/>
+      <c r="W108" s="91"/>
+      <c r="X108" s="92"/>
+      <c r="Y108" s="93"/>
+      <c r="Z108" s="91"/>
+      <c r="AA108" s="94"/>
       <c r="AB108" s="57"/>
       <c r="AC108" s="58"/>
       <c r="AD108" s="72"/>
@@ -5237,22 +5270,22 @@
       <c r="I109" s="61"/>
       <c r="J109" s="62"/>
       <c r="K109" s="54"/>
-      <c r="L109" s="55"/>
-      <c r="M109" s="63"/>
+      <c r="L109" s="92"/>
+      <c r="M109" s="94"/>
       <c r="N109" s="64"/>
       <c r="O109" s="61"/>
       <c r="P109" s="62"/>
       <c r="Q109" s="54"/>
-      <c r="R109" s="55"/>
-      <c r="S109" s="63"/>
+      <c r="R109" s="92"/>
+      <c r="S109" s="94"/>
       <c r="T109" s="64"/>
       <c r="U109" s="61"/>
       <c r="V109" s="62"/>
-      <c r="W109" s="54"/>
-      <c r="X109" s="55"/>
-      <c r="Y109" s="56"/>
-      <c r="Z109" s="54"/>
-      <c r="AA109" s="63"/>
+      <c r="W109" s="91"/>
+      <c r="X109" s="92"/>
+      <c r="Y109" s="93"/>
+      <c r="Z109" s="91"/>
+      <c r="AA109" s="94"/>
       <c r="AB109" s="57"/>
       <c r="AC109" s="58"/>
       <c r="AD109" s="72"/>
@@ -5273,22 +5306,22 @@
       <c r="I110" s="61"/>
       <c r="J110" s="62"/>
       <c r="K110" s="54"/>
-      <c r="L110" s="55"/>
-      <c r="M110" s="63"/>
+      <c r="L110" s="92"/>
+      <c r="M110" s="94"/>
       <c r="N110" s="64"/>
       <c r="O110" s="61"/>
       <c r="P110" s="62"/>
       <c r="Q110" s="54"/>
-      <c r="R110" s="55"/>
-      <c r="S110" s="63"/>
+      <c r="R110" s="92"/>
+      <c r="S110" s="94"/>
       <c r="T110" s="64"/>
       <c r="U110" s="61"/>
       <c r="V110" s="62"/>
-      <c r="W110" s="54"/>
-      <c r="X110" s="55"/>
-      <c r="Y110" s="56"/>
-      <c r="Z110" s="54"/>
-      <c r="AA110" s="63"/>
+      <c r="W110" s="91"/>
+      <c r="X110" s="92"/>
+      <c r="Y110" s="93"/>
+      <c r="Z110" s="91"/>
+      <c r="AA110" s="94"/>
       <c r="AB110" s="57"/>
       <c r="AC110" s="58"/>
       <c r="AD110" s="72"/>
@@ -5309,22 +5342,22 @@
       <c r="I111" s="61"/>
       <c r="J111" s="62"/>
       <c r="K111" s="54"/>
-      <c r="L111" s="55"/>
-      <c r="M111" s="63"/>
+      <c r="L111" s="92"/>
+      <c r="M111" s="94"/>
       <c r="N111" s="64"/>
       <c r="O111" s="61"/>
       <c r="P111" s="62"/>
       <c r="Q111" s="54"/>
-      <c r="R111" s="55"/>
-      <c r="S111" s="63"/>
+      <c r="R111" s="92"/>
+      <c r="S111" s="94"/>
       <c r="T111" s="64"/>
       <c r="U111" s="61"/>
       <c r="V111" s="62"/>
-      <c r="W111" s="54"/>
-      <c r="X111" s="55"/>
-      <c r="Y111" s="56"/>
-      <c r="Z111" s="54"/>
-      <c r="AA111" s="63"/>
+      <c r="W111" s="91"/>
+      <c r="X111" s="92"/>
+      <c r="Y111" s="93"/>
+      <c r="Z111" s="91"/>
+      <c r="AA111" s="94"/>
       <c r="AB111" s="57"/>
       <c r="AC111" s="58"/>
       <c r="AD111" s="72"/>
@@ -5345,22 +5378,22 @@
       <c r="I112" s="61"/>
       <c r="J112" s="62"/>
       <c r="K112" s="54"/>
-      <c r="L112" s="55"/>
-      <c r="M112" s="63"/>
+      <c r="L112" s="92"/>
+      <c r="M112" s="94"/>
       <c r="N112" s="64"/>
       <c r="O112" s="61"/>
       <c r="P112" s="62"/>
       <c r="Q112" s="54"/>
-      <c r="R112" s="55"/>
-      <c r="S112" s="63"/>
+      <c r="R112" s="92"/>
+      <c r="S112" s="94"/>
       <c r="T112" s="64"/>
       <c r="U112" s="61"/>
       <c r="V112" s="62"/>
-      <c r="W112" s="54"/>
-      <c r="X112" s="55"/>
-      <c r="Y112" s="56"/>
-      <c r="Z112" s="54"/>
-      <c r="AA112" s="63"/>
+      <c r="W112" s="91"/>
+      <c r="X112" s="92"/>
+      <c r="Y112" s="93"/>
+      <c r="Z112" s="91"/>
+      <c r="AA112" s="94"/>
       <c r="AB112" s="57"/>
       <c r="AC112" s="58"/>
       <c r="AD112" s="72"/>
@@ -5381,22 +5414,22 @@
       <c r="I113" s="61"/>
       <c r="J113" s="62"/>
       <c r="K113" s="54"/>
-      <c r="L113" s="55"/>
-      <c r="M113" s="63"/>
+      <c r="L113" s="92"/>
+      <c r="M113" s="94"/>
       <c r="N113" s="64"/>
       <c r="O113" s="61"/>
       <c r="P113" s="62"/>
       <c r="Q113" s="54"/>
-      <c r="R113" s="55"/>
-      <c r="S113" s="63"/>
+      <c r="R113" s="92"/>
+      <c r="S113" s="94"/>
       <c r="T113" s="64"/>
       <c r="U113" s="61"/>
       <c r="V113" s="62"/>
-      <c r="W113" s="54"/>
-      <c r="X113" s="55"/>
-      <c r="Y113" s="56"/>
-      <c r="Z113" s="54"/>
-      <c r="AA113" s="63"/>
+      <c r="W113" s="91"/>
+      <c r="X113" s="92"/>
+      <c r="Y113" s="93"/>
+      <c r="Z113" s="91"/>
+      <c r="AA113" s="94"/>
       <c r="AB113" s="57"/>
       <c r="AC113" s="58"/>
       <c r="AD113" s="72"/>
@@ -5417,22 +5450,22 @@
       <c r="I114" s="61"/>
       <c r="J114" s="62"/>
       <c r="K114" s="54"/>
-      <c r="L114" s="55"/>
-      <c r="M114" s="63"/>
+      <c r="L114" s="92"/>
+      <c r="M114" s="94"/>
       <c r="N114" s="64"/>
       <c r="O114" s="61"/>
       <c r="P114" s="62"/>
       <c r="Q114" s="54"/>
-      <c r="R114" s="55"/>
-      <c r="S114" s="63"/>
+      <c r="R114" s="92"/>
+      <c r="S114" s="94"/>
       <c r="T114" s="64"/>
       <c r="U114" s="61"/>
       <c r="V114" s="62"/>
-      <c r="W114" s="54"/>
-      <c r="X114" s="55"/>
-      <c r="Y114" s="56"/>
-      <c r="Z114" s="54"/>
-      <c r="AA114" s="63"/>
+      <c r="W114" s="91"/>
+      <c r="X114" s="92"/>
+      <c r="Y114" s="93"/>
+      <c r="Z114" s="91"/>
+      <c r="AA114" s="94"/>
       <c r="AB114" s="57"/>
       <c r="AC114" s="58"/>
       <c r="AD114" s="72"/>
@@ -5453,22 +5486,22 @@
       <c r="I115" s="61"/>
       <c r="J115" s="62"/>
       <c r="K115" s="54"/>
-      <c r="L115" s="55"/>
-      <c r="M115" s="63"/>
+      <c r="L115" s="92"/>
+      <c r="M115" s="94"/>
       <c r="N115" s="64"/>
       <c r="O115" s="61"/>
       <c r="P115" s="62"/>
       <c r="Q115" s="54"/>
-      <c r="R115" s="55"/>
-      <c r="S115" s="63"/>
+      <c r="R115" s="92"/>
+      <c r="S115" s="94"/>
       <c r="T115" s="64"/>
       <c r="U115" s="61"/>
       <c r="V115" s="62"/>
-      <c r="W115" s="54"/>
-      <c r="X115" s="55"/>
-      <c r="Y115" s="56"/>
-      <c r="Z115" s="54"/>
-      <c r="AA115" s="63"/>
+      <c r="W115" s="91"/>
+      <c r="X115" s="92"/>
+      <c r="Y115" s="93"/>
+      <c r="Z115" s="91"/>
+      <c r="AA115" s="94"/>
       <c r="AB115" s="57"/>
       <c r="AC115" s="58"/>
       <c r="AD115" s="72"/>
@@ -5489,22 +5522,22 @@
       <c r="I116" s="61"/>
       <c r="J116" s="62"/>
       <c r="K116" s="54"/>
-      <c r="L116" s="55"/>
-      <c r="M116" s="63"/>
+      <c r="L116" s="92"/>
+      <c r="M116" s="94"/>
       <c r="N116" s="64"/>
       <c r="O116" s="61"/>
       <c r="P116" s="62"/>
       <c r="Q116" s="54"/>
-      <c r="R116" s="55"/>
-      <c r="S116" s="63"/>
+      <c r="R116" s="92"/>
+      <c r="S116" s="94"/>
       <c r="T116" s="64"/>
       <c r="U116" s="61"/>
       <c r="V116" s="62"/>
-      <c r="W116" s="54"/>
-      <c r="X116" s="55"/>
-      <c r="Y116" s="56"/>
-      <c r="Z116" s="54"/>
-      <c r="AA116" s="63"/>
+      <c r="W116" s="91"/>
+      <c r="X116" s="92"/>
+      <c r="Y116" s="93"/>
+      <c r="Z116" s="91"/>
+      <c r="AA116" s="94"/>
       <c r="AB116" s="57"/>
       <c r="AC116" s="58"/>
       <c r="AD116" s="72"/>
@@ -5525,22 +5558,22 @@
       <c r="I117" s="61"/>
       <c r="J117" s="62"/>
       <c r="K117" s="54"/>
-      <c r="L117" s="55"/>
-      <c r="M117" s="63"/>
+      <c r="L117" s="92"/>
+      <c r="M117" s="94"/>
       <c r="N117" s="64"/>
       <c r="O117" s="61"/>
       <c r="P117" s="62"/>
       <c r="Q117" s="54"/>
-      <c r="R117" s="55"/>
-      <c r="S117" s="63"/>
+      <c r="R117" s="92"/>
+      <c r="S117" s="94"/>
       <c r="T117" s="64"/>
       <c r="U117" s="61"/>
       <c r="V117" s="62"/>
-      <c r="W117" s="54"/>
-      <c r="X117" s="55"/>
-      <c r="Y117" s="56"/>
-      <c r="Z117" s="54"/>
-      <c r="AA117" s="63"/>
+      <c r="W117" s="91"/>
+      <c r="X117" s="92"/>
+      <c r="Y117" s="93"/>
+      <c r="Z117" s="91"/>
+      <c r="AA117" s="94"/>
       <c r="AB117" s="57"/>
       <c r="AC117" s="58"/>
       <c r="AD117" s="72"/>
@@ -5561,22 +5594,22 @@
       <c r="I118" s="77"/>
       <c r="J118" s="78"/>
       <c r="K118" s="79"/>
-      <c r="L118" s="80"/>
-      <c r="M118" s="81"/>
+      <c r="L118" s="96"/>
+      <c r="M118" s="97"/>
       <c r="N118" s="76"/>
       <c r="O118" s="77"/>
       <c r="P118" s="78"/>
       <c r="Q118" s="79"/>
-      <c r="R118" s="80"/>
-      <c r="S118" s="81"/>
+      <c r="R118" s="96"/>
+      <c r="S118" s="97"/>
       <c r="T118" s="76"/>
       <c r="U118" s="77"/>
       <c r="V118" s="78"/>
-      <c r="W118" s="79"/>
-      <c r="X118" s="80"/>
-      <c r="Y118" s="82"/>
-      <c r="Z118" s="79"/>
-      <c r="AA118" s="81"/>
+      <c r="W118" s="95"/>
+      <c r="X118" s="96"/>
+      <c r="Y118" s="98"/>
+      <c r="Z118" s="95"/>
+      <c r="AA118" s="97"/>
       <c r="AB118" s="57"/>
       <c r="AC118" s="83"/>
       <c r="AD118" s="84"/>

</xml_diff>

<commit_message>
v1.0.27 - Add dark-mode visual optimization
</commit_message>
<xml_diff>
--- a/templates/ECR official Template.xlsx
+++ b/templates/ECR official Template.xlsx
@@ -741,7 +741,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="99">
+  <cellXfs count="88">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1040,39 +1040,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="15" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="15" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="15" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="15" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="15" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="15" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="15" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="15" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="15" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="15" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="15" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1994,22 +1961,22 @@
       <c r="I18" s="48"/>
       <c r="J18" s="49"/>
       <c r="K18" s="50"/>
-      <c r="L18" s="89"/>
-      <c r="M18" s="90"/>
+      <c r="L18" s="51"/>
+      <c r="M18" s="52"/>
       <c r="N18" s="53"/>
       <c r="O18" s="48"/>
       <c r="P18" s="49"/>
       <c r="Q18" s="50"/>
-      <c r="R18" s="89"/>
-      <c r="S18" s="90"/>
+      <c r="R18" s="51"/>
+      <c r="S18" s="52"/>
       <c r="T18" s="53"/>
       <c r="U18" s="48"/>
       <c r="V18" s="49"/>
-      <c r="W18" s="91"/>
-      <c r="X18" s="92"/>
-      <c r="Y18" s="93"/>
-      <c r="Z18" s="88"/>
-      <c r="AA18" s="90"/>
+      <c r="W18" s="54"/>
+      <c r="X18" s="55"/>
+      <c r="Y18" s="56"/>
+      <c r="Z18" s="50"/>
+      <c r="AA18" s="52"/>
       <c r="AB18" s="57"/>
       <c r="AC18" s="58"/>
       <c r="AD18" s="59"/>
@@ -2030,22 +1997,22 @@
       <c r="I19" s="61"/>
       <c r="J19" s="62"/>
       <c r="K19" s="54"/>
-      <c r="L19" s="92"/>
-      <c r="M19" s="94"/>
+      <c r="L19" s="55"/>
+      <c r="M19" s="63"/>
       <c r="N19" s="64"/>
       <c r="O19" s="61"/>
       <c r="P19" s="62"/>
       <c r="Q19" s="54"/>
-      <c r="R19" s="92"/>
-      <c r="S19" s="94"/>
+      <c r="R19" s="55"/>
+      <c r="S19" s="63"/>
       <c r="T19" s="64"/>
       <c r="U19" s="61"/>
       <c r="V19" s="62"/>
-      <c r="W19" s="91"/>
-      <c r="X19" s="92"/>
-      <c r="Y19" s="93"/>
-      <c r="Z19" s="91"/>
-      <c r="AA19" s="94"/>
+      <c r="W19" s="54"/>
+      <c r="X19" s="55"/>
+      <c r="Y19" s="56"/>
+      <c r="Z19" s="54"/>
+      <c r="AA19" s="63"/>
       <c r="AB19" s="57"/>
       <c r="AC19" s="58"/>
       <c r="AD19" s="59"/>
@@ -2066,22 +2033,22 @@
       <c r="I20" s="61"/>
       <c r="J20" s="62"/>
       <c r="K20" s="54"/>
-      <c r="L20" s="92"/>
-      <c r="M20" s="94"/>
+      <c r="L20" s="55"/>
+      <c r="M20" s="63"/>
       <c r="N20" s="64"/>
       <c r="O20" s="61"/>
       <c r="P20" s="62"/>
       <c r="Q20" s="54"/>
-      <c r="R20" s="92"/>
-      <c r="S20" s="94"/>
+      <c r="R20" s="55"/>
+      <c r="S20" s="63"/>
       <c r="T20" s="64"/>
       <c r="U20" s="61"/>
       <c r="V20" s="62"/>
-      <c r="W20" s="91"/>
-      <c r="X20" s="92"/>
-      <c r="Y20" s="93"/>
-      <c r="Z20" s="91"/>
-      <c r="AA20" s="94"/>
+      <c r="W20" s="54"/>
+      <c r="X20" s="55"/>
+      <c r="Y20" s="56"/>
+      <c r="Z20" s="54"/>
+      <c r="AA20" s="63"/>
       <c r="AB20" s="57"/>
       <c r="AC20" s="58"/>
       <c r="AD20" s="59"/>
@@ -2102,22 +2069,22 @@
       <c r="I21" s="61"/>
       <c r="J21" s="62"/>
       <c r="K21" s="54"/>
-      <c r="L21" s="92"/>
-      <c r="M21" s="94"/>
+      <c r="L21" s="55"/>
+      <c r="M21" s="63"/>
       <c r="N21" s="64"/>
       <c r="O21" s="61"/>
       <c r="P21" s="62"/>
       <c r="Q21" s="54"/>
-      <c r="R21" s="92"/>
-      <c r="S21" s="94"/>
+      <c r="R21" s="55"/>
+      <c r="S21" s="63"/>
       <c r="T21" s="64"/>
       <c r="U21" s="61"/>
       <c r="V21" s="62"/>
-      <c r="W21" s="91"/>
-      <c r="X21" s="92"/>
-      <c r="Y21" s="93"/>
-      <c r="Z21" s="91"/>
-      <c r="AA21" s="94"/>
+      <c r="W21" s="54"/>
+      <c r="X21" s="55"/>
+      <c r="Y21" s="56"/>
+      <c r="Z21" s="54"/>
+      <c r="AA21" s="63"/>
       <c r="AB21" s="57"/>
       <c r="AC21" s="58"/>
       <c r="AD21" s="59"/>
@@ -2138,22 +2105,22 @@
       <c r="I22" s="61"/>
       <c r="J22" s="62"/>
       <c r="K22" s="54"/>
-      <c r="L22" s="92"/>
-      <c r="M22" s="94"/>
+      <c r="L22" s="55"/>
+      <c r="M22" s="63"/>
       <c r="N22" s="64"/>
       <c r="O22" s="61"/>
       <c r="P22" s="62"/>
       <c r="Q22" s="54"/>
-      <c r="R22" s="92"/>
-      <c r="S22" s="94"/>
+      <c r="R22" s="55"/>
+      <c r="S22" s="63"/>
       <c r="T22" s="64"/>
       <c r="U22" s="61"/>
       <c r="V22" s="62"/>
-      <c r="W22" s="91"/>
-      <c r="X22" s="92"/>
-      <c r="Y22" s="93"/>
-      <c r="Z22" s="91"/>
-      <c r="AA22" s="94"/>
+      <c r="W22" s="54"/>
+      <c r="X22" s="55"/>
+      <c r="Y22" s="56"/>
+      <c r="Z22" s="54"/>
+      <c r="AA22" s="63"/>
       <c r="AB22" s="57"/>
       <c r="AC22" s="58"/>
       <c r="AD22" s="59"/>
@@ -2174,22 +2141,22 @@
       <c r="I23" s="61"/>
       <c r="J23" s="62"/>
       <c r="K23" s="54"/>
-      <c r="L23" s="92"/>
-      <c r="M23" s="94"/>
+      <c r="L23" s="55"/>
+      <c r="M23" s="63"/>
       <c r="N23" s="64"/>
       <c r="O23" s="61"/>
       <c r="P23" s="62"/>
       <c r="Q23" s="54"/>
-      <c r="R23" s="92"/>
-      <c r="S23" s="94"/>
+      <c r="R23" s="55"/>
+      <c r="S23" s="63"/>
       <c r="T23" s="64"/>
       <c r="U23" s="61"/>
       <c r="V23" s="62"/>
-      <c r="W23" s="91"/>
-      <c r="X23" s="92"/>
-      <c r="Y23" s="93"/>
-      <c r="Z23" s="91"/>
-      <c r="AA23" s="94"/>
+      <c r="W23" s="54"/>
+      <c r="X23" s="55"/>
+      <c r="Y23" s="56"/>
+      <c r="Z23" s="54"/>
+      <c r="AA23" s="63"/>
       <c r="AB23" s="57"/>
       <c r="AC23" s="58"/>
       <c r="AD23" s="59"/>
@@ -2210,22 +2177,22 @@
       <c r="I24" s="61"/>
       <c r="J24" s="62"/>
       <c r="K24" s="54"/>
-      <c r="L24" s="92"/>
-      <c r="M24" s="94"/>
+      <c r="L24" s="55"/>
+      <c r="M24" s="63"/>
       <c r="N24" s="64"/>
       <c r="O24" s="61"/>
       <c r="P24" s="62"/>
       <c r="Q24" s="54"/>
-      <c r="R24" s="92"/>
-      <c r="S24" s="94"/>
+      <c r="R24" s="55"/>
+      <c r="S24" s="63"/>
       <c r="T24" s="64"/>
       <c r="U24" s="61"/>
       <c r="V24" s="62"/>
-      <c r="W24" s="91"/>
-      <c r="X24" s="92"/>
-      <c r="Y24" s="93"/>
-      <c r="Z24" s="91"/>
-      <c r="AA24" s="94"/>
+      <c r="W24" s="54"/>
+      <c r="X24" s="55"/>
+      <c r="Y24" s="56"/>
+      <c r="Z24" s="54"/>
+      <c r="AA24" s="63"/>
       <c r="AB24" s="57"/>
       <c r="AC24" s="58"/>
       <c r="AD24" s="59"/>
@@ -2246,22 +2213,22 @@
       <c r="I25" s="61"/>
       <c r="J25" s="62"/>
       <c r="K25" s="54"/>
-      <c r="L25" s="92"/>
-      <c r="M25" s="94"/>
+      <c r="L25" s="55"/>
+      <c r="M25" s="63"/>
       <c r="N25" s="64"/>
       <c r="O25" s="61"/>
       <c r="P25" s="62"/>
       <c r="Q25" s="54"/>
-      <c r="R25" s="92"/>
-      <c r="S25" s="94"/>
+      <c r="R25" s="55"/>
+      <c r="S25" s="63"/>
       <c r="T25" s="64"/>
       <c r="U25" s="61"/>
       <c r="V25" s="62"/>
-      <c r="W25" s="91"/>
-      <c r="X25" s="92"/>
-      <c r="Y25" s="93"/>
-      <c r="Z25" s="91"/>
-      <c r="AA25" s="94"/>
+      <c r="W25" s="54"/>
+      <c r="X25" s="55"/>
+      <c r="Y25" s="56"/>
+      <c r="Z25" s="54"/>
+      <c r="AA25" s="63"/>
       <c r="AB25" s="57"/>
       <c r="AC25" s="58"/>
       <c r="AD25" s="59"/>
@@ -2282,22 +2249,22 @@
       <c r="I26" s="61"/>
       <c r="J26" s="62"/>
       <c r="K26" s="54"/>
-      <c r="L26" s="92"/>
-      <c r="M26" s="94"/>
+      <c r="L26" s="55"/>
+      <c r="M26" s="63"/>
       <c r="N26" s="64"/>
       <c r="O26" s="61"/>
       <c r="P26" s="62"/>
       <c r="Q26" s="54"/>
-      <c r="R26" s="92"/>
-      <c r="S26" s="94"/>
+      <c r="R26" s="55"/>
+      <c r="S26" s="63"/>
       <c r="T26" s="64"/>
       <c r="U26" s="61"/>
       <c r="V26" s="62"/>
-      <c r="W26" s="91"/>
-      <c r="X26" s="92"/>
-      <c r="Y26" s="93"/>
-      <c r="Z26" s="91"/>
-      <c r="AA26" s="94"/>
+      <c r="W26" s="54"/>
+      <c r="X26" s="55"/>
+      <c r="Y26" s="56"/>
+      <c r="Z26" s="54"/>
+      <c r="AA26" s="63"/>
       <c r="AB26" s="57"/>
       <c r="AC26" s="58"/>
       <c r="AD26" s="59"/>
@@ -2318,22 +2285,22 @@
       <c r="I27" s="61"/>
       <c r="J27" s="62"/>
       <c r="K27" s="54"/>
-      <c r="L27" s="92"/>
-      <c r="M27" s="94"/>
+      <c r="L27" s="55"/>
+      <c r="M27" s="63"/>
       <c r="N27" s="64"/>
       <c r="O27" s="61"/>
       <c r="P27" s="62"/>
       <c r="Q27" s="54"/>
-      <c r="R27" s="92"/>
-      <c r="S27" s="94"/>
+      <c r="R27" s="55"/>
+      <c r="S27" s="63"/>
       <c r="T27" s="64"/>
       <c r="U27" s="61"/>
       <c r="V27" s="62"/>
-      <c r="W27" s="91"/>
-      <c r="X27" s="92"/>
-      <c r="Y27" s="93"/>
-      <c r="Z27" s="91"/>
-      <c r="AA27" s="94"/>
+      <c r="W27" s="54"/>
+      <c r="X27" s="55"/>
+      <c r="Y27" s="56"/>
+      <c r="Z27" s="54"/>
+      <c r="AA27" s="63"/>
       <c r="AB27" s="57"/>
       <c r="AC27" s="58"/>
       <c r="AD27" s="59"/>
@@ -2354,22 +2321,22 @@
       <c r="I28" s="61"/>
       <c r="J28" s="62"/>
       <c r="K28" s="54"/>
-      <c r="L28" s="92"/>
-      <c r="M28" s="94"/>
+      <c r="L28" s="55"/>
+      <c r="M28" s="63"/>
       <c r="N28" s="64"/>
       <c r="O28" s="61"/>
       <c r="P28" s="62"/>
       <c r="Q28" s="54"/>
-      <c r="R28" s="92"/>
-      <c r="S28" s="94"/>
+      <c r="R28" s="55"/>
+      <c r="S28" s="63"/>
       <c r="T28" s="64"/>
       <c r="U28" s="61"/>
       <c r="V28" s="62"/>
-      <c r="W28" s="91"/>
-      <c r="X28" s="92"/>
-      <c r="Y28" s="93"/>
-      <c r="Z28" s="91"/>
-      <c r="AA28" s="94"/>
+      <c r="W28" s="54"/>
+      <c r="X28" s="55"/>
+      <c r="Y28" s="56"/>
+      <c r="Z28" s="54"/>
+      <c r="AA28" s="63"/>
       <c r="AB28" s="57"/>
       <c r="AC28" s="58"/>
       <c r="AD28" s="59"/>
@@ -2390,22 +2357,22 @@
       <c r="I29" s="61"/>
       <c r="J29" s="62"/>
       <c r="K29" s="54"/>
-      <c r="L29" s="92"/>
-      <c r="M29" s="94"/>
+      <c r="L29" s="55"/>
+      <c r="M29" s="63"/>
       <c r="N29" s="64"/>
       <c r="O29" s="61"/>
       <c r="P29" s="62"/>
       <c r="Q29" s="54"/>
-      <c r="R29" s="92"/>
-      <c r="S29" s="94"/>
+      <c r="R29" s="55"/>
+      <c r="S29" s="63"/>
       <c r="T29" s="64"/>
       <c r="U29" s="61"/>
       <c r="V29" s="62"/>
-      <c r="W29" s="91"/>
-      <c r="X29" s="92"/>
-      <c r="Y29" s="93"/>
-      <c r="Z29" s="91"/>
-      <c r="AA29" s="94"/>
+      <c r="W29" s="54"/>
+      <c r="X29" s="55"/>
+      <c r="Y29" s="56"/>
+      <c r="Z29" s="54"/>
+      <c r="AA29" s="63"/>
       <c r="AB29" s="57"/>
       <c r="AC29" s="58"/>
       <c r="AD29" s="59"/>
@@ -2426,22 +2393,22 @@
       <c r="I30" s="61"/>
       <c r="J30" s="62"/>
       <c r="K30" s="54"/>
-      <c r="L30" s="92"/>
-      <c r="M30" s="94"/>
+      <c r="L30" s="55"/>
+      <c r="M30" s="63"/>
       <c r="N30" s="64"/>
       <c r="O30" s="61"/>
       <c r="P30" s="62"/>
       <c r="Q30" s="54"/>
-      <c r="R30" s="92"/>
-      <c r="S30" s="94"/>
+      <c r="R30" s="55"/>
+      <c r="S30" s="63"/>
       <c r="T30" s="64"/>
       <c r="U30" s="61"/>
       <c r="V30" s="62"/>
-      <c r="W30" s="91"/>
-      <c r="X30" s="92"/>
-      <c r="Y30" s="93"/>
-      <c r="Z30" s="91"/>
-      <c r="AA30" s="94"/>
+      <c r="W30" s="54"/>
+      <c r="X30" s="55"/>
+      <c r="Y30" s="56"/>
+      <c r="Z30" s="54"/>
+      <c r="AA30" s="63"/>
       <c r="AB30" s="57"/>
       <c r="AC30" s="58"/>
       <c r="AD30" s="59"/>
@@ -2462,22 +2429,22 @@
       <c r="I31" s="61"/>
       <c r="J31" s="62"/>
       <c r="K31" s="54"/>
-      <c r="L31" s="92"/>
-      <c r="M31" s="94"/>
+      <c r="L31" s="55"/>
+      <c r="M31" s="63"/>
       <c r="N31" s="64"/>
       <c r="O31" s="61"/>
       <c r="P31" s="62"/>
       <c r="Q31" s="54"/>
-      <c r="R31" s="92"/>
-      <c r="S31" s="94"/>
+      <c r="R31" s="55"/>
+      <c r="S31" s="63"/>
       <c r="T31" s="64"/>
       <c r="U31" s="61"/>
       <c r="V31" s="62"/>
-      <c r="W31" s="91"/>
-      <c r="X31" s="92"/>
-      <c r="Y31" s="93"/>
-      <c r="Z31" s="91"/>
-      <c r="AA31" s="94"/>
+      <c r="W31" s="54"/>
+      <c r="X31" s="55"/>
+      <c r="Y31" s="56"/>
+      <c r="Z31" s="54"/>
+      <c r="AA31" s="63"/>
       <c r="AB31" s="57"/>
       <c r="AC31" s="58"/>
       <c r="AD31" s="59"/>
@@ -2498,22 +2465,22 @@
       <c r="I32" s="61"/>
       <c r="J32" s="62"/>
       <c r="K32" s="54"/>
-      <c r="L32" s="92"/>
-      <c r="M32" s="94"/>
+      <c r="L32" s="55"/>
+      <c r="M32" s="63"/>
       <c r="N32" s="64"/>
       <c r="O32" s="61"/>
       <c r="P32" s="62"/>
       <c r="Q32" s="54"/>
-      <c r="R32" s="92"/>
-      <c r="S32" s="94"/>
+      <c r="R32" s="55"/>
+      <c r="S32" s="63"/>
       <c r="T32" s="64"/>
       <c r="U32" s="61"/>
       <c r="V32" s="62"/>
-      <c r="W32" s="91"/>
-      <c r="X32" s="92"/>
-      <c r="Y32" s="93"/>
-      <c r="Z32" s="91"/>
-      <c r="AA32" s="94"/>
+      <c r="W32" s="54"/>
+      <c r="X32" s="55"/>
+      <c r="Y32" s="56"/>
+      <c r="Z32" s="54"/>
+      <c r="AA32" s="63"/>
       <c r="AB32" s="57"/>
       <c r="AC32" s="58"/>
       <c r="AD32" s="59"/>
@@ -2534,22 +2501,22 @@
       <c r="I33" s="61"/>
       <c r="J33" s="62"/>
       <c r="K33" s="54"/>
-      <c r="L33" s="92"/>
-      <c r="M33" s="94"/>
+      <c r="L33" s="55"/>
+      <c r="M33" s="63"/>
       <c r="N33" s="64"/>
       <c r="O33" s="61"/>
       <c r="P33" s="62"/>
       <c r="Q33" s="54"/>
-      <c r="R33" s="92"/>
-      <c r="S33" s="94"/>
+      <c r="R33" s="55"/>
+      <c r="S33" s="63"/>
       <c r="T33" s="64"/>
       <c r="U33" s="61"/>
       <c r="V33" s="62"/>
-      <c r="W33" s="91"/>
-      <c r="X33" s="92"/>
-      <c r="Y33" s="93"/>
-      <c r="Z33" s="91"/>
-      <c r="AA33" s="94"/>
+      <c r="W33" s="54"/>
+      <c r="X33" s="55"/>
+      <c r="Y33" s="56"/>
+      <c r="Z33" s="54"/>
+      <c r="AA33" s="63"/>
       <c r="AB33" s="57"/>
       <c r="AC33" s="58"/>
       <c r="AD33" s="59"/>
@@ -2570,22 +2537,22 @@
       <c r="I34" s="61"/>
       <c r="J34" s="62"/>
       <c r="K34" s="54"/>
-      <c r="L34" s="92"/>
-      <c r="M34" s="94"/>
+      <c r="L34" s="55"/>
+      <c r="M34" s="63"/>
       <c r="N34" s="64"/>
       <c r="O34" s="61"/>
       <c r="P34" s="62"/>
       <c r="Q34" s="54"/>
-      <c r="R34" s="92"/>
-      <c r="S34" s="94"/>
+      <c r="R34" s="55"/>
+      <c r="S34" s="63"/>
       <c r="T34" s="64"/>
       <c r="U34" s="61"/>
       <c r="V34" s="62"/>
-      <c r="W34" s="91"/>
-      <c r="X34" s="92"/>
-      <c r="Y34" s="93"/>
-      <c r="Z34" s="91"/>
-      <c r="AA34" s="94"/>
+      <c r="W34" s="54"/>
+      <c r="X34" s="55"/>
+      <c r="Y34" s="56"/>
+      <c r="Z34" s="54"/>
+      <c r="AA34" s="63"/>
       <c r="AB34" s="57"/>
       <c r="AC34" s="58"/>
       <c r="AD34" s="59"/>
@@ -2606,22 +2573,22 @@
       <c r="I35" s="61"/>
       <c r="J35" s="62"/>
       <c r="K35" s="54"/>
-      <c r="L35" s="92"/>
-      <c r="M35" s="94"/>
+      <c r="L35" s="55"/>
+      <c r="M35" s="63"/>
       <c r="N35" s="64"/>
       <c r="O35" s="61"/>
       <c r="P35" s="62"/>
       <c r="Q35" s="54"/>
-      <c r="R35" s="92"/>
-      <c r="S35" s="94"/>
+      <c r="R35" s="55"/>
+      <c r="S35" s="63"/>
       <c r="T35" s="64"/>
       <c r="U35" s="61"/>
       <c r="V35" s="62"/>
-      <c r="W35" s="91"/>
-      <c r="X35" s="92"/>
-      <c r="Y35" s="93"/>
-      <c r="Z35" s="91"/>
-      <c r="AA35" s="94"/>
+      <c r="W35" s="54"/>
+      <c r="X35" s="55"/>
+      <c r="Y35" s="56"/>
+      <c r="Z35" s="54"/>
+      <c r="AA35" s="63"/>
       <c r="AB35" s="57"/>
       <c r="AC35" s="58"/>
       <c r="AD35" s="59"/>
@@ -2642,22 +2609,22 @@
       <c r="I36" s="61"/>
       <c r="J36" s="62"/>
       <c r="K36" s="54"/>
-      <c r="L36" s="92"/>
-      <c r="M36" s="94"/>
+      <c r="L36" s="55"/>
+      <c r="M36" s="63"/>
       <c r="N36" s="64"/>
       <c r="O36" s="61"/>
       <c r="P36" s="62"/>
       <c r="Q36" s="54"/>
-      <c r="R36" s="92"/>
-      <c r="S36" s="94"/>
+      <c r="R36" s="55"/>
+      <c r="S36" s="63"/>
       <c r="T36" s="64"/>
       <c r="U36" s="61"/>
       <c r="V36" s="62"/>
-      <c r="W36" s="91"/>
-      <c r="X36" s="92"/>
-      <c r="Y36" s="93"/>
-      <c r="Z36" s="91"/>
-      <c r="AA36" s="94"/>
+      <c r="W36" s="54"/>
+      <c r="X36" s="55"/>
+      <c r="Y36" s="56"/>
+      <c r="Z36" s="54"/>
+      <c r="AA36" s="63"/>
       <c r="AB36" s="57"/>
       <c r="AC36" s="58"/>
       <c r="AD36" s="59"/>
@@ -2678,22 +2645,22 @@
       <c r="I37" s="61"/>
       <c r="J37" s="62"/>
       <c r="K37" s="54"/>
-      <c r="L37" s="92"/>
-      <c r="M37" s="94"/>
+      <c r="L37" s="55"/>
+      <c r="M37" s="63"/>
       <c r="N37" s="64"/>
       <c r="O37" s="61"/>
       <c r="P37" s="62"/>
       <c r="Q37" s="54"/>
-      <c r="R37" s="92"/>
-      <c r="S37" s="94"/>
+      <c r="R37" s="55"/>
+      <c r="S37" s="63"/>
       <c r="T37" s="64"/>
       <c r="U37" s="61"/>
       <c r="V37" s="62"/>
-      <c r="W37" s="91"/>
-      <c r="X37" s="92"/>
-      <c r="Y37" s="93"/>
-      <c r="Z37" s="91"/>
-      <c r="AA37" s="94"/>
+      <c r="W37" s="54"/>
+      <c r="X37" s="55"/>
+      <c r="Y37" s="56"/>
+      <c r="Z37" s="54"/>
+      <c r="AA37" s="63"/>
       <c r="AB37" s="57"/>
       <c r="AC37" s="58"/>
       <c r="AD37" s="59"/>
@@ -2714,22 +2681,22 @@
       <c r="I38" s="61"/>
       <c r="J38" s="62"/>
       <c r="K38" s="54"/>
-      <c r="L38" s="92"/>
-      <c r="M38" s="94"/>
+      <c r="L38" s="55"/>
+      <c r="M38" s="63"/>
       <c r="N38" s="64"/>
       <c r="O38" s="61"/>
       <c r="P38" s="62"/>
       <c r="Q38" s="54"/>
-      <c r="R38" s="92"/>
-      <c r="S38" s="94"/>
+      <c r="R38" s="55"/>
+      <c r="S38" s="63"/>
       <c r="T38" s="64"/>
       <c r="U38" s="61"/>
       <c r="V38" s="62"/>
-      <c r="W38" s="91"/>
-      <c r="X38" s="92"/>
-      <c r="Y38" s="93"/>
-      <c r="Z38" s="91"/>
-      <c r="AA38" s="94"/>
+      <c r="W38" s="54"/>
+      <c r="X38" s="55"/>
+      <c r="Y38" s="56"/>
+      <c r="Z38" s="54"/>
+      <c r="AA38" s="63"/>
       <c r="AB38" s="57"/>
       <c r="AC38" s="58"/>
       <c r="AD38" s="59"/>
@@ -2750,22 +2717,22 @@
       <c r="I39" s="61"/>
       <c r="J39" s="62"/>
       <c r="K39" s="54"/>
-      <c r="L39" s="92"/>
-      <c r="M39" s="94"/>
+      <c r="L39" s="55"/>
+      <c r="M39" s="63"/>
       <c r="N39" s="64"/>
       <c r="O39" s="61"/>
       <c r="P39" s="62"/>
       <c r="Q39" s="54"/>
-      <c r="R39" s="92"/>
-      <c r="S39" s="94"/>
+      <c r="R39" s="55"/>
+      <c r="S39" s="63"/>
       <c r="T39" s="64"/>
       <c r="U39" s="61"/>
       <c r="V39" s="62"/>
-      <c r="W39" s="91"/>
-      <c r="X39" s="92"/>
-      <c r="Y39" s="93"/>
-      <c r="Z39" s="91"/>
-      <c r="AA39" s="94"/>
+      <c r="W39" s="54"/>
+      <c r="X39" s="55"/>
+      <c r="Y39" s="56"/>
+      <c r="Z39" s="54"/>
+      <c r="AA39" s="63"/>
       <c r="AB39" s="57"/>
       <c r="AC39" s="58"/>
       <c r="AD39" s="59"/>
@@ -2786,22 +2753,22 @@
       <c r="I40" s="61"/>
       <c r="J40" s="62"/>
       <c r="K40" s="54"/>
-      <c r="L40" s="92"/>
-      <c r="M40" s="94"/>
+      <c r="L40" s="55"/>
+      <c r="M40" s="63"/>
       <c r="N40" s="64"/>
       <c r="O40" s="61"/>
       <c r="P40" s="62"/>
       <c r="Q40" s="54"/>
-      <c r="R40" s="92"/>
-      <c r="S40" s="94"/>
+      <c r="R40" s="55"/>
+      <c r="S40" s="63"/>
       <c r="T40" s="64"/>
       <c r="U40" s="61"/>
       <c r="V40" s="62"/>
-      <c r="W40" s="91"/>
-      <c r="X40" s="92"/>
-      <c r="Y40" s="93"/>
-      <c r="Z40" s="91"/>
-      <c r="AA40" s="94"/>
+      <c r="W40" s="54"/>
+      <c r="X40" s="55"/>
+      <c r="Y40" s="56"/>
+      <c r="Z40" s="54"/>
+      <c r="AA40" s="63"/>
       <c r="AB40" s="57"/>
       <c r="AC40" s="58"/>
       <c r="AD40" s="59"/>
@@ -2822,22 +2789,22 @@
       <c r="I41" s="61"/>
       <c r="J41" s="62"/>
       <c r="K41" s="54"/>
-      <c r="L41" s="92"/>
-      <c r="M41" s="94"/>
+      <c r="L41" s="55"/>
+      <c r="M41" s="63"/>
       <c r="N41" s="64"/>
       <c r="O41" s="61"/>
       <c r="P41" s="62"/>
       <c r="Q41" s="54"/>
-      <c r="R41" s="92"/>
-      <c r="S41" s="94"/>
+      <c r="R41" s="55"/>
+      <c r="S41" s="63"/>
       <c r="T41" s="64"/>
       <c r="U41" s="61"/>
       <c r="V41" s="62"/>
-      <c r="W41" s="91"/>
-      <c r="X41" s="92"/>
-      <c r="Y41" s="93"/>
-      <c r="Z41" s="91"/>
-      <c r="AA41" s="94"/>
+      <c r="W41" s="54"/>
+      <c r="X41" s="55"/>
+      <c r="Y41" s="56"/>
+      <c r="Z41" s="54"/>
+      <c r="AA41" s="63"/>
       <c r="AB41" s="57"/>
       <c r="AC41" s="58"/>
       <c r="AD41" s="59"/>
@@ -2858,22 +2825,22 @@
       <c r="I42" s="61"/>
       <c r="J42" s="62"/>
       <c r="K42" s="54"/>
-      <c r="L42" s="92"/>
-      <c r="M42" s="94"/>
+      <c r="L42" s="55"/>
+      <c r="M42" s="63"/>
       <c r="N42" s="64"/>
       <c r="O42" s="61"/>
       <c r="P42" s="62"/>
       <c r="Q42" s="54"/>
-      <c r="R42" s="92"/>
-      <c r="S42" s="94"/>
+      <c r="R42" s="55"/>
+      <c r="S42" s="63"/>
       <c r="T42" s="64"/>
       <c r="U42" s="61"/>
       <c r="V42" s="62"/>
-      <c r="W42" s="91"/>
-      <c r="X42" s="92"/>
-      <c r="Y42" s="93"/>
-      <c r="Z42" s="91"/>
-      <c r="AA42" s="94"/>
+      <c r="W42" s="54"/>
+      <c r="X42" s="55"/>
+      <c r="Y42" s="56"/>
+      <c r="Z42" s="54"/>
+      <c r="AA42" s="63"/>
       <c r="AB42" s="57"/>
       <c r="AC42" s="58"/>
       <c r="AD42" s="59"/>
@@ -2894,22 +2861,22 @@
       <c r="I43" s="61"/>
       <c r="J43" s="62"/>
       <c r="K43" s="54"/>
-      <c r="L43" s="92"/>
-      <c r="M43" s="94"/>
+      <c r="L43" s="55"/>
+      <c r="M43" s="63"/>
       <c r="N43" s="64"/>
       <c r="O43" s="61"/>
       <c r="P43" s="62"/>
       <c r="Q43" s="54"/>
-      <c r="R43" s="92"/>
-      <c r="S43" s="94"/>
+      <c r="R43" s="55"/>
+      <c r="S43" s="63"/>
       <c r="T43" s="64"/>
       <c r="U43" s="61"/>
       <c r="V43" s="62"/>
-      <c r="W43" s="91"/>
-      <c r="X43" s="92"/>
-      <c r="Y43" s="93"/>
-      <c r="Z43" s="91"/>
-      <c r="AA43" s="94"/>
+      <c r="W43" s="54"/>
+      <c r="X43" s="55"/>
+      <c r="Y43" s="56"/>
+      <c r="Z43" s="54"/>
+      <c r="AA43" s="63"/>
       <c r="AB43" s="57"/>
       <c r="AC43" s="58"/>
       <c r="AD43" s="59"/>
@@ -2930,22 +2897,22 @@
       <c r="I44" s="61"/>
       <c r="J44" s="62"/>
       <c r="K44" s="54"/>
-      <c r="L44" s="92"/>
-      <c r="M44" s="94"/>
+      <c r="L44" s="55"/>
+      <c r="M44" s="63"/>
       <c r="N44" s="64"/>
       <c r="O44" s="61"/>
       <c r="P44" s="62"/>
       <c r="Q44" s="54"/>
-      <c r="R44" s="92"/>
-      <c r="S44" s="94"/>
+      <c r="R44" s="55"/>
+      <c r="S44" s="63"/>
       <c r="T44" s="64"/>
       <c r="U44" s="61"/>
       <c r="V44" s="62"/>
-      <c r="W44" s="91"/>
-      <c r="X44" s="92"/>
-      <c r="Y44" s="93"/>
-      <c r="Z44" s="91"/>
-      <c r="AA44" s="94"/>
+      <c r="W44" s="54"/>
+      <c r="X44" s="55"/>
+      <c r="Y44" s="56"/>
+      <c r="Z44" s="54"/>
+      <c r="AA44" s="63"/>
       <c r="AB44" s="57"/>
       <c r="AC44" s="58"/>
       <c r="AD44" s="59"/>
@@ -2966,22 +2933,22 @@
       <c r="I45" s="61"/>
       <c r="J45" s="62"/>
       <c r="K45" s="54"/>
-      <c r="L45" s="92"/>
-      <c r="M45" s="94"/>
+      <c r="L45" s="55"/>
+      <c r="M45" s="63"/>
       <c r="N45" s="64"/>
       <c r="O45" s="61"/>
       <c r="P45" s="62"/>
       <c r="Q45" s="54"/>
-      <c r="R45" s="92"/>
-      <c r="S45" s="94"/>
+      <c r="R45" s="55"/>
+      <c r="S45" s="63"/>
       <c r="T45" s="64"/>
       <c r="U45" s="61"/>
       <c r="V45" s="62"/>
-      <c r="W45" s="91"/>
-      <c r="X45" s="92"/>
-      <c r="Y45" s="93"/>
-      <c r="Z45" s="91"/>
-      <c r="AA45" s="94"/>
+      <c r="W45" s="54"/>
+      <c r="X45" s="55"/>
+      <c r="Y45" s="56"/>
+      <c r="Z45" s="54"/>
+      <c r="AA45" s="63"/>
       <c r="AB45" s="57"/>
       <c r="AC45" s="58"/>
       <c r="AD45" s="59"/>
@@ -3002,22 +2969,22 @@
       <c r="I46" s="61"/>
       <c r="J46" s="62"/>
       <c r="K46" s="54"/>
-      <c r="L46" s="92"/>
-      <c r="M46" s="94"/>
+      <c r="L46" s="55"/>
+      <c r="M46" s="63"/>
       <c r="N46" s="64"/>
       <c r="O46" s="61"/>
       <c r="P46" s="62"/>
       <c r="Q46" s="54"/>
-      <c r="R46" s="92"/>
-      <c r="S46" s="94"/>
+      <c r="R46" s="55"/>
+      <c r="S46" s="63"/>
       <c r="T46" s="64"/>
       <c r="U46" s="61"/>
       <c r="V46" s="62"/>
-      <c r="W46" s="91"/>
-      <c r="X46" s="92"/>
-      <c r="Y46" s="93"/>
-      <c r="Z46" s="91"/>
-      <c r="AA46" s="94"/>
+      <c r="W46" s="54"/>
+      <c r="X46" s="55"/>
+      <c r="Y46" s="56"/>
+      <c r="Z46" s="54"/>
+      <c r="AA46" s="63"/>
       <c r="AB46" s="57"/>
       <c r="AC46" s="58"/>
       <c r="AD46" s="59"/>
@@ -3038,22 +3005,22 @@
       <c r="I47" s="61"/>
       <c r="J47" s="62"/>
       <c r="K47" s="54"/>
-      <c r="L47" s="92"/>
-      <c r="M47" s="94"/>
+      <c r="L47" s="55"/>
+      <c r="M47" s="63"/>
       <c r="N47" s="64"/>
       <c r="O47" s="61"/>
       <c r="P47" s="62"/>
       <c r="Q47" s="54"/>
-      <c r="R47" s="92"/>
-      <c r="S47" s="94"/>
+      <c r="R47" s="55"/>
+      <c r="S47" s="63"/>
       <c r="T47" s="64"/>
       <c r="U47" s="61"/>
       <c r="V47" s="62"/>
-      <c r="W47" s="91"/>
-      <c r="X47" s="92"/>
-      <c r="Y47" s="93"/>
-      <c r="Z47" s="91"/>
-      <c r="AA47" s="94"/>
+      <c r="W47" s="54"/>
+      <c r="X47" s="55"/>
+      <c r="Y47" s="56"/>
+      <c r="Z47" s="54"/>
+      <c r="AA47" s="63"/>
       <c r="AB47" s="57"/>
       <c r="AC47" s="58"/>
       <c r="AD47" s="59"/>
@@ -3074,22 +3041,22 @@
       <c r="I48" s="61"/>
       <c r="J48" s="62"/>
       <c r="K48" s="54"/>
-      <c r="L48" s="92"/>
-      <c r="M48" s="94"/>
+      <c r="L48" s="55"/>
+      <c r="M48" s="63"/>
       <c r="N48" s="64"/>
       <c r="O48" s="61"/>
       <c r="P48" s="62"/>
       <c r="Q48" s="54"/>
-      <c r="R48" s="92"/>
-      <c r="S48" s="94"/>
+      <c r="R48" s="55"/>
+      <c r="S48" s="63"/>
       <c r="T48" s="64"/>
       <c r="U48" s="61"/>
       <c r="V48" s="62"/>
-      <c r="W48" s="91"/>
-      <c r="X48" s="92"/>
-      <c r="Y48" s="93"/>
-      <c r="Z48" s="91"/>
-      <c r="AA48" s="94"/>
+      <c r="W48" s="54"/>
+      <c r="X48" s="55"/>
+      <c r="Y48" s="56"/>
+      <c r="Z48" s="54"/>
+      <c r="AA48" s="63"/>
       <c r="AB48" s="57"/>
       <c r="AC48" s="58"/>
       <c r="AD48" s="59"/>
@@ -3110,22 +3077,22 @@
       <c r="I49" s="61"/>
       <c r="J49" s="62"/>
       <c r="K49" s="54"/>
-      <c r="L49" s="92"/>
-      <c r="M49" s="94"/>
+      <c r="L49" s="55"/>
+      <c r="M49" s="63"/>
       <c r="N49" s="64"/>
       <c r="O49" s="61"/>
       <c r="P49" s="62"/>
       <c r="Q49" s="54"/>
-      <c r="R49" s="92"/>
-      <c r="S49" s="94"/>
+      <c r="R49" s="55"/>
+      <c r="S49" s="63"/>
       <c r="T49" s="64"/>
       <c r="U49" s="61"/>
       <c r="V49" s="62"/>
-      <c r="W49" s="91"/>
-      <c r="X49" s="92"/>
-      <c r="Y49" s="93"/>
-      <c r="Z49" s="91"/>
-      <c r="AA49" s="94"/>
+      <c r="W49" s="54"/>
+      <c r="X49" s="55"/>
+      <c r="Y49" s="56"/>
+      <c r="Z49" s="54"/>
+      <c r="AA49" s="63"/>
       <c r="AB49" s="57"/>
       <c r="AC49" s="58"/>
       <c r="AD49" s="59"/>
@@ -3146,22 +3113,22 @@
       <c r="I50" s="61"/>
       <c r="J50" s="62"/>
       <c r="K50" s="54"/>
-      <c r="L50" s="92"/>
-      <c r="M50" s="94"/>
+      <c r="L50" s="55"/>
+      <c r="M50" s="63"/>
       <c r="N50" s="64"/>
       <c r="O50" s="61"/>
       <c r="P50" s="62"/>
       <c r="Q50" s="54"/>
-      <c r="R50" s="92"/>
-      <c r="S50" s="94"/>
+      <c r="R50" s="55"/>
+      <c r="S50" s="63"/>
       <c r="T50" s="64"/>
       <c r="U50" s="61"/>
       <c r="V50" s="62"/>
-      <c r="W50" s="91"/>
-      <c r="X50" s="92"/>
-      <c r="Y50" s="93"/>
-      <c r="Z50" s="91"/>
-      <c r="AA50" s="94"/>
+      <c r="W50" s="54"/>
+      <c r="X50" s="55"/>
+      <c r="Y50" s="56"/>
+      <c r="Z50" s="54"/>
+      <c r="AA50" s="63"/>
       <c r="AB50" s="57"/>
       <c r="AC50" s="58"/>
       <c r="AD50" s="59"/>
@@ -3182,22 +3149,22 @@
       <c r="I51" s="61"/>
       <c r="J51" s="62"/>
       <c r="K51" s="54"/>
-      <c r="L51" s="92"/>
-      <c r="M51" s="94"/>
+      <c r="L51" s="55"/>
+      <c r="M51" s="63"/>
       <c r="N51" s="64"/>
       <c r="O51" s="61"/>
       <c r="P51" s="62"/>
       <c r="Q51" s="54"/>
-      <c r="R51" s="92"/>
-      <c r="S51" s="94"/>
+      <c r="R51" s="55"/>
+      <c r="S51" s="63"/>
       <c r="T51" s="64"/>
       <c r="U51" s="61"/>
       <c r="V51" s="62"/>
-      <c r="W51" s="91"/>
-      <c r="X51" s="92"/>
-      <c r="Y51" s="93"/>
-      <c r="Z51" s="91"/>
-      <c r="AA51" s="94"/>
+      <c r="W51" s="54"/>
+      <c r="X51" s="55"/>
+      <c r="Y51" s="56"/>
+      <c r="Z51" s="54"/>
+      <c r="AA51" s="63"/>
       <c r="AB51" s="57"/>
       <c r="AC51" s="58"/>
       <c r="AD51" s="59"/>
@@ -3218,22 +3185,22 @@
       <c r="I52" s="61"/>
       <c r="J52" s="62"/>
       <c r="K52" s="54"/>
-      <c r="L52" s="92"/>
-      <c r="M52" s="94"/>
+      <c r="L52" s="55"/>
+      <c r="M52" s="63"/>
       <c r="N52" s="64"/>
       <c r="O52" s="61"/>
       <c r="P52" s="62"/>
       <c r="Q52" s="54"/>
-      <c r="R52" s="92"/>
-      <c r="S52" s="94"/>
+      <c r="R52" s="55"/>
+      <c r="S52" s="63"/>
       <c r="T52" s="64"/>
       <c r="U52" s="61"/>
       <c r="V52" s="62"/>
-      <c r="W52" s="91"/>
-      <c r="X52" s="92"/>
-      <c r="Y52" s="93"/>
-      <c r="Z52" s="91"/>
-      <c r="AA52" s="94"/>
+      <c r="W52" s="54"/>
+      <c r="X52" s="55"/>
+      <c r="Y52" s="56"/>
+      <c r="Z52" s="54"/>
+      <c r="AA52" s="63"/>
       <c r="AB52" s="57"/>
       <c r="AC52" s="58"/>
       <c r="AD52" s="59"/>
@@ -3254,22 +3221,22 @@
       <c r="I53" s="61"/>
       <c r="J53" s="62"/>
       <c r="K53" s="54"/>
-      <c r="L53" s="92"/>
-      <c r="M53" s="94"/>
+      <c r="L53" s="55"/>
+      <c r="M53" s="63"/>
       <c r="N53" s="64"/>
       <c r="O53" s="61"/>
       <c r="P53" s="62"/>
       <c r="Q53" s="54"/>
-      <c r="R53" s="92"/>
-      <c r="S53" s="94"/>
+      <c r="R53" s="55"/>
+      <c r="S53" s="63"/>
       <c r="T53" s="64"/>
       <c r="U53" s="61"/>
       <c r="V53" s="62"/>
-      <c r="W53" s="91"/>
-      <c r="X53" s="92"/>
-      <c r="Y53" s="93"/>
-      <c r="Z53" s="91"/>
-      <c r="AA53" s="94"/>
+      <c r="W53" s="54"/>
+      <c r="X53" s="55"/>
+      <c r="Y53" s="56"/>
+      <c r="Z53" s="54"/>
+      <c r="AA53" s="63"/>
       <c r="AB53" s="57"/>
       <c r="AC53" s="58"/>
       <c r="AD53" s="59"/>
@@ -3290,22 +3257,22 @@
       <c r="I54" s="61"/>
       <c r="J54" s="62"/>
       <c r="K54" s="54"/>
-      <c r="L54" s="92"/>
-      <c r="M54" s="94"/>
+      <c r="L54" s="55"/>
+      <c r="M54" s="63"/>
       <c r="N54" s="64"/>
       <c r="O54" s="61"/>
       <c r="P54" s="62"/>
       <c r="Q54" s="54"/>
-      <c r="R54" s="92"/>
-      <c r="S54" s="94"/>
+      <c r="R54" s="55"/>
+      <c r="S54" s="63"/>
       <c r="T54" s="64"/>
       <c r="U54" s="61"/>
       <c r="V54" s="62"/>
-      <c r="W54" s="91"/>
-      <c r="X54" s="92"/>
-      <c r="Y54" s="93"/>
-      <c r="Z54" s="91"/>
-      <c r="AA54" s="94"/>
+      <c r="W54" s="54"/>
+      <c r="X54" s="55"/>
+      <c r="Y54" s="56"/>
+      <c r="Z54" s="54"/>
+      <c r="AA54" s="63"/>
       <c r="AB54" s="57"/>
       <c r="AC54" s="58"/>
       <c r="AD54" s="59"/>
@@ -3326,22 +3293,22 @@
       <c r="I55" s="61"/>
       <c r="J55" s="62"/>
       <c r="K55" s="54"/>
-      <c r="L55" s="92"/>
-      <c r="M55" s="94"/>
+      <c r="L55" s="55"/>
+      <c r="M55" s="63"/>
       <c r="N55" s="64"/>
       <c r="O55" s="61"/>
       <c r="P55" s="62"/>
       <c r="Q55" s="54"/>
-      <c r="R55" s="92"/>
-      <c r="S55" s="94"/>
+      <c r="R55" s="55"/>
+      <c r="S55" s="63"/>
       <c r="T55" s="64"/>
       <c r="U55" s="61"/>
       <c r="V55" s="62"/>
-      <c r="W55" s="91"/>
-      <c r="X55" s="92"/>
-      <c r="Y55" s="93"/>
-      <c r="Z55" s="91"/>
-      <c r="AA55" s="94"/>
+      <c r="W55" s="54"/>
+      <c r="X55" s="55"/>
+      <c r="Y55" s="56"/>
+      <c r="Z55" s="54"/>
+      <c r="AA55" s="63"/>
       <c r="AB55" s="57"/>
       <c r="AC55" s="58"/>
       <c r="AD55" s="59"/>
@@ -3362,22 +3329,22 @@
       <c r="I56" s="61"/>
       <c r="J56" s="62"/>
       <c r="K56" s="54"/>
-      <c r="L56" s="92"/>
-      <c r="M56" s="94"/>
+      <c r="L56" s="55"/>
+      <c r="M56" s="63"/>
       <c r="N56" s="64"/>
       <c r="O56" s="61"/>
       <c r="P56" s="62"/>
       <c r="Q56" s="54"/>
-      <c r="R56" s="92"/>
-      <c r="S56" s="94"/>
+      <c r="R56" s="55"/>
+      <c r="S56" s="63"/>
       <c r="T56" s="64"/>
       <c r="U56" s="61"/>
       <c r="V56" s="62"/>
-      <c r="W56" s="91"/>
-      <c r="X56" s="92"/>
-      <c r="Y56" s="93"/>
-      <c r="Z56" s="91"/>
-      <c r="AA56" s="94"/>
+      <c r="W56" s="54"/>
+      <c r="X56" s="55"/>
+      <c r="Y56" s="56"/>
+      <c r="Z56" s="54"/>
+      <c r="AA56" s="63"/>
       <c r="AB56" s="57"/>
       <c r="AC56" s="58"/>
       <c r="AD56" s="59"/>
@@ -3398,22 +3365,22 @@
       <c r="I57" s="61"/>
       <c r="J57" s="62"/>
       <c r="K57" s="54"/>
-      <c r="L57" s="92"/>
-      <c r="M57" s="94"/>
+      <c r="L57" s="55"/>
+      <c r="M57" s="63"/>
       <c r="N57" s="64"/>
       <c r="O57" s="61"/>
       <c r="P57" s="62"/>
       <c r="Q57" s="54"/>
-      <c r="R57" s="92"/>
-      <c r="S57" s="94"/>
+      <c r="R57" s="55"/>
+      <c r="S57" s="63"/>
       <c r="T57" s="64"/>
       <c r="U57" s="61"/>
       <c r="V57" s="62"/>
-      <c r="W57" s="91"/>
-      <c r="X57" s="92"/>
-      <c r="Y57" s="93"/>
-      <c r="Z57" s="91"/>
-      <c r="AA57" s="94"/>
+      <c r="W57" s="54"/>
+      <c r="X57" s="55"/>
+      <c r="Y57" s="56"/>
+      <c r="Z57" s="54"/>
+      <c r="AA57" s="63"/>
       <c r="AB57" s="57"/>
       <c r="AC57" s="58"/>
       <c r="AD57" s="59"/>
@@ -3434,22 +3401,22 @@
       <c r="I58" s="61"/>
       <c r="J58" s="62"/>
       <c r="K58" s="54"/>
-      <c r="L58" s="92"/>
-      <c r="M58" s="94"/>
+      <c r="L58" s="55"/>
+      <c r="M58" s="63"/>
       <c r="N58" s="64"/>
       <c r="O58" s="61"/>
       <c r="P58" s="62"/>
       <c r="Q58" s="54"/>
-      <c r="R58" s="92"/>
-      <c r="S58" s="94"/>
+      <c r="R58" s="55"/>
+      <c r="S58" s="63"/>
       <c r="T58" s="64"/>
       <c r="U58" s="61"/>
       <c r="V58" s="62"/>
-      <c r="W58" s="91"/>
-      <c r="X58" s="92"/>
-      <c r="Y58" s="93"/>
-      <c r="Z58" s="91"/>
-      <c r="AA58" s="94"/>
+      <c r="W58" s="54"/>
+      <c r="X58" s="55"/>
+      <c r="Y58" s="56"/>
+      <c r="Z58" s="54"/>
+      <c r="AA58" s="63"/>
       <c r="AB58" s="57"/>
       <c r="AC58" s="58"/>
       <c r="AD58" s="59"/>
@@ -3470,22 +3437,22 @@
       <c r="I59" s="61"/>
       <c r="J59" s="62"/>
       <c r="K59" s="54"/>
-      <c r="L59" s="92"/>
-      <c r="M59" s="94"/>
+      <c r="L59" s="55"/>
+      <c r="M59" s="63"/>
       <c r="N59" s="64"/>
       <c r="O59" s="61"/>
       <c r="P59" s="62"/>
       <c r="Q59" s="54"/>
-      <c r="R59" s="92"/>
-      <c r="S59" s="94"/>
+      <c r="R59" s="55"/>
+      <c r="S59" s="63"/>
       <c r="T59" s="64"/>
       <c r="U59" s="61"/>
       <c r="V59" s="62"/>
-      <c r="W59" s="91"/>
-      <c r="X59" s="92"/>
-      <c r="Y59" s="93"/>
-      <c r="Z59" s="91"/>
-      <c r="AA59" s="94"/>
+      <c r="W59" s="54"/>
+      <c r="X59" s="55"/>
+      <c r="Y59" s="56"/>
+      <c r="Z59" s="54"/>
+      <c r="AA59" s="63"/>
       <c r="AB59" s="57"/>
       <c r="AC59" s="58"/>
       <c r="AD59" s="59"/>
@@ -3506,22 +3473,22 @@
       <c r="I60" s="61"/>
       <c r="J60" s="62"/>
       <c r="K60" s="54"/>
-      <c r="L60" s="92"/>
-      <c r="M60" s="94"/>
+      <c r="L60" s="55"/>
+      <c r="M60" s="63"/>
       <c r="N60" s="64"/>
       <c r="O60" s="61"/>
       <c r="P60" s="62"/>
       <c r="Q60" s="54"/>
-      <c r="R60" s="92"/>
-      <c r="S60" s="94"/>
+      <c r="R60" s="55"/>
+      <c r="S60" s="63"/>
       <c r="T60" s="64"/>
       <c r="U60" s="61"/>
       <c r="V60" s="62"/>
-      <c r="W60" s="91"/>
-      <c r="X60" s="92"/>
-      <c r="Y60" s="93"/>
-      <c r="Z60" s="91"/>
-      <c r="AA60" s="94"/>
+      <c r="W60" s="54"/>
+      <c r="X60" s="55"/>
+      <c r="Y60" s="56"/>
+      <c r="Z60" s="54"/>
+      <c r="AA60" s="63"/>
       <c r="AB60" s="57"/>
       <c r="AC60" s="58"/>
       <c r="AD60" s="59"/>
@@ -3542,22 +3509,22 @@
       <c r="I61" s="61"/>
       <c r="J61" s="62"/>
       <c r="K61" s="54"/>
-      <c r="L61" s="92"/>
-      <c r="M61" s="94"/>
+      <c r="L61" s="55"/>
+      <c r="M61" s="63"/>
       <c r="N61" s="64"/>
       <c r="O61" s="61"/>
       <c r="P61" s="62"/>
       <c r="Q61" s="54"/>
-      <c r="R61" s="92"/>
-      <c r="S61" s="94"/>
+      <c r="R61" s="55"/>
+      <c r="S61" s="63"/>
       <c r="T61" s="64"/>
       <c r="U61" s="61"/>
       <c r="V61" s="62"/>
-      <c r="W61" s="91"/>
-      <c r="X61" s="92"/>
-      <c r="Y61" s="93"/>
-      <c r="Z61" s="91"/>
-      <c r="AA61" s="94"/>
+      <c r="W61" s="54"/>
+      <c r="X61" s="55"/>
+      <c r="Y61" s="56"/>
+      <c r="Z61" s="54"/>
+      <c r="AA61" s="63"/>
       <c r="AB61" s="57"/>
       <c r="AC61" s="58"/>
       <c r="AD61" s="59"/>
@@ -3578,22 +3545,22 @@
       <c r="I62" s="61"/>
       <c r="J62" s="62"/>
       <c r="K62" s="54"/>
-      <c r="L62" s="92"/>
-      <c r="M62" s="94"/>
+      <c r="L62" s="55"/>
+      <c r="M62" s="63"/>
       <c r="N62" s="64"/>
       <c r="O62" s="61"/>
       <c r="P62" s="62"/>
       <c r="Q62" s="54"/>
-      <c r="R62" s="92"/>
-      <c r="S62" s="94"/>
+      <c r="R62" s="55"/>
+      <c r="S62" s="63"/>
       <c r="T62" s="64"/>
       <c r="U62" s="61"/>
       <c r="V62" s="62"/>
-      <c r="W62" s="91"/>
-      <c r="X62" s="92"/>
-      <c r="Y62" s="93"/>
-      <c r="Z62" s="91"/>
-      <c r="AA62" s="94"/>
+      <c r="W62" s="54"/>
+      <c r="X62" s="55"/>
+      <c r="Y62" s="56"/>
+      <c r="Z62" s="54"/>
+      <c r="AA62" s="63"/>
       <c r="AB62" s="57"/>
       <c r="AC62" s="58"/>
       <c r="AD62" s="59"/>
@@ -3614,22 +3581,22 @@
       <c r="I63" s="61"/>
       <c r="J63" s="62"/>
       <c r="K63" s="54"/>
-      <c r="L63" s="92"/>
-      <c r="M63" s="94"/>
+      <c r="L63" s="55"/>
+      <c r="M63" s="63"/>
       <c r="N63" s="64"/>
       <c r="O63" s="61"/>
       <c r="P63" s="62"/>
       <c r="Q63" s="54"/>
-      <c r="R63" s="92"/>
-      <c r="S63" s="94"/>
+      <c r="R63" s="55"/>
+      <c r="S63" s="63"/>
       <c r="T63" s="64"/>
       <c r="U63" s="61"/>
       <c r="V63" s="62"/>
-      <c r="W63" s="91"/>
-      <c r="X63" s="92"/>
-      <c r="Y63" s="93"/>
-      <c r="Z63" s="91"/>
-      <c r="AA63" s="94"/>
+      <c r="W63" s="54"/>
+      <c r="X63" s="55"/>
+      <c r="Y63" s="56"/>
+      <c r="Z63" s="54"/>
+      <c r="AA63" s="63"/>
       <c r="AB63" s="57"/>
       <c r="AC63" s="58"/>
       <c r="AD63" s="59"/>
@@ -3650,22 +3617,22 @@
       <c r="I64" s="61"/>
       <c r="J64" s="62"/>
       <c r="K64" s="54"/>
-      <c r="L64" s="92"/>
-      <c r="M64" s="94"/>
+      <c r="L64" s="55"/>
+      <c r="M64" s="63"/>
       <c r="N64" s="64"/>
       <c r="O64" s="61"/>
       <c r="P64" s="62"/>
       <c r="Q64" s="54"/>
-      <c r="R64" s="92"/>
-      <c r="S64" s="94"/>
+      <c r="R64" s="55"/>
+      <c r="S64" s="63"/>
       <c r="T64" s="64"/>
       <c r="U64" s="61"/>
       <c r="V64" s="62"/>
-      <c r="W64" s="91"/>
-      <c r="X64" s="92"/>
-      <c r="Y64" s="93"/>
-      <c r="Z64" s="91"/>
-      <c r="AA64" s="94"/>
+      <c r="W64" s="54"/>
+      <c r="X64" s="55"/>
+      <c r="Y64" s="56"/>
+      <c r="Z64" s="54"/>
+      <c r="AA64" s="63"/>
       <c r="AB64" s="57"/>
       <c r="AC64" s="58"/>
       <c r="AD64" s="59"/>
@@ -3686,22 +3653,22 @@
       <c r="I65" s="61"/>
       <c r="J65" s="62"/>
       <c r="K65" s="54"/>
-      <c r="L65" s="92"/>
-      <c r="M65" s="94"/>
+      <c r="L65" s="55"/>
+      <c r="M65" s="63"/>
       <c r="N65" s="64"/>
       <c r="O65" s="61"/>
       <c r="P65" s="62"/>
       <c r="Q65" s="54"/>
-      <c r="R65" s="92"/>
-      <c r="S65" s="94"/>
+      <c r="R65" s="55"/>
+      <c r="S65" s="63"/>
       <c r="T65" s="64"/>
       <c r="U65" s="61"/>
       <c r="V65" s="62"/>
-      <c r="W65" s="91"/>
-      <c r="X65" s="92"/>
-      <c r="Y65" s="93"/>
-      <c r="Z65" s="91"/>
-      <c r="AA65" s="94"/>
+      <c r="W65" s="54"/>
+      <c r="X65" s="55"/>
+      <c r="Y65" s="56"/>
+      <c r="Z65" s="54"/>
+      <c r="AA65" s="63"/>
       <c r="AB65" s="57"/>
       <c r="AC65" s="58"/>
       <c r="AD65" s="59"/>
@@ -3722,22 +3689,22 @@
       <c r="I66" s="61"/>
       <c r="J66" s="62"/>
       <c r="K66" s="54"/>
-      <c r="L66" s="92"/>
-      <c r="M66" s="94"/>
+      <c r="L66" s="55"/>
+      <c r="M66" s="63"/>
       <c r="N66" s="64"/>
       <c r="O66" s="61"/>
       <c r="P66" s="62"/>
       <c r="Q66" s="54"/>
-      <c r="R66" s="92"/>
-      <c r="S66" s="94"/>
+      <c r="R66" s="55"/>
+      <c r="S66" s="63"/>
       <c r="T66" s="64"/>
       <c r="U66" s="61"/>
       <c r="V66" s="62"/>
-      <c r="W66" s="91"/>
-      <c r="X66" s="92"/>
-      <c r="Y66" s="93"/>
-      <c r="Z66" s="91"/>
-      <c r="AA66" s="94"/>
+      <c r="W66" s="54"/>
+      <c r="X66" s="55"/>
+      <c r="Y66" s="56"/>
+      <c r="Z66" s="54"/>
+      <c r="AA66" s="63"/>
       <c r="AB66" s="57"/>
       <c r="AC66" s="58"/>
       <c r="AD66" s="59"/>
@@ -3758,22 +3725,22 @@
       <c r="I67" s="61"/>
       <c r="J67" s="62"/>
       <c r="K67" s="54"/>
-      <c r="L67" s="92"/>
-      <c r="M67" s="94"/>
+      <c r="L67" s="55"/>
+      <c r="M67" s="63"/>
       <c r="N67" s="64"/>
       <c r="O67" s="61"/>
       <c r="P67" s="62"/>
       <c r="Q67" s="54"/>
-      <c r="R67" s="92"/>
-      <c r="S67" s="94"/>
+      <c r="R67" s="55"/>
+      <c r="S67" s="63"/>
       <c r="T67" s="64"/>
       <c r="U67" s="61"/>
       <c r="V67" s="62"/>
-      <c r="W67" s="91"/>
-      <c r="X67" s="92"/>
-      <c r="Y67" s="93"/>
-      <c r="Z67" s="91"/>
-      <c r="AA67" s="94"/>
+      <c r="W67" s="54"/>
+      <c r="X67" s="55"/>
+      <c r="Y67" s="56"/>
+      <c r="Z67" s="54"/>
+      <c r="AA67" s="63"/>
       <c r="AB67" s="57"/>
       <c r="AC67" s="58"/>
       <c r="AD67" s="59"/>
@@ -3830,22 +3797,22 @@
       <c r="I69" s="48"/>
       <c r="J69" s="49"/>
       <c r="K69" s="50"/>
-      <c r="L69" s="89"/>
-      <c r="M69" s="90"/>
+      <c r="L69" s="51"/>
+      <c r="M69" s="52"/>
       <c r="N69" s="53"/>
       <c r="O69" s="48"/>
       <c r="P69" s="49"/>
       <c r="Q69" s="50"/>
-      <c r="R69" s="89"/>
-      <c r="S69" s="90"/>
+      <c r="R69" s="51"/>
+      <c r="S69" s="52"/>
       <c r="T69" s="53"/>
       <c r="U69" s="48"/>
       <c r="V69" s="49"/>
-      <c r="W69" s="91"/>
-      <c r="X69" s="92"/>
-      <c r="Y69" s="93"/>
-      <c r="Z69" s="88"/>
-      <c r="AA69" s="90"/>
+      <c r="W69" s="54"/>
+      <c r="X69" s="55"/>
+      <c r="Y69" s="56"/>
+      <c r="Z69" s="50"/>
+      <c r="AA69" s="52"/>
       <c r="AB69" s="57"/>
       <c r="AC69" s="58"/>
       <c r="AD69" s="69"/>
@@ -3866,22 +3833,22 @@
       <c r="I70" s="61"/>
       <c r="J70" s="62"/>
       <c r="K70" s="54"/>
-      <c r="L70" s="92"/>
-      <c r="M70" s="94"/>
+      <c r="L70" s="55"/>
+      <c r="M70" s="63"/>
       <c r="N70" s="64"/>
       <c r="O70" s="61"/>
       <c r="P70" s="62"/>
       <c r="Q70" s="54"/>
-      <c r="R70" s="92"/>
-      <c r="S70" s="94"/>
+      <c r="R70" s="55"/>
+      <c r="S70" s="63"/>
       <c r="T70" s="64"/>
       <c r="U70" s="61"/>
       <c r="V70" s="62"/>
-      <c r="W70" s="91"/>
-      <c r="X70" s="92"/>
-      <c r="Y70" s="93"/>
-      <c r="Z70" s="91"/>
-      <c r="AA70" s="94"/>
+      <c r="W70" s="54"/>
+      <c r="X70" s="55"/>
+      <c r="Y70" s="56"/>
+      <c r="Z70" s="54"/>
+      <c r="AA70" s="63"/>
       <c r="AB70" s="57"/>
       <c r="AC70" s="58"/>
       <c r="AD70" s="59"/>
@@ -3902,22 +3869,22 @@
       <c r="I71" s="61"/>
       <c r="J71" s="62"/>
       <c r="K71" s="54"/>
-      <c r="L71" s="92"/>
-      <c r="M71" s="94"/>
+      <c r="L71" s="55"/>
+      <c r="M71" s="63"/>
       <c r="N71" s="64"/>
       <c r="O71" s="61"/>
       <c r="P71" s="62"/>
       <c r="Q71" s="54"/>
-      <c r="R71" s="92"/>
-      <c r="S71" s="94"/>
+      <c r="R71" s="55"/>
+      <c r="S71" s="63"/>
       <c r="T71" s="64"/>
       <c r="U71" s="61"/>
       <c r="V71" s="62"/>
-      <c r="W71" s="91"/>
-      <c r="X71" s="92"/>
-      <c r="Y71" s="93"/>
-      <c r="Z71" s="91"/>
-      <c r="AA71" s="94"/>
+      <c r="W71" s="54"/>
+      <c r="X71" s="55"/>
+      <c r="Y71" s="56"/>
+      <c r="Z71" s="54"/>
+      <c r="AA71" s="63"/>
       <c r="AB71" s="57"/>
       <c r="AC71" s="58"/>
       <c r="AD71" s="59"/>
@@ -3938,22 +3905,22 @@
       <c r="I72" s="61"/>
       <c r="J72" s="62"/>
       <c r="K72" s="54"/>
-      <c r="L72" s="92"/>
-      <c r="M72" s="94"/>
+      <c r="L72" s="55"/>
+      <c r="M72" s="63"/>
       <c r="N72" s="64"/>
       <c r="O72" s="61"/>
       <c r="P72" s="62"/>
       <c r="Q72" s="54"/>
-      <c r="R72" s="92"/>
-      <c r="S72" s="94"/>
+      <c r="R72" s="55"/>
+      <c r="S72" s="63"/>
       <c r="T72" s="64"/>
       <c r="U72" s="61"/>
       <c r="V72" s="62"/>
-      <c r="W72" s="91"/>
-      <c r="X72" s="92"/>
-      <c r="Y72" s="93"/>
-      <c r="Z72" s="91"/>
-      <c r="AA72" s="94"/>
+      <c r="W72" s="54"/>
+      <c r="X72" s="55"/>
+      <c r="Y72" s="56"/>
+      <c r="Z72" s="54"/>
+      <c r="AA72" s="63"/>
       <c r="AB72" s="57"/>
       <c r="AC72" s="58"/>
       <c r="AD72" s="59"/>
@@ -3974,22 +3941,22 @@
       <c r="I73" s="61"/>
       <c r="J73" s="62"/>
       <c r="K73" s="54"/>
-      <c r="L73" s="92"/>
-      <c r="M73" s="94"/>
+      <c r="L73" s="55"/>
+      <c r="M73" s="63"/>
       <c r="N73" s="64"/>
       <c r="O73" s="61"/>
       <c r="P73" s="62"/>
       <c r="Q73" s="54"/>
-      <c r="R73" s="92"/>
-      <c r="S73" s="94"/>
+      <c r="R73" s="55"/>
+      <c r="S73" s="63"/>
       <c r="T73" s="64"/>
       <c r="U73" s="61"/>
       <c r="V73" s="62"/>
-      <c r="W73" s="91"/>
-      <c r="X73" s="92"/>
-      <c r="Y73" s="93"/>
-      <c r="Z73" s="91"/>
-      <c r="AA73" s="94"/>
+      <c r="W73" s="54"/>
+      <c r="X73" s="55"/>
+      <c r="Y73" s="56"/>
+      <c r="Z73" s="54"/>
+      <c r="AA73" s="63"/>
       <c r="AB73" s="57"/>
       <c r="AC73" s="58"/>
       <c r="AD73" s="72"/>
@@ -4010,22 +3977,22 @@
       <c r="I74" s="61"/>
       <c r="J74" s="62"/>
       <c r="K74" s="54"/>
-      <c r="L74" s="92"/>
-      <c r="M74" s="94"/>
+      <c r="L74" s="55"/>
+      <c r="M74" s="63"/>
       <c r="N74" s="64"/>
       <c r="O74" s="61"/>
       <c r="P74" s="62"/>
       <c r="Q74" s="54"/>
-      <c r="R74" s="92"/>
-      <c r="S74" s="94"/>
+      <c r="R74" s="55"/>
+      <c r="S74" s="63"/>
       <c r="T74" s="64"/>
       <c r="U74" s="61"/>
       <c r="V74" s="62"/>
-      <c r="W74" s="91"/>
-      <c r="X74" s="92"/>
-      <c r="Y74" s="93"/>
-      <c r="Z74" s="91"/>
-      <c r="AA74" s="94"/>
+      <c r="W74" s="54"/>
+      <c r="X74" s="55"/>
+      <c r="Y74" s="56"/>
+      <c r="Z74" s="54"/>
+      <c r="AA74" s="63"/>
       <c r="AB74" s="57"/>
       <c r="AC74" s="58"/>
       <c r="AD74" s="72"/>
@@ -4046,22 +4013,22 @@
       <c r="I75" s="61"/>
       <c r="J75" s="62"/>
       <c r="K75" s="54"/>
-      <c r="L75" s="92"/>
-      <c r="M75" s="94"/>
+      <c r="L75" s="55"/>
+      <c r="M75" s="63"/>
       <c r="N75" s="64"/>
       <c r="O75" s="61"/>
       <c r="P75" s="62"/>
       <c r="Q75" s="54"/>
-      <c r="R75" s="92"/>
-      <c r="S75" s="94"/>
+      <c r="R75" s="55"/>
+      <c r="S75" s="63"/>
       <c r="T75" s="64"/>
       <c r="U75" s="61"/>
       <c r="V75" s="62"/>
-      <c r="W75" s="91"/>
-      <c r="X75" s="92"/>
-      <c r="Y75" s="93"/>
-      <c r="Z75" s="91"/>
-      <c r="AA75" s="94"/>
+      <c r="W75" s="54"/>
+      <c r="X75" s="55"/>
+      <c r="Y75" s="56"/>
+      <c r="Z75" s="54"/>
+      <c r="AA75" s="63"/>
       <c r="AB75" s="57"/>
       <c r="AC75" s="58"/>
       <c r="AD75" s="72"/>
@@ -4082,22 +4049,22 @@
       <c r="I76" s="61"/>
       <c r="J76" s="62"/>
       <c r="K76" s="54"/>
-      <c r="L76" s="92"/>
-      <c r="M76" s="94"/>
+      <c r="L76" s="55"/>
+      <c r="M76" s="63"/>
       <c r="N76" s="64"/>
       <c r="O76" s="61"/>
       <c r="P76" s="62"/>
       <c r="Q76" s="54"/>
-      <c r="R76" s="92"/>
-      <c r="S76" s="94"/>
+      <c r="R76" s="55"/>
+      <c r="S76" s="63"/>
       <c r="T76" s="64"/>
       <c r="U76" s="61"/>
       <c r="V76" s="62"/>
-      <c r="W76" s="91"/>
-      <c r="X76" s="92"/>
-      <c r="Y76" s="93"/>
-      <c r="Z76" s="91"/>
-      <c r="AA76" s="94"/>
+      <c r="W76" s="54"/>
+      <c r="X76" s="55"/>
+      <c r="Y76" s="56"/>
+      <c r="Z76" s="54"/>
+      <c r="AA76" s="63"/>
       <c r="AB76" s="57"/>
       <c r="AC76" s="58"/>
       <c r="AD76" s="72"/>
@@ -4118,22 +4085,22 @@
       <c r="I77" s="61"/>
       <c r="J77" s="62"/>
       <c r="K77" s="54"/>
-      <c r="L77" s="92"/>
-      <c r="M77" s="94"/>
+      <c r="L77" s="55"/>
+      <c r="M77" s="63"/>
       <c r="N77" s="64"/>
       <c r="O77" s="61"/>
       <c r="P77" s="62"/>
       <c r="Q77" s="54"/>
-      <c r="R77" s="92"/>
-      <c r="S77" s="94"/>
+      <c r="R77" s="55"/>
+      <c r="S77" s="63"/>
       <c r="T77" s="64"/>
       <c r="U77" s="61"/>
       <c r="V77" s="62"/>
-      <c r="W77" s="91"/>
-      <c r="X77" s="92"/>
-      <c r="Y77" s="93"/>
-      <c r="Z77" s="91"/>
-      <c r="AA77" s="94"/>
+      <c r="W77" s="54"/>
+      <c r="X77" s="55"/>
+      <c r="Y77" s="56"/>
+      <c r="Z77" s="54"/>
+      <c r="AA77" s="63"/>
       <c r="AB77" s="57"/>
       <c r="AC77" s="58"/>
       <c r="AD77" s="72"/>
@@ -4154,22 +4121,22 @@
       <c r="I78" s="61"/>
       <c r="J78" s="62"/>
       <c r="K78" s="54"/>
-      <c r="L78" s="92"/>
-      <c r="M78" s="94"/>
+      <c r="L78" s="55"/>
+      <c r="M78" s="63"/>
       <c r="N78" s="64"/>
       <c r="O78" s="61"/>
       <c r="P78" s="62"/>
       <c r="Q78" s="54"/>
-      <c r="R78" s="92"/>
-      <c r="S78" s="94"/>
+      <c r="R78" s="55"/>
+      <c r="S78" s="63"/>
       <c r="T78" s="64"/>
       <c r="U78" s="61"/>
       <c r="V78" s="62"/>
-      <c r="W78" s="91"/>
-      <c r="X78" s="92"/>
-      <c r="Y78" s="93"/>
-      <c r="Z78" s="91"/>
-      <c r="AA78" s="94"/>
+      <c r="W78" s="54"/>
+      <c r="X78" s="55"/>
+      <c r="Y78" s="56"/>
+      <c r="Z78" s="54"/>
+      <c r="AA78" s="63"/>
       <c r="AB78" s="57"/>
       <c r="AC78" s="58"/>
       <c r="AD78" s="72"/>
@@ -4190,22 +4157,22 @@
       <c r="I79" s="61"/>
       <c r="J79" s="62"/>
       <c r="K79" s="54"/>
-      <c r="L79" s="92"/>
-      <c r="M79" s="94"/>
+      <c r="L79" s="55"/>
+      <c r="M79" s="63"/>
       <c r="N79" s="64"/>
       <c r="O79" s="61"/>
       <c r="P79" s="62"/>
       <c r="Q79" s="54"/>
-      <c r="R79" s="92"/>
-      <c r="S79" s="94"/>
+      <c r="R79" s="55"/>
+      <c r="S79" s="63"/>
       <c r="T79" s="64"/>
       <c r="U79" s="61"/>
       <c r="V79" s="62"/>
-      <c r="W79" s="91"/>
-      <c r="X79" s="92"/>
-      <c r="Y79" s="93"/>
-      <c r="Z79" s="91"/>
-      <c r="AA79" s="94"/>
+      <c r="W79" s="54"/>
+      <c r="X79" s="55"/>
+      <c r="Y79" s="56"/>
+      <c r="Z79" s="54"/>
+      <c r="AA79" s="63"/>
       <c r="AB79" s="57"/>
       <c r="AC79" s="58"/>
       <c r="AD79" s="72"/>
@@ -4226,22 +4193,22 @@
       <c r="I80" s="61"/>
       <c r="J80" s="62"/>
       <c r="K80" s="54"/>
-      <c r="L80" s="92"/>
-      <c r="M80" s="94"/>
+      <c r="L80" s="55"/>
+      <c r="M80" s="63"/>
       <c r="N80" s="64"/>
       <c r="O80" s="61"/>
       <c r="P80" s="62"/>
       <c r="Q80" s="54"/>
-      <c r="R80" s="92"/>
-      <c r="S80" s="94"/>
+      <c r="R80" s="55"/>
+      <c r="S80" s="63"/>
       <c r="T80" s="64"/>
       <c r="U80" s="61"/>
       <c r="V80" s="62"/>
-      <c r="W80" s="91"/>
-      <c r="X80" s="92"/>
-      <c r="Y80" s="93"/>
-      <c r="Z80" s="91"/>
-      <c r="AA80" s="94"/>
+      <c r="W80" s="54"/>
+      <c r="X80" s="55"/>
+      <c r="Y80" s="56"/>
+      <c r="Z80" s="54"/>
+      <c r="AA80" s="63"/>
       <c r="AB80" s="57"/>
       <c r="AC80" s="58"/>
       <c r="AD80" s="72"/>
@@ -4262,22 +4229,22 @@
       <c r="I81" s="61"/>
       <c r="J81" s="62"/>
       <c r="K81" s="54"/>
-      <c r="L81" s="92"/>
-      <c r="M81" s="94"/>
+      <c r="L81" s="55"/>
+      <c r="M81" s="63"/>
       <c r="N81" s="64"/>
       <c r="O81" s="61"/>
       <c r="P81" s="62"/>
       <c r="Q81" s="54"/>
-      <c r="R81" s="92"/>
-      <c r="S81" s="94"/>
+      <c r="R81" s="55"/>
+      <c r="S81" s="63"/>
       <c r="T81" s="64"/>
       <c r="U81" s="61"/>
       <c r="V81" s="62"/>
-      <c r="W81" s="91"/>
-      <c r="X81" s="92"/>
-      <c r="Y81" s="93"/>
-      <c r="Z81" s="91"/>
-      <c r="AA81" s="94"/>
+      <c r="W81" s="54"/>
+      <c r="X81" s="55"/>
+      <c r="Y81" s="56"/>
+      <c r="Z81" s="54"/>
+      <c r="AA81" s="63"/>
       <c r="AB81" s="57"/>
       <c r="AC81" s="58"/>
       <c r="AD81" s="72"/>
@@ -4298,22 +4265,22 @@
       <c r="I82" s="61"/>
       <c r="J82" s="62"/>
       <c r="K82" s="54"/>
-      <c r="L82" s="92"/>
-      <c r="M82" s="94"/>
+      <c r="L82" s="55"/>
+      <c r="M82" s="63"/>
       <c r="N82" s="64"/>
       <c r="O82" s="61"/>
       <c r="P82" s="62"/>
       <c r="Q82" s="54"/>
-      <c r="R82" s="92"/>
-      <c r="S82" s="94"/>
+      <c r="R82" s="55"/>
+      <c r="S82" s="63"/>
       <c r="T82" s="64"/>
       <c r="U82" s="61"/>
       <c r="V82" s="62"/>
-      <c r="W82" s="91"/>
-      <c r="X82" s="92"/>
-      <c r="Y82" s="93"/>
-      <c r="Z82" s="91"/>
-      <c r="AA82" s="94"/>
+      <c r="W82" s="54"/>
+      <c r="X82" s="55"/>
+      <c r="Y82" s="56"/>
+      <c r="Z82" s="54"/>
+      <c r="AA82" s="63"/>
       <c r="AB82" s="57"/>
       <c r="AC82" s="58"/>
       <c r="AD82" s="72"/>
@@ -4334,22 +4301,22 @@
       <c r="I83" s="61"/>
       <c r="J83" s="62"/>
       <c r="K83" s="54"/>
-      <c r="L83" s="92"/>
-      <c r="M83" s="94"/>
+      <c r="L83" s="55"/>
+      <c r="M83" s="63"/>
       <c r="N83" s="64"/>
       <c r="O83" s="61"/>
       <c r="P83" s="62"/>
       <c r="Q83" s="54"/>
-      <c r="R83" s="92"/>
-      <c r="S83" s="94"/>
+      <c r="R83" s="55"/>
+      <c r="S83" s="63"/>
       <c r="T83" s="64"/>
       <c r="U83" s="61"/>
       <c r="V83" s="62"/>
-      <c r="W83" s="91"/>
-      <c r="X83" s="92"/>
-      <c r="Y83" s="93"/>
-      <c r="Z83" s="91"/>
-      <c r="AA83" s="94"/>
+      <c r="W83" s="54"/>
+      <c r="X83" s="55"/>
+      <c r="Y83" s="56"/>
+      <c r="Z83" s="54"/>
+      <c r="AA83" s="63"/>
       <c r="AB83" s="57"/>
       <c r="AC83" s="58"/>
       <c r="AD83" s="72"/>
@@ -4370,22 +4337,22 @@
       <c r="I84" s="61"/>
       <c r="J84" s="62"/>
       <c r="K84" s="54"/>
-      <c r="L84" s="92"/>
-      <c r="M84" s="94"/>
+      <c r="L84" s="55"/>
+      <c r="M84" s="63"/>
       <c r="N84" s="64"/>
       <c r="O84" s="61"/>
       <c r="P84" s="62"/>
       <c r="Q84" s="54"/>
-      <c r="R84" s="92"/>
-      <c r="S84" s="94"/>
+      <c r="R84" s="55"/>
+      <c r="S84" s="63"/>
       <c r="T84" s="64"/>
       <c r="U84" s="61"/>
       <c r="V84" s="62"/>
-      <c r="W84" s="91"/>
-      <c r="X84" s="92"/>
-      <c r="Y84" s="93"/>
-      <c r="Z84" s="91"/>
-      <c r="AA84" s="94"/>
+      <c r="W84" s="54"/>
+      <c r="X84" s="55"/>
+      <c r="Y84" s="56"/>
+      <c r="Z84" s="54"/>
+      <c r="AA84" s="63"/>
       <c r="AB84" s="57"/>
       <c r="AC84" s="58"/>
       <c r="AD84" s="72"/>
@@ -4406,22 +4373,22 @@
       <c r="I85" s="61"/>
       <c r="J85" s="62"/>
       <c r="K85" s="54"/>
-      <c r="L85" s="92"/>
-      <c r="M85" s="94"/>
+      <c r="L85" s="55"/>
+      <c r="M85" s="63"/>
       <c r="N85" s="64"/>
       <c r="O85" s="61"/>
       <c r="P85" s="62"/>
       <c r="Q85" s="54"/>
-      <c r="R85" s="92"/>
-      <c r="S85" s="94"/>
+      <c r="R85" s="55"/>
+      <c r="S85" s="63"/>
       <c r="T85" s="64"/>
       <c r="U85" s="61"/>
       <c r="V85" s="62"/>
-      <c r="W85" s="91"/>
-      <c r="X85" s="92"/>
-      <c r="Y85" s="93"/>
-      <c r="Z85" s="91"/>
-      <c r="AA85" s="94"/>
+      <c r="W85" s="54"/>
+      <c r="X85" s="55"/>
+      <c r="Y85" s="56"/>
+      <c r="Z85" s="54"/>
+      <c r="AA85" s="63"/>
       <c r="AB85" s="57"/>
       <c r="AC85" s="58"/>
       <c r="AD85" s="72"/>
@@ -4442,22 +4409,22 @@
       <c r="I86" s="61"/>
       <c r="J86" s="62"/>
       <c r="K86" s="54"/>
-      <c r="L86" s="92"/>
-      <c r="M86" s="94"/>
+      <c r="L86" s="55"/>
+      <c r="M86" s="63"/>
       <c r="N86" s="64"/>
       <c r="O86" s="61"/>
       <c r="P86" s="62"/>
       <c r="Q86" s="54"/>
-      <c r="R86" s="92"/>
-      <c r="S86" s="94"/>
+      <c r="R86" s="55"/>
+      <c r="S86" s="63"/>
       <c r="T86" s="64"/>
       <c r="U86" s="61"/>
       <c r="V86" s="62"/>
-      <c r="W86" s="91"/>
-      <c r="X86" s="92"/>
-      <c r="Y86" s="93"/>
-      <c r="Z86" s="91"/>
-      <c r="AA86" s="94"/>
+      <c r="W86" s="54"/>
+      <c r="X86" s="55"/>
+      <c r="Y86" s="56"/>
+      <c r="Z86" s="54"/>
+      <c r="AA86" s="63"/>
       <c r="AB86" s="57"/>
       <c r="AC86" s="58"/>
       <c r="AD86" s="72"/>
@@ -4478,22 +4445,22 @@
       <c r="I87" s="61"/>
       <c r="J87" s="62"/>
       <c r="K87" s="54"/>
-      <c r="L87" s="92"/>
-      <c r="M87" s="94"/>
+      <c r="L87" s="55"/>
+      <c r="M87" s="63"/>
       <c r="N87" s="64"/>
       <c r="O87" s="61"/>
       <c r="P87" s="62"/>
       <c r="Q87" s="54"/>
-      <c r="R87" s="92"/>
-      <c r="S87" s="94"/>
+      <c r="R87" s="55"/>
+      <c r="S87" s="63"/>
       <c r="T87" s="64"/>
       <c r="U87" s="61"/>
       <c r="V87" s="62"/>
-      <c r="W87" s="91"/>
-      <c r="X87" s="92"/>
-      <c r="Y87" s="93"/>
-      <c r="Z87" s="91"/>
-      <c r="AA87" s="94"/>
+      <c r="W87" s="54"/>
+      <c r="X87" s="55"/>
+      <c r="Y87" s="56"/>
+      <c r="Z87" s="54"/>
+      <c r="AA87" s="63"/>
       <c r="AB87" s="57"/>
       <c r="AC87" s="58"/>
       <c r="AD87" s="72"/>
@@ -4514,22 +4481,22 @@
       <c r="I88" s="61"/>
       <c r="J88" s="62"/>
       <c r="K88" s="54"/>
-      <c r="L88" s="92"/>
-      <c r="M88" s="94"/>
+      <c r="L88" s="55"/>
+      <c r="M88" s="63"/>
       <c r="N88" s="64"/>
       <c r="O88" s="61"/>
       <c r="P88" s="62"/>
       <c r="Q88" s="54"/>
-      <c r="R88" s="92"/>
-      <c r="S88" s="94"/>
+      <c r="R88" s="55"/>
+      <c r="S88" s="63"/>
       <c r="T88" s="64"/>
       <c r="U88" s="61"/>
       <c r="V88" s="62"/>
-      <c r="W88" s="91"/>
-      <c r="X88" s="92"/>
-      <c r="Y88" s="93"/>
-      <c r="Z88" s="91"/>
-      <c r="AA88" s="94"/>
+      <c r="W88" s="54"/>
+      <c r="X88" s="55"/>
+      <c r="Y88" s="56"/>
+      <c r="Z88" s="54"/>
+      <c r="AA88" s="63"/>
       <c r="AB88" s="57"/>
       <c r="AC88" s="58"/>
       <c r="AD88" s="72"/>
@@ -4550,22 +4517,22 @@
       <c r="I89" s="61"/>
       <c r="J89" s="62"/>
       <c r="K89" s="54"/>
-      <c r="L89" s="92"/>
-      <c r="M89" s="94"/>
+      <c r="L89" s="55"/>
+      <c r="M89" s="63"/>
       <c r="N89" s="64"/>
       <c r="O89" s="61"/>
       <c r="P89" s="62"/>
       <c r="Q89" s="54"/>
-      <c r="R89" s="92"/>
-      <c r="S89" s="94"/>
+      <c r="R89" s="55"/>
+      <c r="S89" s="63"/>
       <c r="T89" s="64"/>
       <c r="U89" s="61"/>
       <c r="V89" s="62"/>
-      <c r="W89" s="91"/>
-      <c r="X89" s="92"/>
-      <c r="Y89" s="93"/>
-      <c r="Z89" s="91"/>
-      <c r="AA89" s="94"/>
+      <c r="W89" s="54"/>
+      <c r="X89" s="55"/>
+      <c r="Y89" s="56"/>
+      <c r="Z89" s="54"/>
+      <c r="AA89" s="63"/>
       <c r="AB89" s="57"/>
       <c r="AC89" s="58"/>
       <c r="AD89" s="72"/>
@@ -4586,22 +4553,22 @@
       <c r="I90" s="61"/>
       <c r="J90" s="62"/>
       <c r="K90" s="54"/>
-      <c r="L90" s="92"/>
-      <c r="M90" s="94"/>
+      <c r="L90" s="55"/>
+      <c r="M90" s="63"/>
       <c r="N90" s="64"/>
       <c r="O90" s="61"/>
       <c r="P90" s="62"/>
       <c r="Q90" s="54"/>
-      <c r="R90" s="92"/>
-      <c r="S90" s="94"/>
+      <c r="R90" s="55"/>
+      <c r="S90" s="63"/>
       <c r="T90" s="64"/>
       <c r="U90" s="61"/>
       <c r="V90" s="62"/>
-      <c r="W90" s="91"/>
-      <c r="X90" s="92"/>
-      <c r="Y90" s="93"/>
-      <c r="Z90" s="91"/>
-      <c r="AA90" s="94"/>
+      <c r="W90" s="54"/>
+      <c r="X90" s="55"/>
+      <c r="Y90" s="56"/>
+      <c r="Z90" s="54"/>
+      <c r="AA90" s="63"/>
       <c r="AB90" s="57"/>
       <c r="AC90" s="58"/>
       <c r="AD90" s="72"/>
@@ -4622,22 +4589,22 @@
       <c r="I91" s="61"/>
       <c r="J91" s="62"/>
       <c r="K91" s="54"/>
-      <c r="L91" s="92"/>
-      <c r="M91" s="94"/>
+      <c r="L91" s="55"/>
+      <c r="M91" s="63"/>
       <c r="N91" s="64"/>
       <c r="O91" s="61"/>
       <c r="P91" s="62"/>
       <c r="Q91" s="54"/>
-      <c r="R91" s="92"/>
-      <c r="S91" s="94"/>
+      <c r="R91" s="55"/>
+      <c r="S91" s="63"/>
       <c r="T91" s="64"/>
       <c r="U91" s="61"/>
       <c r="V91" s="62"/>
-      <c r="W91" s="91"/>
-      <c r="X91" s="92"/>
-      <c r="Y91" s="93"/>
-      <c r="Z91" s="91"/>
-      <c r="AA91" s="94"/>
+      <c r="W91" s="54"/>
+      <c r="X91" s="55"/>
+      <c r="Y91" s="56"/>
+      <c r="Z91" s="54"/>
+      <c r="AA91" s="63"/>
       <c r="AB91" s="57"/>
       <c r="AC91" s="58"/>
       <c r="AD91" s="72"/>
@@ -4658,22 +4625,22 @@
       <c r="I92" s="61"/>
       <c r="J92" s="62"/>
       <c r="K92" s="54"/>
-      <c r="L92" s="92"/>
-      <c r="M92" s="94"/>
+      <c r="L92" s="55"/>
+      <c r="M92" s="63"/>
       <c r="N92" s="64"/>
       <c r="O92" s="61"/>
       <c r="P92" s="62"/>
       <c r="Q92" s="54"/>
-      <c r="R92" s="92"/>
-      <c r="S92" s="94"/>
+      <c r="R92" s="55"/>
+      <c r="S92" s="63"/>
       <c r="T92" s="64"/>
       <c r="U92" s="61"/>
       <c r="V92" s="62"/>
-      <c r="W92" s="91"/>
-      <c r="X92" s="92"/>
-      <c r="Y92" s="93"/>
-      <c r="Z92" s="91"/>
-      <c r="AA92" s="94"/>
+      <c r="W92" s="54"/>
+      <c r="X92" s="55"/>
+      <c r="Y92" s="56"/>
+      <c r="Z92" s="54"/>
+      <c r="AA92" s="63"/>
       <c r="AB92" s="57"/>
       <c r="AC92" s="58"/>
       <c r="AD92" s="72"/>
@@ -4694,22 +4661,22 @@
       <c r="I93" s="61"/>
       <c r="J93" s="62"/>
       <c r="K93" s="54"/>
-      <c r="L93" s="92"/>
-      <c r="M93" s="94"/>
+      <c r="L93" s="55"/>
+      <c r="M93" s="63"/>
       <c r="N93" s="64"/>
       <c r="O93" s="61"/>
       <c r="P93" s="62"/>
       <c r="Q93" s="54"/>
-      <c r="R93" s="92"/>
-      <c r="S93" s="94"/>
+      <c r="R93" s="55"/>
+      <c r="S93" s="63"/>
       <c r="T93" s="64"/>
       <c r="U93" s="61"/>
       <c r="V93" s="62"/>
-      <c r="W93" s="91"/>
-      <c r="X93" s="92"/>
-      <c r="Y93" s="93"/>
-      <c r="Z93" s="91"/>
-      <c r="AA93" s="94"/>
+      <c r="W93" s="54"/>
+      <c r="X93" s="55"/>
+      <c r="Y93" s="56"/>
+      <c r="Z93" s="54"/>
+      <c r="AA93" s="63"/>
       <c r="AB93" s="57"/>
       <c r="AC93" s="58"/>
       <c r="AD93" s="72"/>
@@ -4730,22 +4697,22 @@
       <c r="I94" s="61"/>
       <c r="J94" s="62"/>
       <c r="K94" s="54"/>
-      <c r="L94" s="92"/>
-      <c r="M94" s="94"/>
+      <c r="L94" s="55"/>
+      <c r="M94" s="63"/>
       <c r="N94" s="64"/>
       <c r="O94" s="61"/>
       <c r="P94" s="62"/>
       <c r="Q94" s="54"/>
-      <c r="R94" s="92"/>
-      <c r="S94" s="94"/>
+      <c r="R94" s="55"/>
+      <c r="S94" s="63"/>
       <c r="T94" s="64"/>
       <c r="U94" s="61"/>
       <c r="V94" s="62"/>
-      <c r="W94" s="91"/>
-      <c r="X94" s="92"/>
-      <c r="Y94" s="93"/>
-      <c r="Z94" s="91"/>
-      <c r="AA94" s="94"/>
+      <c r="W94" s="54"/>
+      <c r="X94" s="55"/>
+      <c r="Y94" s="56"/>
+      <c r="Z94" s="54"/>
+      <c r="AA94" s="63"/>
       <c r="AB94" s="57"/>
       <c r="AC94" s="58"/>
       <c r="AD94" s="72"/>
@@ -4766,22 +4733,22 @@
       <c r="I95" s="61"/>
       <c r="J95" s="62"/>
       <c r="K95" s="54"/>
-      <c r="L95" s="92"/>
-      <c r="M95" s="94"/>
+      <c r="L95" s="55"/>
+      <c r="M95" s="63"/>
       <c r="N95" s="64"/>
       <c r="O95" s="61"/>
       <c r="P95" s="62"/>
       <c r="Q95" s="54"/>
-      <c r="R95" s="92"/>
-      <c r="S95" s="94"/>
+      <c r="R95" s="55"/>
+      <c r="S95" s="63"/>
       <c r="T95" s="64"/>
       <c r="U95" s="61"/>
       <c r="V95" s="62"/>
-      <c r="W95" s="91"/>
-      <c r="X95" s="92"/>
-      <c r="Y95" s="93"/>
-      <c r="Z95" s="91"/>
-      <c r="AA95" s="94"/>
+      <c r="W95" s="54"/>
+      <c r="X95" s="55"/>
+      <c r="Y95" s="56"/>
+      <c r="Z95" s="54"/>
+      <c r="AA95" s="63"/>
       <c r="AB95" s="57"/>
       <c r="AC95" s="58"/>
       <c r="AD95" s="72"/>
@@ -4802,22 +4769,22 @@
       <c r="I96" s="61"/>
       <c r="J96" s="62"/>
       <c r="K96" s="54"/>
-      <c r="L96" s="92"/>
-      <c r="M96" s="94"/>
+      <c r="L96" s="55"/>
+      <c r="M96" s="63"/>
       <c r="N96" s="64"/>
       <c r="O96" s="61"/>
       <c r="P96" s="62"/>
       <c r="Q96" s="54"/>
-      <c r="R96" s="92"/>
-      <c r="S96" s="94"/>
+      <c r="R96" s="55"/>
+      <c r="S96" s="63"/>
       <c r="T96" s="64"/>
       <c r="U96" s="61"/>
       <c r="V96" s="62"/>
-      <c r="W96" s="91"/>
-      <c r="X96" s="92"/>
-      <c r="Y96" s="93"/>
-      <c r="Z96" s="91"/>
-      <c r="AA96" s="94"/>
+      <c r="W96" s="54"/>
+      <c r="X96" s="55"/>
+      <c r="Y96" s="56"/>
+      <c r="Z96" s="54"/>
+      <c r="AA96" s="63"/>
       <c r="AB96" s="57"/>
       <c r="AC96" s="58"/>
       <c r="AD96" s="72"/>
@@ -4838,22 +4805,22 @@
       <c r="I97" s="61"/>
       <c r="J97" s="62"/>
       <c r="K97" s="54"/>
-      <c r="L97" s="92"/>
-      <c r="M97" s="94"/>
+      <c r="L97" s="55"/>
+      <c r="M97" s="63"/>
       <c r="N97" s="64"/>
       <c r="O97" s="61"/>
       <c r="P97" s="62"/>
       <c r="Q97" s="54"/>
-      <c r="R97" s="92"/>
-      <c r="S97" s="94"/>
+      <c r="R97" s="55"/>
+      <c r="S97" s="63"/>
       <c r="T97" s="64"/>
       <c r="U97" s="61"/>
       <c r="V97" s="62"/>
-      <c r="W97" s="91"/>
-      <c r="X97" s="92"/>
-      <c r="Y97" s="93"/>
-      <c r="Z97" s="91"/>
-      <c r="AA97" s="94"/>
+      <c r="W97" s="54"/>
+      <c r="X97" s="55"/>
+      <c r="Y97" s="56"/>
+      <c r="Z97" s="54"/>
+      <c r="AA97" s="63"/>
       <c r="AB97" s="57"/>
       <c r="AC97" s="58"/>
       <c r="AD97" s="72"/>
@@ -4874,22 +4841,22 @@
       <c r="I98" s="61"/>
       <c r="J98" s="62"/>
       <c r="K98" s="54"/>
-      <c r="L98" s="92"/>
-      <c r="M98" s="94"/>
+      <c r="L98" s="55"/>
+      <c r="M98" s="63"/>
       <c r="N98" s="64"/>
       <c r="O98" s="61"/>
       <c r="P98" s="62"/>
       <c r="Q98" s="54"/>
-      <c r="R98" s="92"/>
-      <c r="S98" s="94"/>
+      <c r="R98" s="55"/>
+      <c r="S98" s="63"/>
       <c r="T98" s="64"/>
       <c r="U98" s="61"/>
       <c r="V98" s="62"/>
-      <c r="W98" s="91"/>
-      <c r="X98" s="92"/>
-      <c r="Y98" s="93"/>
-      <c r="Z98" s="91"/>
-      <c r="AA98" s="94"/>
+      <c r="W98" s="54"/>
+      <c r="X98" s="55"/>
+      <c r="Y98" s="56"/>
+      <c r="Z98" s="54"/>
+      <c r="AA98" s="63"/>
       <c r="AB98" s="57"/>
       <c r="AC98" s="58"/>
       <c r="AD98" s="72"/>
@@ -4910,22 +4877,22 @@
       <c r="I99" s="61"/>
       <c r="J99" s="62"/>
       <c r="K99" s="54"/>
-      <c r="L99" s="92"/>
-      <c r="M99" s="94"/>
+      <c r="L99" s="55"/>
+      <c r="M99" s="63"/>
       <c r="N99" s="64"/>
       <c r="O99" s="61"/>
       <c r="P99" s="62"/>
       <c r="Q99" s="54"/>
-      <c r="R99" s="92"/>
-      <c r="S99" s="94"/>
+      <c r="R99" s="55"/>
+      <c r="S99" s="63"/>
       <c r="T99" s="64"/>
       <c r="U99" s="61"/>
       <c r="V99" s="62"/>
-      <c r="W99" s="91"/>
-      <c r="X99" s="92"/>
-      <c r="Y99" s="93"/>
-      <c r="Z99" s="91"/>
-      <c r="AA99" s="94"/>
+      <c r="W99" s="54"/>
+      <c r="X99" s="55"/>
+      <c r="Y99" s="56"/>
+      <c r="Z99" s="54"/>
+      <c r="AA99" s="63"/>
       <c r="AB99" s="57"/>
       <c r="AC99" s="58"/>
       <c r="AD99" s="72"/>
@@ -4946,22 +4913,22 @@
       <c r="I100" s="61"/>
       <c r="J100" s="62"/>
       <c r="K100" s="54"/>
-      <c r="L100" s="92"/>
-      <c r="M100" s="94"/>
+      <c r="L100" s="55"/>
+      <c r="M100" s="63"/>
       <c r="N100" s="64"/>
       <c r="O100" s="61"/>
       <c r="P100" s="62"/>
       <c r="Q100" s="54"/>
-      <c r="R100" s="92"/>
-      <c r="S100" s="94"/>
+      <c r="R100" s="55"/>
+      <c r="S100" s="63"/>
       <c r="T100" s="64"/>
       <c r="U100" s="61"/>
       <c r="V100" s="62"/>
-      <c r="W100" s="91"/>
-      <c r="X100" s="92"/>
-      <c r="Y100" s="93"/>
-      <c r="Z100" s="91"/>
-      <c r="AA100" s="94"/>
+      <c r="W100" s="54"/>
+      <c r="X100" s="55"/>
+      <c r="Y100" s="56"/>
+      <c r="Z100" s="54"/>
+      <c r="AA100" s="63"/>
       <c r="AB100" s="57"/>
       <c r="AC100" s="58"/>
       <c r="AD100" s="72"/>
@@ -4982,22 +4949,22 @@
       <c r="I101" s="61"/>
       <c r="J101" s="62"/>
       <c r="K101" s="54"/>
-      <c r="L101" s="92"/>
-      <c r="M101" s="94"/>
+      <c r="L101" s="55"/>
+      <c r="M101" s="63"/>
       <c r="N101" s="64"/>
       <c r="O101" s="61"/>
       <c r="P101" s="62"/>
       <c r="Q101" s="54"/>
-      <c r="R101" s="92"/>
-      <c r="S101" s="94"/>
+      <c r="R101" s="55"/>
+      <c r="S101" s="63"/>
       <c r="T101" s="64"/>
       <c r="U101" s="61"/>
       <c r="V101" s="62"/>
-      <c r="W101" s="91"/>
-      <c r="X101" s="92"/>
-      <c r="Y101" s="93"/>
-      <c r="Z101" s="91"/>
-      <c r="AA101" s="94"/>
+      <c r="W101" s="54"/>
+      <c r="X101" s="55"/>
+      <c r="Y101" s="56"/>
+      <c r="Z101" s="54"/>
+      <c r="AA101" s="63"/>
       <c r="AB101" s="57"/>
       <c r="AC101" s="58"/>
       <c r="AD101" s="72"/>
@@ -5018,22 +4985,22 @@
       <c r="I102" s="61"/>
       <c r="J102" s="62"/>
       <c r="K102" s="54"/>
-      <c r="L102" s="92"/>
-      <c r="M102" s="94"/>
+      <c r="L102" s="55"/>
+      <c r="M102" s="63"/>
       <c r="N102" s="64"/>
       <c r="O102" s="61"/>
       <c r="P102" s="62"/>
       <c r="Q102" s="54"/>
-      <c r="R102" s="92"/>
-      <c r="S102" s="94"/>
+      <c r="R102" s="55"/>
+      <c r="S102" s="63"/>
       <c r="T102" s="64"/>
       <c r="U102" s="61"/>
       <c r="V102" s="62"/>
-      <c r="W102" s="91"/>
-      <c r="X102" s="92"/>
-      <c r="Y102" s="93"/>
-      <c r="Z102" s="91"/>
-      <c r="AA102" s="94"/>
+      <c r="W102" s="54"/>
+      <c r="X102" s="55"/>
+      <c r="Y102" s="56"/>
+      <c r="Z102" s="54"/>
+      <c r="AA102" s="63"/>
       <c r="AB102" s="57"/>
       <c r="AC102" s="58"/>
       <c r="AD102" s="72"/>
@@ -5054,22 +5021,22 @@
       <c r="I103" s="61"/>
       <c r="J103" s="62"/>
       <c r="K103" s="54"/>
-      <c r="L103" s="92"/>
-      <c r="M103" s="94"/>
+      <c r="L103" s="55"/>
+      <c r="M103" s="63"/>
       <c r="N103" s="64"/>
       <c r="O103" s="61"/>
       <c r="P103" s="62"/>
       <c r="Q103" s="54"/>
-      <c r="R103" s="92"/>
-      <c r="S103" s="94"/>
+      <c r="R103" s="55"/>
+      <c r="S103" s="63"/>
       <c r="T103" s="64"/>
       <c r="U103" s="61"/>
       <c r="V103" s="62"/>
-      <c r="W103" s="91"/>
-      <c r="X103" s="92"/>
-      <c r="Y103" s="93"/>
-      <c r="Z103" s="91"/>
-      <c r="AA103" s="94"/>
+      <c r="W103" s="54"/>
+      <c r="X103" s="55"/>
+      <c r="Y103" s="56"/>
+      <c r="Z103" s="54"/>
+      <c r="AA103" s="63"/>
       <c r="AB103" s="57"/>
       <c r="AC103" s="58"/>
       <c r="AD103" s="72"/>
@@ -5090,22 +5057,22 @@
       <c r="I104" s="61"/>
       <c r="J104" s="62"/>
       <c r="K104" s="54"/>
-      <c r="L104" s="92"/>
-      <c r="M104" s="94"/>
+      <c r="L104" s="55"/>
+      <c r="M104" s="63"/>
       <c r="N104" s="64"/>
       <c r="O104" s="61"/>
       <c r="P104" s="62"/>
       <c r="Q104" s="54"/>
-      <c r="R104" s="92"/>
-      <c r="S104" s="94"/>
+      <c r="R104" s="55"/>
+      <c r="S104" s="63"/>
       <c r="T104" s="64"/>
       <c r="U104" s="61"/>
       <c r="V104" s="62"/>
-      <c r="W104" s="91"/>
-      <c r="X104" s="92"/>
-      <c r="Y104" s="93"/>
-      <c r="Z104" s="91"/>
-      <c r="AA104" s="94"/>
+      <c r="W104" s="54"/>
+      <c r="X104" s="55"/>
+      <c r="Y104" s="56"/>
+      <c r="Z104" s="54"/>
+      <c r="AA104" s="63"/>
       <c r="AB104" s="57"/>
       <c r="AC104" s="58"/>
       <c r="AD104" s="72"/>
@@ -5126,22 +5093,22 @@
       <c r="I105" s="61"/>
       <c r="J105" s="62"/>
       <c r="K105" s="54"/>
-      <c r="L105" s="92"/>
-      <c r="M105" s="94"/>
+      <c r="L105" s="55"/>
+      <c r="M105" s="63"/>
       <c r="N105" s="64"/>
       <c r="O105" s="61"/>
       <c r="P105" s="62"/>
       <c r="Q105" s="54"/>
-      <c r="R105" s="92"/>
-      <c r="S105" s="94"/>
+      <c r="R105" s="55"/>
+      <c r="S105" s="63"/>
       <c r="T105" s="64"/>
       <c r="U105" s="61"/>
       <c r="V105" s="62"/>
-      <c r="W105" s="91"/>
-      <c r="X105" s="92"/>
-      <c r="Y105" s="93"/>
-      <c r="Z105" s="91"/>
-      <c r="AA105" s="94"/>
+      <c r="W105" s="54"/>
+      <c r="X105" s="55"/>
+      <c r="Y105" s="56"/>
+      <c r="Z105" s="54"/>
+      <c r="AA105" s="63"/>
       <c r="AB105" s="57"/>
       <c r="AC105" s="58"/>
       <c r="AD105" s="72"/>
@@ -5162,22 +5129,22 @@
       <c r="I106" s="61"/>
       <c r="J106" s="62"/>
       <c r="K106" s="54"/>
-      <c r="L106" s="92"/>
-      <c r="M106" s="94"/>
+      <c r="L106" s="55"/>
+      <c r="M106" s="63"/>
       <c r="N106" s="64"/>
       <c r="O106" s="61"/>
       <c r="P106" s="62"/>
       <c r="Q106" s="54"/>
-      <c r="R106" s="92"/>
-      <c r="S106" s="94"/>
+      <c r="R106" s="55"/>
+      <c r="S106" s="63"/>
       <c r="T106" s="64"/>
       <c r="U106" s="61"/>
       <c r="V106" s="62"/>
-      <c r="W106" s="91"/>
-      <c r="X106" s="92"/>
-      <c r="Y106" s="93"/>
-      <c r="Z106" s="91"/>
-      <c r="AA106" s="94"/>
+      <c r="W106" s="54"/>
+      <c r="X106" s="55"/>
+      <c r="Y106" s="56"/>
+      <c r="Z106" s="54"/>
+      <c r="AA106" s="63"/>
       <c r="AB106" s="57"/>
       <c r="AC106" s="58"/>
       <c r="AD106" s="72"/>
@@ -5198,22 +5165,22 @@
       <c r="I107" s="61"/>
       <c r="J107" s="62"/>
       <c r="K107" s="54"/>
-      <c r="L107" s="92"/>
-      <c r="M107" s="94"/>
+      <c r="L107" s="55"/>
+      <c r="M107" s="63"/>
       <c r="N107" s="64"/>
       <c r="O107" s="61"/>
       <c r="P107" s="62"/>
       <c r="Q107" s="54"/>
-      <c r="R107" s="92"/>
-      <c r="S107" s="94"/>
+      <c r="R107" s="55"/>
+      <c r="S107" s="63"/>
       <c r="T107" s="64"/>
       <c r="U107" s="61"/>
       <c r="V107" s="62"/>
-      <c r="W107" s="91"/>
-      <c r="X107" s="92"/>
-      <c r="Y107" s="93"/>
-      <c r="Z107" s="91"/>
-      <c r="AA107" s="94"/>
+      <c r="W107" s="54"/>
+      <c r="X107" s="55"/>
+      <c r="Y107" s="56"/>
+      <c r="Z107" s="54"/>
+      <c r="AA107" s="63"/>
       <c r="AB107" s="57"/>
       <c r="AC107" s="58"/>
       <c r="AD107" s="72"/>
@@ -5234,22 +5201,22 @@
       <c r="I108" s="61"/>
       <c r="J108" s="62"/>
       <c r="K108" s="54"/>
-      <c r="L108" s="92"/>
-      <c r="M108" s="94"/>
+      <c r="L108" s="55"/>
+      <c r="M108" s="63"/>
       <c r="N108" s="64"/>
       <c r="O108" s="61"/>
       <c r="P108" s="62"/>
       <c r="Q108" s="54"/>
-      <c r="R108" s="92"/>
-      <c r="S108" s="94"/>
+      <c r="R108" s="55"/>
+      <c r="S108" s="63"/>
       <c r="T108" s="64"/>
       <c r="U108" s="61"/>
       <c r="V108" s="62"/>
-      <c r="W108" s="91"/>
-      <c r="X108" s="92"/>
-      <c r="Y108" s="93"/>
-      <c r="Z108" s="91"/>
-      <c r="AA108" s="94"/>
+      <c r="W108" s="54"/>
+      <c r="X108" s="55"/>
+      <c r="Y108" s="56"/>
+      <c r="Z108" s="54"/>
+      <c r="AA108" s="63"/>
       <c r="AB108" s="57"/>
       <c r="AC108" s="58"/>
       <c r="AD108" s="72"/>
@@ -5270,22 +5237,22 @@
       <c r="I109" s="61"/>
       <c r="J109" s="62"/>
       <c r="K109" s="54"/>
-      <c r="L109" s="92"/>
-      <c r="M109" s="94"/>
+      <c r="L109" s="55"/>
+      <c r="M109" s="63"/>
       <c r="N109" s="64"/>
       <c r="O109" s="61"/>
       <c r="P109" s="62"/>
       <c r="Q109" s="54"/>
-      <c r="R109" s="92"/>
-      <c r="S109" s="94"/>
+      <c r="R109" s="55"/>
+      <c r="S109" s="63"/>
       <c r="T109" s="64"/>
       <c r="U109" s="61"/>
       <c r="V109" s="62"/>
-      <c r="W109" s="91"/>
-      <c r="X109" s="92"/>
-      <c r="Y109" s="93"/>
-      <c r="Z109" s="91"/>
-      <c r="AA109" s="94"/>
+      <c r="W109" s="54"/>
+      <c r="X109" s="55"/>
+      <c r="Y109" s="56"/>
+      <c r="Z109" s="54"/>
+      <c r="AA109" s="63"/>
       <c r="AB109" s="57"/>
       <c r="AC109" s="58"/>
       <c r="AD109" s="72"/>
@@ -5306,22 +5273,22 @@
       <c r="I110" s="61"/>
       <c r="J110" s="62"/>
       <c r="K110" s="54"/>
-      <c r="L110" s="92"/>
-      <c r="M110" s="94"/>
+      <c r="L110" s="55"/>
+      <c r="M110" s="63"/>
       <c r="N110" s="64"/>
       <c r="O110" s="61"/>
       <c r="P110" s="62"/>
       <c r="Q110" s="54"/>
-      <c r="R110" s="92"/>
-      <c r="S110" s="94"/>
+      <c r="R110" s="55"/>
+      <c r="S110" s="63"/>
       <c r="T110" s="64"/>
       <c r="U110" s="61"/>
       <c r="V110" s="62"/>
-      <c r="W110" s="91"/>
-      <c r="X110" s="92"/>
-      <c r="Y110" s="93"/>
-      <c r="Z110" s="91"/>
-      <c r="AA110" s="94"/>
+      <c r="W110" s="54"/>
+      <c r="X110" s="55"/>
+      <c r="Y110" s="56"/>
+      <c r="Z110" s="54"/>
+      <c r="AA110" s="63"/>
       <c r="AB110" s="57"/>
       <c r="AC110" s="58"/>
       <c r="AD110" s="72"/>
@@ -5342,22 +5309,22 @@
       <c r="I111" s="61"/>
       <c r="J111" s="62"/>
       <c r="K111" s="54"/>
-      <c r="L111" s="92"/>
-      <c r="M111" s="94"/>
+      <c r="L111" s="55"/>
+      <c r="M111" s="63"/>
       <c r="N111" s="64"/>
       <c r="O111" s="61"/>
       <c r="P111" s="62"/>
       <c r="Q111" s="54"/>
-      <c r="R111" s="92"/>
-      <c r="S111" s="94"/>
+      <c r="R111" s="55"/>
+      <c r="S111" s="63"/>
       <c r="T111" s="64"/>
       <c r="U111" s="61"/>
       <c r="V111" s="62"/>
-      <c r="W111" s="91"/>
-      <c r="X111" s="92"/>
-      <c r="Y111" s="93"/>
-      <c r="Z111" s="91"/>
-      <c r="AA111" s="94"/>
+      <c r="W111" s="54"/>
+      <c r="X111" s="55"/>
+      <c r="Y111" s="56"/>
+      <c r="Z111" s="54"/>
+      <c r="AA111" s="63"/>
       <c r="AB111" s="57"/>
       <c r="AC111" s="58"/>
       <c r="AD111" s="72"/>
@@ -5378,22 +5345,22 @@
       <c r="I112" s="61"/>
       <c r="J112" s="62"/>
       <c r="K112" s="54"/>
-      <c r="L112" s="92"/>
-      <c r="M112" s="94"/>
+      <c r="L112" s="55"/>
+      <c r="M112" s="63"/>
       <c r="N112" s="64"/>
       <c r="O112" s="61"/>
       <c r="P112" s="62"/>
       <c r="Q112" s="54"/>
-      <c r="R112" s="92"/>
-      <c r="S112" s="94"/>
+      <c r="R112" s="55"/>
+      <c r="S112" s="63"/>
       <c r="T112" s="64"/>
       <c r="U112" s="61"/>
       <c r="V112" s="62"/>
-      <c r="W112" s="91"/>
-      <c r="X112" s="92"/>
-      <c r="Y112" s="93"/>
-      <c r="Z112" s="91"/>
-      <c r="AA112" s="94"/>
+      <c r="W112" s="54"/>
+      <c r="X112" s="55"/>
+      <c r="Y112" s="56"/>
+      <c r="Z112" s="54"/>
+      <c r="AA112" s="63"/>
       <c r="AB112" s="57"/>
       <c r="AC112" s="58"/>
       <c r="AD112" s="72"/>
@@ -5414,22 +5381,22 @@
       <c r="I113" s="61"/>
       <c r="J113" s="62"/>
       <c r="K113" s="54"/>
-      <c r="L113" s="92"/>
-      <c r="M113" s="94"/>
+      <c r="L113" s="55"/>
+      <c r="M113" s="63"/>
       <c r="N113" s="64"/>
       <c r="O113" s="61"/>
       <c r="P113" s="62"/>
       <c r="Q113" s="54"/>
-      <c r="R113" s="92"/>
-      <c r="S113" s="94"/>
+      <c r="R113" s="55"/>
+      <c r="S113" s="63"/>
       <c r="T113" s="64"/>
       <c r="U113" s="61"/>
       <c r="V113" s="62"/>
-      <c r="W113" s="91"/>
-      <c r="X113" s="92"/>
-      <c r="Y113" s="93"/>
-      <c r="Z113" s="91"/>
-      <c r="AA113" s="94"/>
+      <c r="W113" s="54"/>
+      <c r="X113" s="55"/>
+      <c r="Y113" s="56"/>
+      <c r="Z113" s="54"/>
+      <c r="AA113" s="63"/>
       <c r="AB113" s="57"/>
       <c r="AC113" s="58"/>
       <c r="AD113" s="72"/>
@@ -5450,22 +5417,22 @@
       <c r="I114" s="61"/>
       <c r="J114" s="62"/>
       <c r="K114" s="54"/>
-      <c r="L114" s="92"/>
-      <c r="M114" s="94"/>
+      <c r="L114" s="55"/>
+      <c r="M114" s="63"/>
       <c r="N114" s="64"/>
       <c r="O114" s="61"/>
       <c r="P114" s="62"/>
       <c r="Q114" s="54"/>
-      <c r="R114" s="92"/>
-      <c r="S114" s="94"/>
+      <c r="R114" s="55"/>
+      <c r="S114" s="63"/>
       <c r="T114" s="64"/>
       <c r="U114" s="61"/>
       <c r="V114" s="62"/>
-      <c r="W114" s="91"/>
-      <c r="X114" s="92"/>
-      <c r="Y114" s="93"/>
-      <c r="Z114" s="91"/>
-      <c r="AA114" s="94"/>
+      <c r="W114" s="54"/>
+      <c r="X114" s="55"/>
+      <c r="Y114" s="56"/>
+      <c r="Z114" s="54"/>
+      <c r="AA114" s="63"/>
       <c r="AB114" s="57"/>
       <c r="AC114" s="58"/>
       <c r="AD114" s="72"/>
@@ -5486,22 +5453,22 @@
       <c r="I115" s="61"/>
       <c r="J115" s="62"/>
       <c r="K115" s="54"/>
-      <c r="L115" s="92"/>
-      <c r="M115" s="94"/>
+      <c r="L115" s="55"/>
+      <c r="M115" s="63"/>
       <c r="N115" s="64"/>
       <c r="O115" s="61"/>
       <c r="P115" s="62"/>
       <c r="Q115" s="54"/>
-      <c r="R115" s="92"/>
-      <c r="S115" s="94"/>
+      <c r="R115" s="55"/>
+      <c r="S115" s="63"/>
       <c r="T115" s="64"/>
       <c r="U115" s="61"/>
       <c r="V115" s="62"/>
-      <c r="W115" s="91"/>
-      <c r="X115" s="92"/>
-      <c r="Y115" s="93"/>
-      <c r="Z115" s="91"/>
-      <c r="AA115" s="94"/>
+      <c r="W115" s="54"/>
+      <c r="X115" s="55"/>
+      <c r="Y115" s="56"/>
+      <c r="Z115" s="54"/>
+      <c r="AA115" s="63"/>
       <c r="AB115" s="57"/>
       <c r="AC115" s="58"/>
       <c r="AD115" s="72"/>
@@ -5522,22 +5489,22 @@
       <c r="I116" s="61"/>
       <c r="J116" s="62"/>
       <c r="K116" s="54"/>
-      <c r="L116" s="92"/>
-      <c r="M116" s="94"/>
+      <c r="L116" s="55"/>
+      <c r="M116" s="63"/>
       <c r="N116" s="64"/>
       <c r="O116" s="61"/>
       <c r="P116" s="62"/>
       <c r="Q116" s="54"/>
-      <c r="R116" s="92"/>
-      <c r="S116" s="94"/>
+      <c r="R116" s="55"/>
+      <c r="S116" s="63"/>
       <c r="T116" s="64"/>
       <c r="U116" s="61"/>
       <c r="V116" s="62"/>
-      <c r="W116" s="91"/>
-      <c r="X116" s="92"/>
-      <c r="Y116" s="93"/>
-      <c r="Z116" s="91"/>
-      <c r="AA116" s="94"/>
+      <c r="W116" s="54"/>
+      <c r="X116" s="55"/>
+      <c r="Y116" s="56"/>
+      <c r="Z116" s="54"/>
+      <c r="AA116" s="63"/>
       <c r="AB116" s="57"/>
       <c r="AC116" s="58"/>
       <c r="AD116" s="72"/>
@@ -5558,22 +5525,22 @@
       <c r="I117" s="61"/>
       <c r="J117" s="62"/>
       <c r="K117" s="54"/>
-      <c r="L117" s="92"/>
-      <c r="M117" s="94"/>
+      <c r="L117" s="55"/>
+      <c r="M117" s="63"/>
       <c r="N117" s="64"/>
       <c r="O117" s="61"/>
       <c r="P117" s="62"/>
       <c r="Q117" s="54"/>
-      <c r="R117" s="92"/>
-      <c r="S117" s="94"/>
+      <c r="R117" s="55"/>
+      <c r="S117" s="63"/>
       <c r="T117" s="64"/>
       <c r="U117" s="61"/>
       <c r="V117" s="62"/>
-      <c r="W117" s="91"/>
-      <c r="X117" s="92"/>
-      <c r="Y117" s="93"/>
-      <c r="Z117" s="91"/>
-      <c r="AA117" s="94"/>
+      <c r="W117" s="54"/>
+      <c r="X117" s="55"/>
+      <c r="Y117" s="56"/>
+      <c r="Z117" s="54"/>
+      <c r="AA117" s="63"/>
       <c r="AB117" s="57"/>
       <c r="AC117" s="58"/>
       <c r="AD117" s="72"/>
@@ -5594,22 +5561,22 @@
       <c r="I118" s="77"/>
       <c r="J118" s="78"/>
       <c r="K118" s="79"/>
-      <c r="L118" s="96"/>
-      <c r="M118" s="97"/>
+      <c r="L118" s="80"/>
+      <c r="M118" s="81"/>
       <c r="N118" s="76"/>
       <c r="O118" s="77"/>
       <c r="P118" s="78"/>
       <c r="Q118" s="79"/>
-      <c r="R118" s="96"/>
-      <c r="S118" s="97"/>
+      <c r="R118" s="80"/>
+      <c r="S118" s="81"/>
       <c r="T118" s="76"/>
       <c r="U118" s="77"/>
       <c r="V118" s="78"/>
-      <c r="W118" s="95"/>
-      <c r="X118" s="96"/>
-      <c r="Y118" s="98"/>
-      <c r="Z118" s="95"/>
-      <c r="AA118" s="97"/>
+      <c r="W118" s="79"/>
+      <c r="X118" s="80"/>
+      <c r="Y118" s="82"/>
+      <c r="Z118" s="79"/>
+      <c r="AA118" s="81"/>
       <c r="AB118" s="57"/>
       <c r="AC118" s="83"/>
       <c r="AD118" s="84"/>

</xml_diff>

<commit_message>
Fix ECR logo placement geometry
</commit_message>
<xml_diff>
--- a/templates/ECR official Template.xlsx
+++ b/templates/ECR official Template.xlsx
@@ -1063,16 +1063,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>259200</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>144720</xdr:rowOff>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>39960</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>85680</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>256680</xdr:colOff>
+      <xdr:col>29</xdr:col>
+      <xdr:colOff>950400</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>141120</xdr:rowOff>
+      <xdr:rowOff>28800</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1106,16 +1106,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>28</xdr:col>
-      <xdr:colOff>39960</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>85680</xdr:rowOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>259200</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>144720</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>29</xdr:col>
-      <xdr:colOff>950400</xdr:colOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>256680</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>28800</xdr:rowOff>
+      <xdr:rowOff>141120</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>

</xml_diff>

<commit_message>
Fix ECR logo placement and aspect ratio
</commit_message>
<xml_diff>
--- a/templates/ECR official Template.xlsx
+++ b/templates/ECR official Template.xlsx
@@ -1061,19 +1061,42 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>28</xdr:col>
-      <xdr:colOff>39960</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>85680</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>29</xdr:col>
-      <xdr:colOff>950400</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>28800</xdr:rowOff>
-    </xdr:to>
+  <xdr:absoluteAnchor>
+    <xdr:pos x="525900" y="144720"/>
+    <xdr:ext cx="1603860" cy="811800"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="image1.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BDA6416A-A72E-4C54-95C3-5D3ADA6D96B6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="525900" y="144720"/>
+          <a:ext cx="1603860" cy="811800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:absoluteAnchor>
+  <xdr:absoluteAnchor>
+    <xdr:pos x="12367680" y="158100"/>
+    <xdr:ext cx="1041420" cy="1063200"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="2" name="image5.png">
@@ -1091,7 +1114,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="525900" y="144720"/>
+          <a:off x="12367680" y="158100"/>
           <a:ext cx="1041420" cy="1063200"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1103,50 +1126,7 @@
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>259200</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>144720</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>256680</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>141120</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="image1.png">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BDA6416A-A72E-4C54-95C3-5D3ADA6D96B6}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="11805240" y="283800"/>
-          <a:ext cx="1603860" cy="811800"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="0">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
+  </xdr:absoluteAnchor>
 </xdr:wsDr>
 </file>
 

</xml_diff>